<commit_message>
Monitor run 2026-05-23 12:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -429,14 +429,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
@@ -484,7 +484,219 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>228</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Icelandair</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>AMS</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>231</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>KLM + Scandinavian Airlines</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>CPH</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Copenhagen</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>286</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Scandinavian Airlines</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>ARN</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Stockholm</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>371</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Scandinavian Airlines</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="G5" t="n">
+        <v>2</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Frankfurt</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>404</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Lufthansa + Austrian</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>12</v>
+      </c>
+      <c r="G6" t="n">
+        <v>2</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>London Heathrow</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>410</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="D2:D7">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -495,16 +707,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="29" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
@@ -562,7 +774,271 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>KEF</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="n">
+        <v>228</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Icelandair</t>
+        </is>
+      </c>
+      <c r="H2" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>KEF</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>AMS</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="n">
+        <v>231</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>KLM + Scandinavian Airlines</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="I3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>KEF</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CPH</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" t="n">
+        <v>286</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Scandinavian Airlines</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>15.6</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>KEF</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>ARN</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="n">
+        <v>371</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Scandinavian Airlines</t>
+        </is>
+      </c>
+      <c r="H5" t="n">
+        <v>16.2</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>KEF</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="n">
+        <v>404</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>Lufthansa + Austrian</t>
+        </is>
+      </c>
+      <c r="H6" t="n">
+        <v>12</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>KEF</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="n">
+        <v>410</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>British Airways</t>
+        </is>
+      </c>
+      <c r="H7" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <conditionalFormatting sqref="F2:F7">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -573,11 +1049,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
     <col width="20" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
@@ -596,6 +1072,96 @@
         <is>
           <t>Preço mínimo (BRL)</t>
         </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>AMS</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>ARN</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CPH</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>410</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-25 18:34 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>228</v>
+        <v>1329</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>231</v>
+        <v>1345</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>286</v>
+        <v>1649</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>371</v>
+        <v>2162</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>404</v>
+        <v>2353</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>410</v>
+        <v>2391</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -680,7 +680,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>228</v>
+        <v>1329</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>231</v>
+        <v>1345</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>286</v>
+        <v>1649</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>371</v>
+        <v>2162</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -938,7 +938,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>404</v>
+        <v>2353</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -980,7 +980,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>410</v>
+        <v>2391</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1092,22 +1092,22 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>371</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1116,28 +1116,28 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>286</v>
+        <v>371</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>228</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1146,22 +1146,112 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>404</v>
+        <v>286</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>CPH</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:34 BRT</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1649</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:34 BRT</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1329</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:34 BRT</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2353</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
           <t>LHR</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
-      <c r="C7" t="n">
+      <c r="C12" t="n">
         <v>410</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:34 BRT</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>2391</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-25 18:35 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1107,16 +1107,16 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>371</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="5">
@@ -1127,47 +1127,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>286</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>1649</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -1176,13 +1176,13 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>228</v>
+        <v>286</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -1191,66 +1191,156 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1329</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>404</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2353</v>
+        <v>228</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>410</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1329</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:34 BRT</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>2353</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>2353</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>LHR</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
         <is>
           <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
-      <c r="C13" t="n">
+      <c r="C18" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
         <v>2391</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-05-25 18:57 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
     </row>
@@ -680,7 +680,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
     </row>
@@ -938,7 +938,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
     </row>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1137,16 +1137,16 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>371</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="7">
@@ -1157,11 +1157,11 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="8">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -1197,31 +1197,31 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>286</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>1649</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="12">
@@ -1232,11 +1232,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="13">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1257,46 +1257,46 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>228</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1329</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1329</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="17">
@@ -1307,47 +1307,47 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>404</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2353</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1356,28 +1356,28 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2353</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2353</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1386,13 +1386,13 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>410</v>
+        <v>404</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1401,13 +1401,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2391</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1416,21 +1416,111 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2391</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>2353</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:57 BRT</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2353</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>LHR</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:34 BRT</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
         <is>
           <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
-      <c r="C25" t="n">
+      <c r="C29" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:57 BRT</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
         <v>2391</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-05-25 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1649</v>
+        <v>1648</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2162</v>
+        <v>2161</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2353</v>
+        <v>2352</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2391</v>
+        <v>2389</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -680,7 +680,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -854,7 +854,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1649</v>
+        <v>1648</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2162</v>
+        <v>2161</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -938,7 +938,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2353</v>
+        <v>2352</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -980,7 +980,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2391</v>
+        <v>2389</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1152,16 +1152,16 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>371</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="8">
@@ -1172,11 +1172,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="9">
@@ -1187,7 +1187,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1227,31 +1227,31 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>286</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1649</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="14">
@@ -1262,11 +1262,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="15">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1302,46 +1302,46 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>228</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1329</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1329</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="20">
@@ -1352,11 +1352,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="21">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1377,61 +1377,61 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>404</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2353</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2353</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2353</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="26">
@@ -1442,47 +1442,47 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>410</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2391</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1491,37 +1491,127 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2391</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2391</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>25/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>2352</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>LHR</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:34 BRT</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
         <is>
           <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
-      <c r="C31" t="n">
+      <c r="C36" t="n">
         <v>2391</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>25/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>2389</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-26 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1329</v>
+        <v>1336</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1345</v>
+        <v>1351</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1648</v>
+        <v>1674</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2161</v>
+        <v>2172</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2352</v>
+        <v>2364</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2389</v>
+        <v>2402</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -680,7 +680,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1329</v>
+        <v>1336</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1345</v>
+        <v>1351</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1648</v>
+        <v>1674</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2161</v>
+        <v>2172</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -938,7 +938,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2352</v>
+        <v>2364</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -980,7 +980,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2389</v>
+        <v>2402</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C37"/>
+  <dimension ref="A1:C43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1167,16 +1167,16 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>371</v>
+        <v>1351</v>
       </c>
     </row>
     <row r="9">
@@ -1187,11 +1187,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="10">
@@ -1202,7 +1202,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1247,41 +1247,41 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>286</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>1649</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="16">
@@ -1292,11 +1292,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="17">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1337,56 +1337,56 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>228</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1329</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1329</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="23">
@@ -1397,11 +1397,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="24">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1437,61 +1437,61 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>404</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2353</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2353</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2353</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="30">
@@ -1502,11 +1502,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="31">
@@ -1517,86 +1517,86 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>410</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2391</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2391</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2391</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2391</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="37">
@@ -1607,11 +1607,101 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
+          <t>23/05/2026 09:17 BRT</t>
+        </is>
+      </c>
+      <c r="C37" t="n">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:34 BRT</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:57 BRT</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
-      <c r="C37" t="n">
+      <c r="C42" t="n">
         <v>2389</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>26/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2402</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-26 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1351</v>
+        <v>1353</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1674</v>
+        <v>1658</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2172</v>
+        <v>2174</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2364</v>
+        <v>2367</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2402</v>
+        <v>2404</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -680,7 +680,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1351</v>
+        <v>1353</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1674</v>
+        <v>1658</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2172</v>
+        <v>2174</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -938,7 +938,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2364</v>
+        <v>2367</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -980,7 +980,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2402</v>
+        <v>2404</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C43"/>
+  <dimension ref="A1:C49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1182,16 +1182,16 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>371</v>
+        <v>1353</v>
       </c>
     </row>
     <row r="10">
@@ -1202,11 +1202,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="11">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1262,11 +1262,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="15">
@@ -1277,41 +1277,41 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>286</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1649</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="18">
@@ -1322,11 +1322,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="19">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1352,7 +1352,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1367,11 +1367,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="22">
@@ -1382,56 +1382,56 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>228</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1329</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1329</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="26">
@@ -1442,11 +1442,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="27">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1487,71 +1487,71 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>404</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2353</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2353</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2353</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="34">
@@ -1562,11 +1562,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="35">
@@ -1577,11 +1577,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="36">
@@ -1592,86 +1592,86 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>410</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2391</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2391</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2391</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2391</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="42">
@@ -1682,11 +1682,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="43">
@@ -1697,11 +1697,101 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>25/05/2026 15:34 BRT</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:57 BRT</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>25/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2389</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
-      <c r="C43" t="n">
+      <c r="C48" t="n">
         <v>2402</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>26/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2404</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-27 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1353</v>
+        <v>1350</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1658</v>
+        <v>1654</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2174</v>
+        <v>2170</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2367</v>
+        <v>2238</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2404</v>
+        <v>2399</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -680,7 +680,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1353</v>
+        <v>1350</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1658</v>
+        <v>1654</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2174</v>
+        <v>2170</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -938,7 +938,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2367</v>
+        <v>2238</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -980,7 +980,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2404</v>
+        <v>2399</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C49"/>
+  <dimension ref="A1:C55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1197,16 +1197,16 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>371</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="11">
@@ -1217,11 +1217,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="12">
@@ -1232,7 +1232,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1277,11 +1277,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="16">
@@ -1292,11 +1292,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="17">
@@ -1307,41 +1307,41 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>286</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1649</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="20">
@@ -1352,11 +1352,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="21">
@@ -1367,7 +1367,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1382,7 +1382,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1397,11 +1397,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="24">
@@ -1412,11 +1412,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="25">
@@ -1427,56 +1427,56 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>228</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1329</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1329</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="29">
@@ -1487,11 +1487,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="30">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1532,11 +1532,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="33">
@@ -1547,71 +1547,71 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>404</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2353</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2353</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2353</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="38">
@@ -1622,11 +1622,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="39">
@@ -1637,11 +1637,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="40">
@@ -1652,11 +1652,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="41">
@@ -1667,86 +1667,86 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>410</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2391</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2391</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2391</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2391</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="47">
@@ -1757,11 +1757,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="48">
@@ -1772,11 +1772,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="49">
@@ -1787,11 +1787,101 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C50" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:57 BRT</t>
+        </is>
+      </c>
+      <c r="C51" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>25/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>2389</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>26/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>2402</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
           <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
-      <c r="C49" t="n">
+      <c r="C54" t="n">
         <v>2404</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>27/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>2399</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-27 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1334</v>
+        <v>1345</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1350</v>
+        <v>1361</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1654</v>
+        <v>1668</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2170</v>
+        <v>2188</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2238</v>
+        <v>2257</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2399</v>
+        <v>2419</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -680,7 +680,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1334</v>
+        <v>1345</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1350</v>
+        <v>1361</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1654</v>
+        <v>1668</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2170</v>
+        <v>2188</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -938,7 +938,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2238</v>
+        <v>2257</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -980,7 +980,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2399</v>
+        <v>2419</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C55"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1212,16 +1212,16 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>371</v>
+        <v>1361</v>
       </c>
     </row>
     <row r="12">
@@ -1232,11 +1232,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="13">
@@ -1247,7 +1247,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1292,11 +1292,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="17">
@@ -1307,11 +1307,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="18">
@@ -1322,11 +1322,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="19">
@@ -1337,41 +1337,41 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>286</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1649</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="22">
@@ -1382,11 +1382,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="23">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1412,7 +1412,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1427,11 +1427,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="26">
@@ -1442,11 +1442,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="27">
@@ -1457,11 +1457,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="28">
@@ -1472,56 +1472,56 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>228</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1329</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1329</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="32">
@@ -1532,11 +1532,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="33">
@@ -1547,7 +1547,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1562,7 +1562,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1577,11 +1577,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="36">
@@ -1592,11 +1592,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="37">
@@ -1607,71 +1607,71 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>404</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2353</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2353</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2353</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="42">
@@ -1682,11 +1682,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="43">
@@ -1697,11 +1697,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="44">
@@ -1712,11 +1712,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="45">
@@ -1727,11 +1727,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="46">
@@ -1742,86 +1742,86 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>410</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2391</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2391</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2391</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2391</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="52">
@@ -1832,11 +1832,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="53">
@@ -1847,11 +1847,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="54">
@@ -1862,11 +1862,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="55">
@@ -1877,11 +1877,101 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>25/05/2026 15:35 BRT</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>25/05/2026 15:57 BRT</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>25/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>2389</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>26/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>2402</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>26/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C59" t="n">
+        <v>2404</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
           <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C55" t="n">
+      <c r="C60" t="n">
         <v>2399</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>27/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>2419</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-27 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -436,7 +436,7 @@
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -529,22 +529,22 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1361</v>
+        <v>1521</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>KLM + Scandinavian Airlines</t>
+          <t>KLM + Transavia</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>11.3</v>
+        <v>13.3</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -554,31 +554,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Copenhagen</t>
+          <t>London Heathrow</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1668</v>
+        <v>1660</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.6</v>
+        <v>26.2</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -588,16 +588,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Stockholm</t>
+          <t>Copenhagen</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2188</v>
+        <v>1667</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -605,14 +605,14 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>16.2</v>
+        <v>15.6</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -622,31 +622,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>Stockholm</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2257</v>
+        <v>2186</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>12</v>
+        <v>16.2</v>
       </c>
       <c r="G6" t="n">
         <v>2</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -656,31 +656,31 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>London Heathrow</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2419</v>
+        <v>2196</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>14.2</v>
+        <v>12</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -716,7 +716,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="29" customWidth="1" min="7" max="7"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
@@ -797,7 +797,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1345</v>
+        <v>1344</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -839,22 +839,22 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1361</v>
+        <v>1521</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>KLM + Scandinavian Airlines</t>
+          <t>KLM + Transavia</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>11.3</v>
+        <v>13.3</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -881,22 +881,22 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1668</v>
+        <v>1660</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>15.6</v>
+        <v>26.2</v>
       </c>
       <c r="I4" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2188</v>
+        <v>1667</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -931,14 +931,14 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>16.2</v>
+        <v>15.6</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -965,22 +965,22 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2257</v>
+        <v>2186</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>12</v>
+        <v>16.2</v>
       </c>
       <c r="I6" t="n">
         <v>2</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1007,22 +1007,22 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2419</v>
+        <v>2196</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>14.2</v>
+        <v>12</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C61"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1227,16 +1227,16 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>371</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="13">
@@ -1247,11 +1247,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="14">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1307,11 +1307,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="18">
@@ -1322,11 +1322,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="19">
@@ -1337,11 +1337,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="20">
@@ -1352,11 +1352,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="21">
@@ -1367,41 +1367,41 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>286</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1649</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="24">
@@ -1412,11 +1412,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="25">
@@ -1427,7 +1427,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1442,7 +1442,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1457,11 +1457,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="28">
@@ -1472,11 +1472,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="29">
@@ -1487,11 +1487,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="30">
@@ -1502,11 +1502,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="31">
@@ -1517,56 +1517,56 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>228</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1329</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1329</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="35">
@@ -1577,11 +1577,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="36">
@@ -1592,7 +1592,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -1607,7 +1607,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1622,11 +1622,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="39">
@@ -1637,11 +1637,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="40">
@@ -1652,11 +1652,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="41">
@@ -1667,71 +1667,71 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>404</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2353</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2353</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2353</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="46">
@@ -1742,11 +1742,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="47">
@@ -1757,11 +1757,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="48">
@@ -1772,11 +1772,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="49">
@@ -1787,11 +1787,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="50">
@@ -1802,11 +1802,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="51">
@@ -1817,86 +1817,86 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>410</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2391</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2391</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2391</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2391</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="57">
@@ -1907,11 +1907,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="58">
@@ -1922,11 +1922,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="59">
@@ -1937,11 +1937,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="60">
@@ -1952,11 +1952,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="61">
@@ -1967,11 +1967,101 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
+          <t>25/05/2026 15:57 BRT</t>
+        </is>
+      </c>
+      <c r="C61" t="n">
+        <v>2391</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>25/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C62" t="n">
+        <v>2389</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>26/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C63" t="n">
+        <v>2402</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>26/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>2404</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>27/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C65" t="n">
+        <v>2399</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
           <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
-      <c r="C61" t="n">
+      <c r="C66" t="n">
         <v>2419</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>27/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>1660</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-28 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1521</v>
+        <v>1514</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1660</v>
+        <v>1652</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1667</v>
+        <v>1658</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2186</v>
+        <v>2181</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -680,7 +680,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1521</v>
+        <v>1514</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1660</v>
+        <v>1652</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1667</v>
+        <v>1658</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -938,7 +938,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2186</v>
+        <v>2181</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -980,7 +980,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C67"/>
+  <dimension ref="A1:C73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1242,16 +1242,16 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>371</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="14">
@@ -1262,11 +1262,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="15">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1322,11 +1322,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="19">
@@ -1337,11 +1337,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="20">
@@ -1352,11 +1352,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="21">
@@ -1367,11 +1367,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="22">
@@ -1382,11 +1382,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="23">
@@ -1397,41 +1397,41 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>286</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>1649</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="26">
@@ -1442,11 +1442,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="27">
@@ -1457,7 +1457,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1472,7 +1472,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1487,11 +1487,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="30">
@@ -1502,11 +1502,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="31">
@@ -1517,11 +1517,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="32">
@@ -1532,11 +1532,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="33">
@@ -1547,11 +1547,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="34">
@@ -1562,56 +1562,56 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>228</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1329</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1329</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="38">
@@ -1622,11 +1622,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="39">
@@ -1637,7 +1637,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1667,11 +1667,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="42">
@@ -1682,11 +1682,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="43">
@@ -1697,11 +1697,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="44">
@@ -1712,11 +1712,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="45">
@@ -1727,71 +1727,71 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>404</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2353</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2353</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2353</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="50">
@@ -1802,11 +1802,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="51">
@@ -1817,11 +1817,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="52">
@@ -1832,11 +1832,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="53">
@@ -1847,11 +1847,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="54">
@@ -1862,11 +1862,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="55">
@@ -1877,11 +1877,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="56">
@@ -1892,86 +1892,86 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>410</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2391</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2391</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2391</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2391</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="62">
@@ -1982,11 +1982,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="63">
@@ -1997,11 +1997,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="64">
@@ -2012,11 +2012,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="65">
@@ -2027,11 +2027,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="66">
@@ -2042,11 +2042,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="67">
@@ -2057,11 +2057,101 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
+          <t>25/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C67" t="n">
+        <v>2389</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>26/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C68" t="n">
+        <v>2402</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>26/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C69" t="n">
+        <v>2404</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>27/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C70" t="n">
+        <v>2399</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>27/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C71" t="n">
+        <v>2419</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
           <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
-      <c r="C67" t="n">
+      <c r="C72" t="n">
         <v>1660</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>28/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>1652</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-28 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1337</v>
+        <v>1340</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1514</v>
+        <v>1516</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1652</v>
+        <v>1655</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1658</v>
+        <v>1661</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2181</v>
+        <v>2185</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2185</v>
+        <v>2189</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -680,7 +680,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1337</v>
+        <v>1340</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1514</v>
+        <v>1516</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -881,7 +881,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1652</v>
+        <v>1655</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -896,7 +896,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -923,7 +923,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1658</v>
+        <v>1661</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -938,7 +938,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2181</v>
+        <v>2185</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -980,7 +980,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1007,7 +1007,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2185</v>
+        <v>2189</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1022,7 +1022,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C73"/>
+  <dimension ref="A1:C79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1257,16 +1257,16 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>371</v>
+        <v>1516</v>
       </c>
     </row>
     <row r="15">
@@ -1277,11 +1277,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="16">
@@ -1292,7 +1292,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1337,11 +1337,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="20">
@@ -1352,11 +1352,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="21">
@@ -1367,11 +1367,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="22">
@@ -1382,11 +1382,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="23">
@@ -1397,11 +1397,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="24">
@@ -1412,11 +1412,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="25">
@@ -1427,41 +1427,41 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>286</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1649</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="28">
@@ -1472,11 +1472,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="29">
@@ -1487,7 +1487,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1502,7 +1502,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1517,11 +1517,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="32">
@@ -1532,11 +1532,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="33">
@@ -1547,11 +1547,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="34">
@@ -1562,11 +1562,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="35">
@@ -1577,11 +1577,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="36">
@@ -1592,11 +1592,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="37">
@@ -1607,56 +1607,56 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>228</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1329</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1329</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="41">
@@ -1667,11 +1667,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="42">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -1697,7 +1697,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -1712,11 +1712,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="45">
@@ -1727,11 +1727,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="46">
@@ -1742,11 +1742,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="47">
@@ -1757,11 +1757,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="48">
@@ -1772,11 +1772,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="49">
@@ -1787,71 +1787,71 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>404</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2353</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2353</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2353</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="54">
@@ -1862,11 +1862,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="55">
@@ -1877,11 +1877,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="56">
@@ -1892,11 +1892,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="57">
@@ -1907,11 +1907,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="58">
@@ -1922,11 +1922,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="59">
@@ -1937,11 +1937,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="60">
@@ -1952,11 +1952,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="61">
@@ -1967,86 +1967,86 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>410</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2391</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2391</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2391</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2391</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="67">
@@ -2057,11 +2057,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="68">
@@ -2072,11 +2072,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="69">
@@ -2087,11 +2087,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="70">
@@ -2102,11 +2102,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="71">
@@ -2117,11 +2117,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="72">
@@ -2132,11 +2132,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1660</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="73">
@@ -2147,11 +2147,101 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
+          <t>26/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C73" t="n">
+        <v>2402</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>26/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C74" t="n">
+        <v>2404</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>27/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C75" t="n">
+        <v>2399</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>27/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C76" t="n">
+        <v>2419</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>27/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C77" t="n">
+        <v>1660</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
           <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C73" t="n">
+      <c r="C78" t="n">
         <v>1652</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>28/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>1655</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-28 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1516</v>
+        <v>1518</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -554,31 +554,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>London Heathrow</t>
+          <t>Copenhagen</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1655</v>
+        <v>1663</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>26.2</v>
+        <v>15.6</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -588,16 +588,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Copenhagen</t>
+          <t>Stockholm</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1661</v>
+        <v>2187</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -605,14 +605,14 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>15.6</v>
+        <v>16.2</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -622,31 +622,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Stockholm</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2185</v>
+        <v>2191</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>16.2</v>
+        <v>12</v>
       </c>
       <c r="G6" t="n">
         <v>2</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -656,31 +656,31 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>London Heathrow</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2189</v>
+        <v>2411</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>12</v>
+        <v>14.2</v>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -797,7 +797,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1340</v>
+        <v>1341</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -812,7 +812,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -839,7 +839,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1516</v>
+        <v>1518</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -854,7 +854,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -871,7 +871,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -881,22 +881,22 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1655</v>
+        <v>1663</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>26.2</v>
+        <v>15.6</v>
       </c>
       <c r="I4" t="n">
         <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -913,7 +913,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1661</v>
+        <v>2187</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -931,14 +931,14 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>15.6</v>
+        <v>16.2</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -955,7 +955,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -965,22 +965,22 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2185</v>
+        <v>2191</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>16.2</v>
+        <v>12</v>
       </c>
       <c r="I6" t="n">
         <v>2</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1007,22 +1007,22 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2189</v>
+        <v>2411</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>12</v>
+        <v>14.2</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C79"/>
+  <dimension ref="A1:C85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1272,16 +1272,16 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>371</v>
+        <v>1518</v>
       </c>
     </row>
     <row r="16">
@@ -1292,11 +1292,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="17">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1352,11 +1352,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="21">
@@ -1367,11 +1367,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="22">
@@ -1382,11 +1382,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="23">
@@ -1397,11 +1397,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="24">
@@ -1412,11 +1412,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="25">
@@ -1427,11 +1427,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="26">
@@ -1442,11 +1442,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="27">
@@ -1457,41 +1457,41 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>286</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>1649</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="30">
@@ -1502,11 +1502,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="31">
@@ -1517,7 +1517,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1532,7 +1532,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1547,11 +1547,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="34">
@@ -1562,11 +1562,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="35">
@@ -1577,11 +1577,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="36">
@@ -1592,11 +1592,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="37">
@@ -1607,11 +1607,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="38">
@@ -1622,11 +1622,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="39">
@@ -1637,11 +1637,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="40">
@@ -1652,56 +1652,56 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>228</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1329</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1329</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="44">
@@ -1712,11 +1712,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="45">
@@ -1727,7 +1727,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -1757,11 +1757,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="48">
@@ -1772,11 +1772,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="49">
@@ -1787,11 +1787,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="50">
@@ -1802,11 +1802,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="51">
@@ -1817,11 +1817,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="52">
@@ -1832,11 +1832,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="53">
@@ -1847,71 +1847,71 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>404</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2353</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2353</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2353</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="58">
@@ -1922,11 +1922,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="59">
@@ -1937,11 +1937,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="60">
@@ -1952,11 +1952,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="61">
@@ -1967,11 +1967,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="62">
@@ -1982,11 +1982,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="63">
@@ -1997,11 +1997,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="64">
@@ -2012,11 +2012,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="65">
@@ -2027,11 +2027,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="66">
@@ -2042,86 +2042,86 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>410</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2391</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2391</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2391</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2391</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="72">
@@ -2132,11 +2132,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="73">
@@ -2147,11 +2147,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="74">
@@ -2162,11 +2162,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="75">
@@ -2177,11 +2177,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="76">
@@ -2192,11 +2192,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="77">
@@ -2207,11 +2207,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1660</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="78">
@@ -2222,11 +2222,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1652</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="79">
@@ -2237,11 +2237,101 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
+          <t>26/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C79" t="n">
+        <v>2404</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>27/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C80" t="n">
+        <v>2399</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>27/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C81" t="n">
+        <v>2419</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>27/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C82" t="n">
+        <v>1660</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>28/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C83" t="n">
+        <v>1652</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
           <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
-      <c r="C79" t="n">
+      <c r="C84" t="n">
         <v>1655</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>28/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>2411</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-29 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1341</v>
+        <v>1337</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1518</v>
+        <v>1513</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -554,31 +554,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Copenhagen</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1663</v>
+        <v>2185</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.6</v>
+        <v>12</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -588,16 +588,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Stockholm</t>
+          <t>Copenhagen</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2187</v>
+        <v>2398</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -605,14 +605,14 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>16.2</v>
+        <v>7</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -622,31 +622,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>London Heathrow</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2191</v>
+        <v>2404</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>12</v>
+        <v>14.2</v>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -656,36 +656,66 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LHR</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>London Heathrow</t>
-        </is>
-      </c>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2411</v>
+        <v>2704</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>14.2</v>
+        <v>11.4</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>ARN</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Stockholm</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>2746</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Scandinavian Airlines</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D7">
+  <conditionalFormatting sqref="D2:D8">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -707,7 +737,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -797,7 +827,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1341</v>
+        <v>1337</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -812,7 +842,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -839,7 +869,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1518</v>
+        <v>1513</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -854,7 +884,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -871,7 +901,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -881,22 +911,22 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1663</v>
+        <v>2185</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>15.6</v>
+        <v>12</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -913,7 +943,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -923,7 +953,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2187</v>
+        <v>2398</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -931,14 +961,14 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>16.2</v>
+        <v>7</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -955,7 +985,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -965,22 +995,22 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2191</v>
+        <v>2404</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>12</v>
+        <v>14.2</v>
       </c>
       <c r="I6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -997,7 +1027,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>ZRH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1007,27 +1037,69 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2411</v>
+        <v>2704</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>14.2</v>
+        <v>11.4</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>KEF</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>ARN</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="n">
+        <v>2746</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Scandinavian Airlines</t>
+        </is>
+      </c>
+      <c r="H8" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F7">
+  <conditionalFormatting sqref="F2:F8">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1049,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C85"/>
+  <dimension ref="A1:C92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1287,16 +1359,16 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>371</v>
+        <v>1513</v>
       </c>
     </row>
     <row r="17">
@@ -1307,11 +1379,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="18">
@@ -1322,7 +1394,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -1352,7 +1424,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1367,11 +1439,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="22">
@@ -1382,11 +1454,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="23">
@@ -1397,11 +1469,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="24">
@@ -1412,11 +1484,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="25">
@@ -1427,11 +1499,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="26">
@@ -1442,11 +1514,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="27">
@@ -1457,11 +1529,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="28">
@@ -1472,11 +1544,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="29">
@@ -1487,41 +1559,41 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>286</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>1649</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="32">
@@ -1532,11 +1604,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="33">
@@ -1547,7 +1619,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1562,7 +1634,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1577,11 +1649,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="36">
@@ -1592,11 +1664,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="37">
@@ -1607,11 +1679,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="38">
@@ -1622,11 +1694,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="39">
@@ -1637,11 +1709,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="40">
@@ -1652,11 +1724,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="41">
@@ -1667,11 +1739,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="42">
@@ -1682,11 +1754,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="43">
@@ -1697,56 +1769,56 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>228</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1329</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1329</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="47">
@@ -1757,11 +1829,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="48">
@@ -1772,7 +1844,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1787,7 +1859,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1802,11 +1874,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="51">
@@ -1817,11 +1889,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="52">
@@ -1832,11 +1904,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="53">
@@ -1847,11 +1919,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="54">
@@ -1862,11 +1934,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="55">
@@ -1877,11 +1949,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="56">
@@ -1892,11 +1964,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="57">
@@ -1907,71 +1979,71 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>404</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2353</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2353</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2353</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="62">
@@ -1982,11 +2054,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="63">
@@ -1997,11 +2069,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="64">
@@ -2012,11 +2084,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="65">
@@ -2027,11 +2099,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="66">
@@ -2042,11 +2114,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="67">
@@ -2057,11 +2129,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="68">
@@ -2072,11 +2144,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="69">
@@ -2087,11 +2159,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="70">
@@ -2102,11 +2174,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="71">
@@ -2117,86 +2189,86 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>410</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2391</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2391</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2391</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2391</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="77">
@@ -2207,11 +2279,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="78">
@@ -2222,11 +2294,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="79">
@@ -2237,11 +2309,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="80">
@@ -2252,11 +2324,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="81">
@@ -2267,11 +2339,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="82">
@@ -2282,11 +2354,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1660</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="83">
@@ -2297,11 +2369,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1652</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="84">
@@ -2312,11 +2384,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1655</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="85">
@@ -2327,11 +2399,116 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
+          <t>27/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C85" t="n">
+        <v>2399</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>27/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C86" t="n">
+        <v>2419</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>27/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C87" t="n">
+        <v>1660</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>28/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>1652</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>28/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>1655</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
           <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
-      <c r="C85" t="n">
+      <c r="C90" t="n">
         <v>2411</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>29/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C91" t="n">
+        <v>2404</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>29/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>2704</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-29 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1513</v>
+        <v>1521</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2398</v>
+        <v>2410</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2404</v>
+        <v>2416</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2704</v>
+        <v>2718</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2746</v>
+        <v>2771</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -842,7 +842,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1513</v>
+        <v>1521</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -884,7 +884,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -926,7 +926,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -953,7 +953,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2398</v>
+        <v>2410</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -968,7 +968,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2404</v>
+        <v>2416</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2704</v>
+        <v>2718</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2746</v>
+        <v>2771</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C92"/>
+  <dimension ref="A1:C99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1374,16 +1374,16 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>371</v>
+        <v>1521</v>
       </c>
     </row>
     <row r="18">
@@ -1394,11 +1394,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="19">
@@ -1409,7 +1409,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1454,11 +1454,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="23">
@@ -1469,11 +1469,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="24">
@@ -1484,11 +1484,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="25">
@@ -1499,11 +1499,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="26">
@@ -1514,11 +1514,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="27">
@@ -1529,11 +1529,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="28">
@@ -1544,11 +1544,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="29">
@@ -1559,11 +1559,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="30">
@@ -1574,11 +1574,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="31">
@@ -1589,41 +1589,41 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>286</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>1649</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="34">
@@ -1634,11 +1634,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="35">
@@ -1649,7 +1649,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -1679,11 +1679,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="38">
@@ -1694,11 +1694,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="39">
@@ -1709,11 +1709,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="40">
@@ -1724,11 +1724,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="41">
@@ -1739,11 +1739,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="42">
@@ -1754,11 +1754,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="43">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="44">
@@ -1784,11 +1784,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="45">
@@ -1799,11 +1799,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="46">
@@ -1814,56 +1814,56 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>228</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1329</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1329</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="50">
@@ -1874,11 +1874,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="51">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -1919,11 +1919,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="54">
@@ -1934,11 +1934,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="55">
@@ -1949,11 +1949,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="56">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="57">
@@ -1979,11 +1979,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="58">
@@ -1994,11 +1994,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="59">
@@ -2009,11 +2009,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="60">
@@ -2024,11 +2024,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="61">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -2049,61 +2049,61 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>404</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2353</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2353</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2353</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="66">
@@ -2114,11 +2114,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="67">
@@ -2129,11 +2129,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="68">
@@ -2144,11 +2144,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="69">
@@ -2159,11 +2159,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="70">
@@ -2174,11 +2174,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="71">
@@ -2189,11 +2189,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="72">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="73">
@@ -2219,11 +2219,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="74">
@@ -2234,11 +2234,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="75">
@@ -2249,11 +2249,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="76">
@@ -2264,86 +2264,86 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>410</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2391</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2391</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2391</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2391</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="82">
@@ -2354,11 +2354,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="83">
@@ -2369,11 +2369,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="84">
@@ -2384,11 +2384,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="85">
@@ -2399,11 +2399,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="86">
@@ -2414,11 +2414,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="87">
@@ -2429,11 +2429,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1660</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="88">
@@ -2444,11 +2444,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1652</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1655</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="90">
@@ -2474,11 +2474,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2411</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="91">
@@ -2489,26 +2489,131 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>2404</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>27/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C92" t="n">
+        <v>1660</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>28/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C93" t="n">
+        <v>1652</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>28/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>1655</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>28/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>2411</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>29/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>2404</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>2416</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
           <t>ZRH</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B98" t="inlineStr">
         <is>
           <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C92" t="n">
+      <c r="C98" t="n">
         <v>2704</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>2718</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-29 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1344</v>
+        <v>1338</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1521</v>
+        <v>1514</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2196</v>
+        <v>2186</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -588,31 +588,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Copenhagen</t>
+          <t>London Heathrow</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2410</v>
+        <v>2405</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>7</v>
+        <v>14.2</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -622,31 +622,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>London Heathrow</t>
+          <t>Copenhagen</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2416</v>
+        <v>2575</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>14.2</v>
+        <v>7</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2718</v>
+        <v>2705</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2771</v>
+        <v>2758</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1344</v>
+        <v>1338</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -842,7 +842,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1521</v>
+        <v>1514</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -884,7 +884,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>2196</v>
+        <v>2186</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -926,7 +926,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -953,22 +953,22 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2410</v>
+        <v>2405</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>7</v>
+        <v>14.2</v>
       </c>
       <c r="I5" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -995,22 +995,22 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2416</v>
+        <v>2575</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>14.2</v>
+        <v>7</v>
       </c>
       <c r="I6" t="n">
         <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2718</v>
+        <v>2705</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2771</v>
+        <v>2758</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C99"/>
+  <dimension ref="A1:C106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1389,16 +1389,16 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>371</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="19">
@@ -1409,11 +1409,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="20">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1469,11 +1469,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="24">
@@ -1484,11 +1484,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="25">
@@ -1499,11 +1499,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="26">
@@ -1514,11 +1514,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="27">
@@ -1529,11 +1529,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="28">
@@ -1544,11 +1544,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="29">
@@ -1559,11 +1559,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="30">
@@ -1574,11 +1574,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="31">
@@ -1589,11 +1589,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="32">
@@ -1604,11 +1604,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="33">
@@ -1619,41 +1619,41 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>286</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1649</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="36">
@@ -1664,11 +1664,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="37">
@@ -1679,7 +1679,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -1709,11 +1709,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="40">
@@ -1724,11 +1724,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="41">
@@ -1739,11 +1739,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="42">
@@ -1754,11 +1754,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="43">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="44">
@@ -1784,11 +1784,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="45">
@@ -1799,11 +1799,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="46">
@@ -1814,11 +1814,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="47">
@@ -1829,11 +1829,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="48">
@@ -1844,11 +1844,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="49">
@@ -1859,56 +1859,56 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>228</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1329</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="53">
@@ -1919,11 +1919,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="54">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="57">
@@ -1979,11 +1979,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="58">
@@ -1994,11 +1994,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="59">
@@ -2009,11 +2009,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="60">
@@ -2024,11 +2024,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="61">
@@ -2039,11 +2039,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="62">
@@ -2054,11 +2054,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="63">
@@ -2069,11 +2069,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="64">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -2099,71 +2099,71 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>404</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2353</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2353</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="70">
@@ -2174,11 +2174,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="71">
@@ -2189,11 +2189,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="72">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="73">
@@ -2219,11 +2219,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="74">
@@ -2234,11 +2234,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="75">
@@ -2249,11 +2249,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="76">
@@ -2264,11 +2264,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="77">
@@ -2279,11 +2279,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="78">
@@ -2294,11 +2294,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="79">
@@ -2309,11 +2309,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="80">
@@ -2324,11 +2324,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="81">
@@ -2339,86 +2339,86 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>410</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2391</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2391</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2391</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="87">
@@ -2429,11 +2429,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="88">
@@ -2444,11 +2444,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="90">
@@ -2474,11 +2474,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="91">
@@ -2489,11 +2489,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="92">
@@ -2504,11 +2504,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1660</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="93">
@@ -2519,11 +2519,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1652</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="94">
@@ -2534,11 +2534,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1655</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="95">
@@ -2549,11 +2549,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2411</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="96">
@@ -2564,11 +2564,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>2404</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="97">
@@ -2579,41 +2579,146 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>2416</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>2704</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>28/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C99" t="n">
+        <v>1655</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>28/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C100" t="n">
+        <v>2411</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>29/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C101" t="n">
+        <v>2404</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C102" t="n">
+        <v>2416</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>29/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C103" t="n">
+        <v>2405</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
           <t>ZRH</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>29/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
         <is>
           <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
-      <c r="C99" t="n">
+      <c r="C105" t="n">
         <v>2718</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>29/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>2705</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-30 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2758</v>
+        <v>3175</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2758</v>
+        <v>3175</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C106"/>
+  <dimension ref="A1:C113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1404,16 +1404,16 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>371</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="20">
@@ -1424,11 +1424,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="21">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1484,11 +1484,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="25">
@@ -1499,11 +1499,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="26">
@@ -1514,11 +1514,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="27">
@@ -1529,11 +1529,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="28">
@@ -1544,11 +1544,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="29">
@@ -1559,11 +1559,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="30">
@@ -1574,11 +1574,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="31">
@@ -1589,11 +1589,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="32">
@@ -1604,11 +1604,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="33">
@@ -1619,11 +1619,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="34">
@@ -1634,11 +1634,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="35">
@@ -1649,41 +1649,41 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>286</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1649</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="38">
@@ -1694,11 +1694,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="39">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -1724,7 +1724,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1739,11 +1739,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="42">
@@ -1754,11 +1754,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="43">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="44">
@@ -1784,11 +1784,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="45">
@@ -1799,11 +1799,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="46">
@@ -1814,11 +1814,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="47">
@@ -1829,11 +1829,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="48">
@@ -1844,11 +1844,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="49">
@@ -1859,11 +1859,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="50">
@@ -1874,11 +1874,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="51">
@@ -1889,11 +1889,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="52">
@@ -1904,56 +1904,56 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2575</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>228</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="56">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="57">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -2009,11 +2009,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="60">
@@ -2024,11 +2024,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="61">
@@ -2039,11 +2039,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="62">
@@ -2054,11 +2054,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="63">
@@ -2069,11 +2069,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="64">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="65">
@@ -2099,11 +2099,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="66">
@@ -2114,11 +2114,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="67">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -2144,11 +2144,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="69">
@@ -2159,71 +2159,71 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1338</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>404</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2353</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="74">
@@ -2234,11 +2234,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="75">
@@ -2249,11 +2249,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="76">
@@ -2264,11 +2264,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="77">
@@ -2279,11 +2279,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="78">
@@ -2294,11 +2294,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="79">
@@ -2309,11 +2309,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="80">
@@ -2324,11 +2324,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="81">
@@ -2339,11 +2339,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="82">
@@ -2354,11 +2354,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="83">
@@ -2369,11 +2369,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="84">
@@ -2384,11 +2384,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="85">
@@ -2399,11 +2399,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="86">
@@ -2414,86 +2414,86 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>410</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2391</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2391</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="92">
@@ -2504,11 +2504,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="93">
@@ -2519,11 +2519,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="94">
@@ -2534,11 +2534,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="95">
@@ -2549,11 +2549,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="96">
@@ -2564,11 +2564,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="97">
@@ -2579,11 +2579,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1660</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="98">
@@ -2594,11 +2594,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1652</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="99">
@@ -2609,11 +2609,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1655</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="100">
@@ -2624,11 +2624,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>2411</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="101">
@@ -2639,11 +2639,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2404</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="102">
@@ -2654,11 +2654,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>2416</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="103">
@@ -2669,55 +2669,160 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>2704</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2718</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>29/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C106" t="n">
+        <v>2404</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C107" t="n">
+        <v>2416</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>29/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C108" t="n">
+        <v>2405</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>30/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C109" t="n">
+        <v>2405</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
           <t>ZRH</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>29/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C110" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C111" t="n">
+        <v>2718</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
         <is>
           <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
-      <c r="C106" t="n">
+      <c r="C112" t="n">
+        <v>2705</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>30/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
         <v>2705</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-05-30 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -588,31 +588,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>London Heathrow</t>
+          <t>Stockholm</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2405</v>
+        <v>2358</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>14.2</v>
+        <v>16.2</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -622,31 +622,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Copenhagen</t>
+          <t>London Heathrow</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2575</v>
+        <v>2406</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7</v>
+        <v>14.2</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -656,27 +656,31 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ZRH</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>CPH</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Copenhagen</t>
+        </is>
+      </c>
       <c r="D7" t="n">
-        <v>2705</v>
+        <v>2576</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>11.4</v>
+        <v>7</v>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -686,31 +690,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ARN</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Stockholm</t>
-        </is>
-      </c>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>3175</v>
+        <v>2706</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>15.4</v>
+        <v>11.4</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -953,22 +953,22 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2405</v>
+        <v>2358</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>14.2</v>
+        <v>16.2</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -995,22 +995,22 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2575</v>
+        <v>2406</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>7</v>
+        <v>14.2</v>
       </c>
       <c r="I6" t="n">
         <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1037,22 +1037,22 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2705</v>
+        <v>2576</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>11.4</v>
+        <v>7</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>ZRH</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1079,22 +1079,22 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>3175</v>
+        <v>2706</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>15.4</v>
+        <v>11.4</v>
       </c>
       <c r="I8" t="n">
         <v>2</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C113"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1419,16 +1419,16 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>371</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="21">
@@ -1439,11 +1439,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="22">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1499,11 +1499,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="26">
@@ -1514,11 +1514,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="27">
@@ -1529,11 +1529,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="28">
@@ -1544,11 +1544,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="29">
@@ -1559,11 +1559,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="30">
@@ -1574,11 +1574,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="31">
@@ -1589,11 +1589,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="32">
@@ -1604,11 +1604,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="33">
@@ -1619,11 +1619,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="34">
@@ -1634,11 +1634,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="35">
@@ -1649,11 +1649,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="36">
@@ -1664,11 +1664,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="37">
@@ -1679,41 +1679,41 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>286</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1649</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="40">
@@ -1724,11 +1724,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="41">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="44">
@@ -1784,11 +1784,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="45">
@@ -1799,11 +1799,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="46">
@@ -1814,11 +1814,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="47">
@@ -1829,11 +1829,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="48">
@@ -1844,11 +1844,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="49">
@@ -1859,11 +1859,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="50">
@@ -1874,11 +1874,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="51">
@@ -1889,11 +1889,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="52">
@@ -1904,11 +1904,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="53">
@@ -1919,11 +1919,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="54">
@@ -1934,11 +1934,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2575</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="55">
@@ -1949,56 +1949,56 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>228</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1329</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="59">
@@ -2009,11 +2009,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="60">
@@ -2024,7 +2024,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -2054,11 +2054,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="63">
@@ -2069,11 +2069,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="64">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="65">
@@ -2099,11 +2099,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="66">
@@ -2114,11 +2114,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="67">
@@ -2129,11 +2129,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="68">
@@ -2144,11 +2144,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="69">
@@ -2159,11 +2159,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="70">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -2189,11 +2189,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="72">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1338</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="73">
@@ -2219,71 +2219,71 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>404</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="78">
@@ -2294,11 +2294,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="79">
@@ -2309,11 +2309,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="80">
@@ -2324,11 +2324,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="81">
@@ -2339,11 +2339,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="82">
@@ -2354,11 +2354,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="83">
@@ -2369,11 +2369,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="84">
@@ -2384,11 +2384,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="85">
@@ -2399,11 +2399,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="86">
@@ -2414,11 +2414,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="87">
@@ -2429,11 +2429,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="88">
@@ -2444,11 +2444,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="90">
@@ -2474,11 +2474,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="91">
@@ -2489,86 +2489,86 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>410</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2391</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="97">
@@ -2579,11 +2579,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="98">
@@ -2594,11 +2594,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="99">
@@ -2609,11 +2609,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="100">
@@ -2624,11 +2624,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="101">
@@ -2639,11 +2639,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="102">
@@ -2654,11 +2654,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1660</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="103">
@@ -2669,11 +2669,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1652</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="104">
@@ -2684,11 +2684,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1655</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="105">
@@ -2699,11 +2699,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2411</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="106">
@@ -2714,11 +2714,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>2404</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="107">
@@ -2729,11 +2729,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>2416</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="108">
@@ -2744,11 +2744,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="109">
@@ -2759,71 +2759,176 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>2704</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>2718</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>2705</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>29/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C113" t="n">
+        <v>2405</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>30/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C114" t="n">
+        <v>2405</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>30/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C115" t="n">
+        <v>2406</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
           <t>ZRH</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr">
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>29/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C116" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C117" t="n">
+        <v>2718</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>29/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C118" t="n">
+        <v>2705</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
         <is>
           <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C113" t="n">
+      <c r="C119" t="n">
         <v>2705</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>30/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>2706</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-05-30 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -588,16 +588,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Stockholm</t>
+          <t>Copenhagen</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2358</v>
+        <v>2329</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -605,14 +605,14 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>16.2</v>
+        <v>22.2</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -622,27 +622,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>London Heathrow</t>
+          <t>Stockholm</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2406</v>
+        <v>2358</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>14.2</v>
+        <v>16.2</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -656,31 +656,31 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Copenhagen</t>
+          <t>London Heathrow</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2576</v>
+        <v>2406</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>7</v>
+        <v>14.2</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2358</v>
+        <v>2329</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -961,14 +961,14 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>16.2</v>
+        <v>22.2</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -995,18 +995,18 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2406</v>
+        <v>2358</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>14.2</v>
+        <v>16.2</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1037,22 +1037,22 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2576</v>
+        <v>2406</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>7</v>
+        <v>14.2</v>
       </c>
       <c r="I7" t="n">
         <v>1</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C120"/>
+  <dimension ref="A1:C126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1434,16 +1434,16 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>371</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="22">
@@ -1454,11 +1454,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="23">
@@ -1469,7 +1469,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1514,11 +1514,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="27">
@@ -1529,11 +1529,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="28">
@@ -1544,11 +1544,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="29">
@@ -1559,11 +1559,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="30">
@@ -1574,11 +1574,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="31">
@@ -1589,11 +1589,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="32">
@@ -1604,11 +1604,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="33">
@@ -1619,11 +1619,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="34">
@@ -1634,11 +1634,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="35">
@@ -1649,11 +1649,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="36">
@@ -1664,11 +1664,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="37">
@@ -1679,11 +1679,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="38">
@@ -1694,11 +1694,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="39">
@@ -1709,26 +1709,26 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>286</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="41">
@@ -1739,11 +1739,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="42">
@@ -1754,7 +1754,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1799,11 +1799,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="46">
@@ -1814,11 +1814,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1674</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="47">
@@ -1829,11 +1829,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1658</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="48">
@@ -1844,11 +1844,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1654</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="49">
@@ -1859,11 +1859,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1668</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="50">
@@ -1874,11 +1874,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1667</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="51">
@@ -1889,11 +1889,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1658</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="52">
@@ -1904,11 +1904,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1661</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="53">
@@ -1919,11 +1919,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1663</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="54">
@@ -1934,11 +1934,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2398</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="55">
@@ -1949,11 +1949,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2410</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="56">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="57">
@@ -1979,7 +1979,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -1994,41 +1994,41 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>228</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1329</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="61">
@@ -2039,11 +2039,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="62">
@@ -2054,7 +2054,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -2069,7 +2069,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -2099,11 +2099,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="66">
@@ -2114,11 +2114,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="67">
@@ -2129,11 +2129,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1334</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="68">
@@ -2144,11 +2144,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1345</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="69">
@@ -2159,11 +2159,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1344</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="70">
@@ -2174,11 +2174,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1337</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="71">
@@ -2189,11 +2189,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1340</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="72">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1341</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="73">
@@ -2219,11 +2219,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1337</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="74">
@@ -2234,11 +2234,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1344</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="75">
@@ -2249,11 +2249,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="76">
@@ -2264,11 +2264,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="77">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -2289,46 +2289,46 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>404</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="81">
@@ -2339,11 +2339,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="82">
@@ -2354,7 +2354,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -2369,11 +2369,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="84">
@@ -2384,11 +2384,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="85">
@@ -2399,11 +2399,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="86">
@@ -2414,11 +2414,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2238</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="87">
@@ -2429,11 +2429,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2257</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="88">
@@ -2444,11 +2444,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2196</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2185</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="90">
@@ -2474,11 +2474,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2189</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="91">
@@ -2489,11 +2489,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>2191</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="92">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -2519,11 +2519,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2196</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="94">
@@ -2534,11 +2534,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="95">
@@ -2549,11 +2549,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="96">
@@ -2564,71 +2564,71 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>410</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="101">
@@ -2639,11 +2639,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="102">
@@ -2654,11 +2654,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="103">
@@ -2669,11 +2669,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="104">
@@ -2684,11 +2684,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="105">
@@ -2699,11 +2699,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="106">
@@ -2714,11 +2714,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="107">
@@ -2729,11 +2729,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="108">
@@ -2744,11 +2744,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="109">
@@ -2759,11 +2759,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="110">
@@ -2774,11 +2774,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="111">
@@ -2789,11 +2789,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="112">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="113">
@@ -2819,11 +2819,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="114">
@@ -2834,11 +2834,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="115">
@@ -2849,85 +2849,175 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>2704</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>2718</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>2705</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>2705</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>30/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C120" t="n">
+        <v>2406</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
           <t>ZRH</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr">
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>29/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C121" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C122" t="n">
+        <v>2718</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>29/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C123" t="n">
+        <v>2705</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>30/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C124" t="n">
+        <v>2705</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
         <is>
           <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
-      <c r="C120" t="n">
+      <c r="C125" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>30/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
         <v>2706</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-05-31 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -554,31 +554,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>London Heathrow</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>2186</v>
+        <v>1652</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>12</v>
+        <v>26.2</v>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -588,31 +588,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Copenhagen</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2329</v>
+        <v>2186</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>22.2</v>
+        <v>12</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -622,16 +622,16 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Stockholm</t>
+          <t>Copenhagen</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2358</v>
+        <v>2575</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -639,14 +639,14 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>16.2</v>
+        <v>7</v>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -656,31 +656,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>LHR</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>London Heathrow</t>
-        </is>
-      </c>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2406</v>
+        <v>2706</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>14.2</v>
+        <v>11.4</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -690,27 +686,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ZRH</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>ARN</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Stockholm</t>
+        </is>
+      </c>
       <c r="D8" t="n">
-        <v>2706</v>
+        <v>3176</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>11.4</v>
+        <v>15.4</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -911,22 +911,22 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>2186</v>
+        <v>1652</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>12</v>
+        <v>26.2</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -953,22 +953,22 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2329</v>
+        <v>2186</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>22.2</v>
+        <v>12</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -985,7 +985,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2358</v>
+        <v>2575</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1003,14 +1003,14 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>16.2</v>
+        <v>7</v>
       </c>
       <c r="I6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>ZRH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1037,22 +1037,22 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2406</v>
+        <v>2706</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>14.2</v>
+        <v>11.4</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1069,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1079,22 +1079,22 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2706</v>
+        <v>3176</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>11.4</v>
+        <v>15.4</v>
       </c>
       <c r="I8" t="n">
         <v>2</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C126"/>
+  <dimension ref="A1:C133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1449,16 +1449,16 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>371</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="23">
@@ -1469,11 +1469,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="24">
@@ -1484,7 +1484,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1529,11 +1529,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="28">
@@ -1544,11 +1544,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="29">
@@ -1559,11 +1559,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="30">
@@ -1574,11 +1574,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="31">
@@ -1589,11 +1589,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="32">
@@ -1604,11 +1604,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="33">
@@ -1619,11 +1619,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="34">
@@ -1634,11 +1634,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="35">
@@ -1649,11 +1649,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="36">
@@ -1664,11 +1664,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="37">
@@ -1679,11 +1679,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="38">
@@ -1694,11 +1694,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="39">
@@ -1709,11 +1709,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="40">
@@ -1724,41 +1724,41 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>286</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1649</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="43">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="44">
@@ -1784,7 +1784,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1799,7 +1799,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1814,11 +1814,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="47">
@@ -1829,11 +1829,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="48">
@@ -1844,11 +1844,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="49">
@@ -1859,11 +1859,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="50">
@@ -1874,11 +1874,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="51">
@@ -1889,11 +1889,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="52">
@@ -1904,11 +1904,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="53">
@@ -1919,11 +1919,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="54">
@@ -1934,11 +1934,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="55">
@@ -1949,11 +1949,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="56">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="57">
@@ -1979,11 +1979,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2575</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="58">
@@ -1994,11 +1994,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="59">
@@ -2009,11 +2009,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="60">
@@ -2024,56 +2024,56 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>228</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1329</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="64">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="65">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -2129,11 +2129,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="68">
@@ -2144,11 +2144,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="69">
@@ -2159,11 +2159,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="70">
@@ -2174,11 +2174,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="71">
@@ -2189,11 +2189,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="72">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="73">
@@ -2219,11 +2219,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="74">
@@ -2234,11 +2234,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="75">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -2264,11 +2264,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="77">
@@ -2279,11 +2279,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1338</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="78">
@@ -2294,11 +2294,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="79">
@@ -2309,11 +2309,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="80">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -2334,61 +2334,61 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>404</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="85">
@@ -2399,11 +2399,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="86">
@@ -2414,11 +2414,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="87">
@@ -2429,11 +2429,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="88">
@@ -2444,11 +2444,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="90">
@@ -2474,11 +2474,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="91">
@@ -2489,11 +2489,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="92">
@@ -2504,11 +2504,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="93">
@@ -2519,11 +2519,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="94">
@@ -2534,11 +2534,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="95">
@@ -2549,11 +2549,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="96">
@@ -2564,11 +2564,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="97">
@@ -2579,11 +2579,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="98">
@@ -2594,11 +2594,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="99">
@@ -2609,11 +2609,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="100">
@@ -2624,86 +2624,86 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>410</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="106">
@@ -2714,11 +2714,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="107">
@@ -2729,11 +2729,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="108">
@@ -2744,11 +2744,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="109">
@@ -2759,11 +2759,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="110">
@@ -2774,11 +2774,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="111">
@@ -2789,11 +2789,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1660</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="112">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1652</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="113">
@@ -2819,11 +2819,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1655</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="114">
@@ -2834,11 +2834,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>2411</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="115">
@@ -2849,11 +2849,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2404</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="116">
@@ -2864,11 +2864,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>2416</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="117">
@@ -2879,11 +2879,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="118">
@@ -2894,11 +2894,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="119">
@@ -2909,11 +2909,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>2406</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="120">
@@ -2924,100 +2924,205 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>2704</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>2718</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>2705</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>2705</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2706</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>31/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C126" t="n">
+        <v>1652</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
           <t>ZRH</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr">
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>29/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C127" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C128" t="n">
+        <v>2718</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>29/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C129" t="n">
+        <v>2705</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>30/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C130" t="n">
+        <v>2705</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>30/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C131" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
         <is>
           <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
-      <c r="C126" t="n">
+      <c r="C132" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>31/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
         <v>2706</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-05-31 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -676,7 +676,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>3176</v>
+        <v>2917</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -926,7 +926,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -968,7 +968,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>3176</v>
+        <v>2917</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C133"/>
+  <dimension ref="A1:C140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1464,16 +1464,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>371</v>
+        <v>1514</v>
       </c>
     </row>
     <row r="24">
@@ -1484,11 +1484,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="25">
@@ -1499,7 +1499,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1544,11 +1544,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="29">
@@ -1559,11 +1559,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="30">
@@ -1574,11 +1574,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="31">
@@ -1589,11 +1589,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="32">
@@ -1604,11 +1604,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="33">
@@ -1619,11 +1619,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="34">
@@ -1634,11 +1634,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="35">
@@ -1649,11 +1649,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="36">
@@ -1664,11 +1664,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="37">
@@ -1679,11 +1679,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="38">
@@ -1694,11 +1694,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="39">
@@ -1709,11 +1709,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="40">
@@ -1724,11 +1724,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="41">
@@ -1739,11 +1739,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="42">
@@ -1754,41 +1754,41 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>286</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>1649</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="45">
@@ -1799,11 +1799,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="46">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1844,11 +1844,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="49">
@@ -1859,11 +1859,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="50">
@@ -1874,11 +1874,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="51">
@@ -1889,11 +1889,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="52">
@@ -1904,11 +1904,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="53">
@@ -1919,11 +1919,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="54">
@@ -1934,11 +1934,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="55">
@@ -1949,11 +1949,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="56">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="57">
@@ -1979,11 +1979,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="58">
@@ -1994,11 +1994,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="59">
@@ -2009,11 +2009,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2575</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="60">
@@ -2024,11 +2024,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="61">
@@ -2039,11 +2039,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="62">
@@ -2054,11 +2054,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="63">
@@ -2069,56 +2069,56 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2575</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>228</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="67">
@@ -2129,11 +2129,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="68">
@@ -2144,7 +2144,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -2174,11 +2174,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="71">
@@ -2189,11 +2189,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="72">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="73">
@@ -2219,11 +2219,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="74">
@@ -2234,11 +2234,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="75">
@@ -2249,11 +2249,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="76">
@@ -2264,11 +2264,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="77">
@@ -2279,11 +2279,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="78">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -2309,11 +2309,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="80">
@@ -2324,11 +2324,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1338</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="81">
@@ -2339,11 +2339,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="82">
@@ -2354,11 +2354,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="83">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -2384,7 +2384,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -2394,61 +2394,61 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>404</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="90">
@@ -2474,11 +2474,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="91">
@@ -2489,11 +2489,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="92">
@@ -2504,11 +2504,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="93">
@@ -2519,11 +2519,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="94">
@@ -2534,11 +2534,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="95">
@@ -2549,11 +2549,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="96">
@@ -2564,11 +2564,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="97">
@@ -2579,11 +2579,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="98">
@@ -2594,11 +2594,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="99">
@@ -2609,11 +2609,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="100">
@@ -2624,11 +2624,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="101">
@@ -2639,11 +2639,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="102">
@@ -2654,11 +2654,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="103">
@@ -2669,11 +2669,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="104">
@@ -2684,11 +2684,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="105">
@@ -2699,7 +2699,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -2709,76 +2709,76 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>410</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="111">
@@ -2789,11 +2789,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="112">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="113">
@@ -2819,11 +2819,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="114">
@@ -2834,11 +2834,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="115">
@@ -2849,11 +2849,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="116">
@@ -2864,11 +2864,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1660</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="117">
@@ -2879,11 +2879,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1652</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="118">
@@ -2894,11 +2894,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1655</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="119">
@@ -2909,11 +2909,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>2411</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="120">
@@ -2924,11 +2924,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2404</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="121">
@@ -2939,11 +2939,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>2416</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="122">
@@ -2954,11 +2954,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="123">
@@ -2969,11 +2969,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="124">
@@ -2984,11 +2984,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>2406</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="125">
@@ -2999,11 +2999,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="126">
@@ -3014,101 +3014,101 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1652</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>2704</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>2718</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>2705</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2705</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2706</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>2706</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="133">
@@ -3119,10 +3119,115 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
+          <t>29/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C133" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>29/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C134" t="n">
+        <v>2718</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>29/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C135" t="n">
+        <v>2705</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>30/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C136" t="n">
+        <v>2705</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>30/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C137" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>30/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C138" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
           <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C133" t="n">
+      <c r="C139" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>31/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
         <v>2706</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-05-31 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1514</v>
+        <v>1513</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -554,31 +554,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>London Heathrow</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1652</v>
+        <v>1680</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>26.2</v>
+        <v>15.5</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -588,31 +588,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>London Heathrow</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2186</v>
+        <v>2404</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>12</v>
+        <v>14.2</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2575</v>
+        <v>2574</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -695,7 +695,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2917</v>
+        <v>2915</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -710,7 +710,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -842,7 +842,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1514</v>
+        <v>1513</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -884,7 +884,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -911,22 +911,22 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1652</v>
+        <v>1680</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>26.2</v>
+        <v>15.5</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -953,22 +953,22 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2186</v>
+        <v>2404</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>12</v>
+        <v>14.2</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2575</v>
+        <v>2574</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1079,7 +1079,7 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2917</v>
+        <v>2915</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C140"/>
+  <dimension ref="A1:C147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1479,16 +1479,16 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>371</v>
+        <v>1513</v>
       </c>
     </row>
     <row r="25">
@@ -1499,11 +1499,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="26">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -1544,7 +1544,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1559,11 +1559,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="30">
@@ -1574,11 +1574,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="31">
@@ -1589,11 +1589,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="32">
@@ -1604,11 +1604,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="33">
@@ -1619,11 +1619,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="34">
@@ -1634,11 +1634,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="35">
@@ -1649,11 +1649,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="36">
@@ -1664,11 +1664,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="37">
@@ -1679,11 +1679,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="38">
@@ -1694,11 +1694,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="39">
@@ -1709,11 +1709,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="40">
@@ -1724,11 +1724,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="41">
@@ -1739,11 +1739,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="42">
@@ -1754,11 +1754,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="43">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="44">
@@ -1784,41 +1784,41 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>286</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>1649</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="47">
@@ -1829,11 +1829,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="48">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1874,11 +1874,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="51">
@@ -1889,11 +1889,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="52">
@@ -1904,11 +1904,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="53">
@@ -1919,11 +1919,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="54">
@@ -1934,11 +1934,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="55">
@@ -1949,11 +1949,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="56">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="57">
@@ -1979,11 +1979,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="58">
@@ -1994,11 +1994,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="59">
@@ -2009,11 +2009,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="60">
@@ -2024,11 +2024,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="61">
@@ -2039,11 +2039,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2575</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="62">
@@ -2054,11 +2054,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="63">
@@ -2069,11 +2069,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="64">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="65">
@@ -2099,11 +2099,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2575</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="66">
@@ -2114,56 +2114,56 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>228</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1329</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="70">
@@ -2174,11 +2174,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="71">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -2204,7 +2204,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
@@ -2219,11 +2219,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="74">
@@ -2234,11 +2234,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="75">
@@ -2249,11 +2249,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="76">
@@ -2264,11 +2264,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="77">
@@ -2279,11 +2279,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="78">
@@ -2294,11 +2294,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="79">
@@ -2309,11 +2309,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="80">
@@ -2324,11 +2324,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="81">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -2354,11 +2354,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="83">
@@ -2369,11 +2369,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1338</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="84">
@@ -2384,11 +2384,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="85">
@@ -2399,11 +2399,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="86">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -2429,7 +2429,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -2454,61 +2454,61 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>404</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>2353</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>2353</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="93">
@@ -2519,11 +2519,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="94">
@@ -2534,11 +2534,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="95">
@@ -2549,11 +2549,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="96">
@@ -2564,11 +2564,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="97">
@@ -2579,11 +2579,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="98">
@@ -2594,11 +2594,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="99">
@@ -2609,11 +2609,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="100">
@@ -2624,11 +2624,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="101">
@@ -2639,11 +2639,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="102">
@@ -2654,11 +2654,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="103">
@@ -2669,11 +2669,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="104">
@@ -2684,11 +2684,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="105">
@@ -2699,11 +2699,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="106">
@@ -2714,11 +2714,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="107">
@@ -2729,11 +2729,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="108">
@@ -2744,11 +2744,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="109">
@@ -2759,7 +2759,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -2774,7 +2774,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -2784,76 +2784,76 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>410</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2391</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="116">
@@ -2864,11 +2864,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="117">
@@ -2879,11 +2879,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="118">
@@ -2894,11 +2894,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="119">
@@ -2909,11 +2909,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="120">
@@ -2924,11 +2924,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="121">
@@ -2939,11 +2939,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1660</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="122">
@@ -2954,11 +2954,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1652</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="123">
@@ -2969,11 +2969,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1655</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="124">
@@ -2984,11 +2984,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>2411</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="125">
@@ -2999,11 +2999,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2404</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="126">
@@ -3014,11 +3014,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>2416</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="127">
@@ -3029,11 +3029,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="128">
@@ -3044,11 +3044,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="129">
@@ -3059,11 +3059,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>2406</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="130">
@@ -3074,11 +3074,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="131">
@@ -3089,11 +3089,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1652</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="132">
@@ -3104,101 +3104,101 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2704</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2718</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2705</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>2705</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>2706</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>2706</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="139">
@@ -3209,11 +3209,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="140">
@@ -3224,11 +3224,116 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
+          <t>29/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C140" t="n">
+        <v>2718</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>29/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C141" t="n">
+        <v>2705</v>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>30/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C142" t="n">
+        <v>2705</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>30/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C143" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>30/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C144" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>31/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C145" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
           <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
-      <c r="C140" t="n">
+      <c r="C146" t="n">
         <v>2706</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>31/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>2704</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-06-01 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -490,27 +490,31 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DIRECT</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>AMS</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
       <c r="D2" t="n">
-        <v>1337</v>
+        <v>1264</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>KLM + Transavia</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2.6</v>
+        <v>13.3</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -520,31 +524,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>AMS</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Amsterdam</t>
-        </is>
-      </c>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
-        <v>1513</v>
+        <v>1340</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>KLM + Transavia</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>13.3</v>
+        <v>2.6</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1680</v>
+        <v>1684</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2404</v>
+        <v>2422</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2574</v>
+        <v>2580</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2704</v>
+        <v>2887</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -827,22 +827,22 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1337</v>
+        <v>1264</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>KLM + Transavia</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>2.6</v>
+        <v>13.3</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>AMS</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -869,22 +869,22 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1513</v>
+        <v>1340</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>KLM + Transavia</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>13.3</v>
+        <v>2.6</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1680</v>
+        <v>1684</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -926,7 +926,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -953,7 +953,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2404</v>
+        <v>2422</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -968,7 +968,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2574</v>
+        <v>2580</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2704</v>
+        <v>2887</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C147"/>
+  <dimension ref="A1:C153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1494,16 +1494,16 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>371</v>
+        <v>1264</v>
       </c>
     </row>
     <row r="26">
@@ -1514,11 +1514,11 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="27">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1574,11 +1574,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="31">
@@ -1589,11 +1589,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="32">
@@ -1604,11 +1604,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="33">
@@ -1619,11 +1619,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="34">
@@ -1634,11 +1634,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="35">
@@ -1649,11 +1649,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="36">
@@ -1664,11 +1664,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="37">
@@ -1679,11 +1679,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="38">
@@ -1694,11 +1694,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="39">
@@ -1709,11 +1709,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="40">
@@ -1724,11 +1724,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="41">
@@ -1739,11 +1739,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="42">
@@ -1754,11 +1754,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="43">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="44">
@@ -1784,11 +1784,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="45">
@@ -1799,11 +1799,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="46">
@@ -1814,26 +1814,26 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>286</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="48">
@@ -1844,11 +1844,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="49">
@@ -1859,7 +1859,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -1904,11 +1904,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="53">
@@ -1919,11 +1919,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1674</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="54">
@@ -1934,11 +1934,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1658</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="55">
@@ -1949,11 +1949,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1654</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="56">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1668</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="57">
@@ -1979,11 +1979,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1667</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="58">
@@ -1994,11 +1994,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1658</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="59">
@@ -2009,11 +2009,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1661</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="60">
@@ -2024,11 +2024,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1663</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="61">
@@ -2039,11 +2039,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2398</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="62">
@@ -2054,11 +2054,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2410</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="63">
@@ -2069,11 +2069,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="64">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -2099,11 +2099,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="66">
@@ -2114,11 +2114,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2329</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="67">
@@ -2129,11 +2129,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="68">
@@ -2144,7 +2144,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -2159,41 +2159,41 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>228</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1329</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="72">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="73">
@@ -2219,7 +2219,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
@@ -2234,7 +2234,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -2264,11 +2264,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="77">
@@ -2279,11 +2279,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="78">
@@ -2294,11 +2294,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1334</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="79">
@@ -2309,11 +2309,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1345</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="80">
@@ -2324,11 +2324,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1344</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="81">
@@ -2339,11 +2339,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1337</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="82">
@@ -2354,11 +2354,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1340</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="83">
@@ -2369,11 +2369,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1341</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="84">
@@ -2384,11 +2384,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1337</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="85">
@@ -2399,11 +2399,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1344</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="86">
@@ -2414,11 +2414,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="87">
@@ -2429,11 +2429,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="88">
@@ -2444,7 +2444,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -2459,7 +2459,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -2504,56 +2504,56 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>404</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>2353</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2353</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="96">
@@ -2564,11 +2564,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="97">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -2594,11 +2594,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="99">
@@ -2609,11 +2609,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="100">
@@ -2624,11 +2624,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="101">
@@ -2639,11 +2639,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2238</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="102">
@@ -2654,11 +2654,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>2257</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="103">
@@ -2669,11 +2669,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2196</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="104">
@@ -2684,11 +2684,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>2185</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="105">
@@ -2699,11 +2699,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2189</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="106">
@@ -2714,11 +2714,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>2191</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="107">
@@ -2729,7 +2729,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -2744,11 +2744,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>2196</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="109">
@@ -2759,11 +2759,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="110">
@@ -2774,11 +2774,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="111">
@@ -2789,11 +2789,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="112">
@@ -2804,7 +2804,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -2819,7 +2819,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -2834,7 +2834,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -2849,71 +2849,71 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>410</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>2391</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>2391</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>2391</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="120">
@@ -2924,11 +2924,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="121">
@@ -2939,11 +2939,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="122">
@@ -2954,11 +2954,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="123">
@@ -2969,11 +2969,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="124">
@@ -2984,11 +2984,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="125">
@@ -2999,11 +2999,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="126">
@@ -3014,11 +3014,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="127">
@@ -3029,11 +3029,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="128">
@@ -3044,11 +3044,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="129">
@@ -3059,11 +3059,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="130">
@@ -3074,11 +3074,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="131">
@@ -3089,11 +3089,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="132">
@@ -3104,11 +3104,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="133">
@@ -3119,11 +3119,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="134">
@@ -3134,11 +3134,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="135">
@@ -3149,11 +3149,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="136">
@@ -3164,11 +3164,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="137">
@@ -3179,11 +3179,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="138">
@@ -3194,86 +3194,86 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>2704</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>2718</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>2705</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2705</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2706</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="144">
@@ -3284,11 +3284,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="145">
@@ -3299,11 +3299,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="146">
@@ -3314,11 +3314,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2706</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="147">
@@ -3329,11 +3329,101 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
+          <t>30/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C147" t="n">
+        <v>2705</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>30/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C148" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>30/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C149" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>31/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C150" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>31/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C151" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
           <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
-      <c r="C147" t="n">
+      <c r="C152" t="n">
         <v>2704</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>01/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>2887</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-06-01 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1264</v>
+        <v>1260</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
-        <v>1340</v>
+        <v>1336</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1684</v>
+        <v>1679</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2422</v>
+        <v>2415</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2580</v>
+        <v>2573</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2887</v>
+        <v>2879</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1264</v>
+        <v>1260</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -842,7 +842,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -869,7 +869,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1340</v>
+        <v>1336</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -884,7 +884,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1684</v>
+        <v>1679</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -926,7 +926,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -953,7 +953,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2422</v>
+        <v>2415</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -968,7 +968,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2580</v>
+        <v>2573</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2887</v>
+        <v>2879</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C153"/>
+  <dimension ref="A1:C159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1509,16 +1509,16 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>371</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="27">
@@ -1529,11 +1529,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="28">
@@ -1544,7 +1544,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1589,11 +1589,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="32">
@@ -1604,11 +1604,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="33">
@@ -1619,11 +1619,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="34">
@@ -1634,11 +1634,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="35">
@@ -1649,11 +1649,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="36">
@@ -1664,11 +1664,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="37">
@@ -1679,11 +1679,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="38">
@@ -1694,11 +1694,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="39">
@@ -1709,11 +1709,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="40">
@@ -1724,11 +1724,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="41">
@@ -1739,11 +1739,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="42">
@@ -1754,11 +1754,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="43">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="44">
@@ -1784,11 +1784,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="45">
@@ -1799,11 +1799,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="46">
@@ -1814,11 +1814,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="47">
@@ -1829,26 +1829,26 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>286</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="49">
@@ -1859,11 +1859,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="50">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -1919,11 +1919,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="54">
@@ -1934,11 +1934,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1674</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="55">
@@ -1949,11 +1949,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1658</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="56">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1654</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="57">
@@ -1979,11 +1979,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1668</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="58">
@@ -1994,11 +1994,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1667</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="59">
@@ -2009,11 +2009,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1658</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="60">
@@ -2024,11 +2024,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1661</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="61">
@@ -2039,11 +2039,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1663</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="62">
@@ -2054,11 +2054,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2398</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="63">
@@ -2069,11 +2069,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2410</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="64">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="65">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -2114,11 +2114,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="67">
@@ -2129,11 +2129,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2329</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="68">
@@ -2144,11 +2144,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="69">
@@ -2159,7 +2159,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -2174,11 +2174,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="71">
@@ -2189,41 +2189,41 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2580</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>228</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1329</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="74">
@@ -2234,11 +2234,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="75">
@@ -2249,7 +2249,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
@@ -2264,7 +2264,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -2294,11 +2294,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="79">
@@ -2309,11 +2309,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="80">
@@ -2324,11 +2324,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1334</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="81">
@@ -2339,11 +2339,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1345</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="82">
@@ -2354,11 +2354,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1344</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="83">
@@ -2369,11 +2369,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1337</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="84">
@@ -2384,11 +2384,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1340</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="85">
@@ -2399,11 +2399,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1341</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="86">
@@ -2414,11 +2414,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1337</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="87">
@@ -2429,11 +2429,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1344</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="88">
@@ -2444,11 +2444,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="90">
@@ -2474,7 +2474,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -2534,11 +2534,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="95">
@@ -2549,56 +2549,56 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>404</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>2353</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>2353</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="99">
@@ -2609,11 +2609,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="100">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -2639,11 +2639,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="102">
@@ -2654,11 +2654,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="103">
@@ -2669,11 +2669,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="104">
@@ -2684,11 +2684,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>2238</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="105">
@@ -2699,11 +2699,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2257</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="106">
@@ -2714,11 +2714,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>2196</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="107">
@@ -2729,11 +2729,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>2185</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="108">
@@ -2744,11 +2744,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>2189</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="109">
@@ -2759,11 +2759,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>2191</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="110">
@@ -2774,7 +2774,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -2789,11 +2789,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>2196</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="112">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="113">
@@ -2819,11 +2819,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="114">
@@ -2834,11 +2834,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="115">
@@ -2849,7 +2849,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -2879,7 +2879,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -2894,11 +2894,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="119">
@@ -2909,71 +2909,71 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>410</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>2391</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>2391</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>2391</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="124">
@@ -2984,11 +2984,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="125">
@@ -2999,11 +2999,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="126">
@@ -3014,11 +3014,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="127">
@@ -3029,11 +3029,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="128">
@@ -3044,11 +3044,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="129">
@@ -3059,11 +3059,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="130">
@@ -3074,11 +3074,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="131">
@@ -3089,11 +3089,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="132">
@@ -3104,11 +3104,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="133">
@@ -3119,11 +3119,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="134">
@@ -3134,11 +3134,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="135">
@@ -3149,11 +3149,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="136">
@@ -3164,11 +3164,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="137">
@@ -3179,11 +3179,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="138">
@@ -3194,11 +3194,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="139">
@@ -3209,11 +3209,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="140">
@@ -3224,11 +3224,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="141">
@@ -3239,11 +3239,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="142">
@@ -3254,11 +3254,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="143">
@@ -3269,86 +3269,86 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>2704</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2718</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2705</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2705</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2706</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="149">
@@ -3359,11 +3359,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="150">
@@ -3374,11 +3374,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="151">
@@ -3389,11 +3389,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2706</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="152">
@@ -3404,11 +3404,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2704</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="153">
@@ -3419,11 +3419,101 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
+          <t>30/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C153" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>30/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C154" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>31/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C155" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>31/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C156" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>31/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C157" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
           <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C153" t="n">
+      <c r="C158" t="n">
         <v>2887</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>01/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>2879</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-06-01 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -554,31 +554,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>London Heathrow</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1679</v>
+        <v>1655</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.5</v>
+        <v>26.2</v>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -588,31 +588,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>London Heathrow</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2415</v>
+        <v>2182</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>14.2</v>
+        <v>12</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2573</v>
+        <v>2571</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2879</v>
+        <v>2877</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -842,7 +842,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -884,7 +884,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -911,22 +911,22 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1679</v>
+        <v>1655</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>15.5</v>
+        <v>26.2</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -953,22 +953,22 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2415</v>
+        <v>2182</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>14.2</v>
+        <v>12</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2573</v>
+        <v>2571</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2879</v>
+        <v>2877</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C159"/>
+  <dimension ref="A1:C165"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1524,16 +1524,16 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>371</v>
+        <v>1259</v>
       </c>
     </row>
     <row r="28">
@@ -1544,11 +1544,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="29">
@@ -1559,7 +1559,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1604,11 +1604,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="33">
@@ -1619,11 +1619,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="34">
@@ -1634,11 +1634,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="35">
@@ -1649,11 +1649,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="36">
@@ -1664,11 +1664,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="37">
@@ -1679,11 +1679,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="38">
@@ -1694,11 +1694,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="39">
@@ -1709,11 +1709,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="40">
@@ -1724,11 +1724,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="41">
@@ -1739,11 +1739,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="42">
@@ -1754,11 +1754,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="43">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="44">
@@ -1784,11 +1784,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="45">
@@ -1799,11 +1799,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="46">
@@ -1814,11 +1814,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="47">
@@ -1829,11 +1829,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="48">
@@ -1844,26 +1844,26 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>286</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="50">
@@ -1874,11 +1874,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="51">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -1919,7 +1919,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -1934,11 +1934,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="55">
@@ -1949,11 +1949,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1674</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="56">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1658</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="57">
@@ -1979,11 +1979,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1654</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="58">
@@ -1994,11 +1994,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1668</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="59">
@@ -2009,11 +2009,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1667</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="60">
@@ -2024,11 +2024,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1658</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="61">
@@ -2039,11 +2039,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1661</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="62">
@@ -2054,11 +2054,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1663</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="63">
@@ -2069,11 +2069,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2398</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="64">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2410</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="65">
@@ -2099,11 +2099,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="66">
@@ -2114,7 +2114,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -2129,11 +2129,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="68">
@@ -2144,11 +2144,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2329</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="69">
@@ -2159,11 +2159,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="70">
@@ -2174,7 +2174,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
@@ -2189,11 +2189,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="72">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2580</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="73">
@@ -2219,41 +2219,41 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2573</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>228</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1329</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="76">
@@ -2264,11 +2264,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="77">
@@ -2279,7 +2279,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
@@ -2309,7 +2309,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -2324,11 +2324,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="81">
@@ -2339,11 +2339,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="82">
@@ -2354,11 +2354,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1334</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="83">
@@ -2369,11 +2369,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1345</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="84">
@@ -2384,11 +2384,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1344</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="85">
@@ -2399,11 +2399,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1337</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="86">
@@ -2414,11 +2414,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1340</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="87">
@@ -2429,11 +2429,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1341</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="88">
@@ -2444,11 +2444,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1337</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1344</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="90">
@@ -2474,11 +2474,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="91">
@@ -2489,11 +2489,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="92">
@@ -2504,7 +2504,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -2519,7 +2519,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -2564,11 +2564,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="97">
@@ -2579,11 +2579,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="98">
@@ -2594,56 +2594,56 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>404</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>2353</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>2353</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="102">
@@ -2654,11 +2654,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="103">
@@ -2669,7 +2669,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -2684,11 +2684,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="105">
@@ -2699,11 +2699,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="106">
@@ -2714,11 +2714,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="107">
@@ -2729,11 +2729,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>2238</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="108">
@@ -2744,11 +2744,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>2257</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="109">
@@ -2759,11 +2759,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>2196</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="110">
@@ -2774,11 +2774,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>2185</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="111">
@@ -2789,11 +2789,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>2189</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="112">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>2191</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="113">
@@ -2819,7 +2819,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -2834,11 +2834,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>2196</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="115">
@@ -2849,11 +2849,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="116">
@@ -2864,11 +2864,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="117">
@@ -2879,11 +2879,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="118">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -2909,7 +2909,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -2924,7 +2924,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -2939,11 +2939,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="122">
@@ -2954,11 +2954,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="123">
@@ -2969,71 +2969,71 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1679</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>410</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2391</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>2391</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>2391</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="128">
@@ -3044,11 +3044,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="129">
@@ -3059,11 +3059,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="130">
@@ -3074,11 +3074,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="131">
@@ -3089,11 +3089,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="132">
@@ -3104,11 +3104,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="133">
@@ -3119,11 +3119,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="134">
@@ -3134,11 +3134,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="135">
@@ -3149,11 +3149,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="136">
@@ -3164,11 +3164,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="137">
@@ -3179,11 +3179,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="138">
@@ -3194,11 +3194,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="139">
@@ -3209,11 +3209,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="140">
@@ -3224,11 +3224,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="141">
@@ -3239,11 +3239,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="142">
@@ -3254,11 +3254,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="143">
@@ -3269,11 +3269,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="144">
@@ -3284,11 +3284,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="145">
@@ -3299,11 +3299,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="146">
@@ -3314,11 +3314,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="147">
@@ -3329,11 +3329,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="148">
@@ -3344,86 +3344,86 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2415</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>2704</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2718</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2705</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2705</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2706</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="154">
@@ -3434,11 +3434,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="155">
@@ -3449,11 +3449,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="156">
@@ -3464,11 +3464,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2706</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="157">
@@ -3479,11 +3479,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2704</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="158">
@@ -3494,11 +3494,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2887</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="159">
@@ -3509,11 +3509,101 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
+          <t>30/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C159" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>31/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C160" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>31/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C161" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>31/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C162" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>01/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C163" t="n">
+        <v>2887</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
           <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
-      <c r="C159" t="n">
+      <c r="C164" t="n">
         <v>2879</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>01/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>2877</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-06-02 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -490,31 +490,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>AMS</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Amsterdam</t>
-        </is>
-      </c>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1259</v>
+        <v>1333</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>KLM + Transavia</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>13.3</v>
+        <v>2.6</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -524,27 +520,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>DIRECT</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr"/>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>London Heathrow</t>
+        </is>
+      </c>
       <c r="D3" t="n">
-        <v>1336</v>
+        <v>1652</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2.6</v>
+        <v>26.2</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -554,31 +554,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>London Heathrow</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1655</v>
+        <v>1675</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>26.2</v>
+        <v>15.5</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -588,31 +588,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>Amsterdam</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2182</v>
+        <v>2023</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>KLM + Icelandair</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>12</v>
+        <v>11.2</v>
       </c>
       <c r="G5" t="n">
         <v>2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2571</v>
+        <v>2566</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2877</v>
+        <v>2843</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -817,7 +817,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>AMS</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -827,22 +827,22 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1259</v>
+        <v>1333</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>KLM + Transavia</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>13.3</v>
+        <v>2.6</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -859,7 +859,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -869,22 +869,22 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1336</v>
+        <v>1652</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>2.6</v>
+        <v>26.2</v>
       </c>
       <c r="I3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -901,7 +901,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -911,22 +911,22 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1655</v>
+        <v>1675</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>26.2</v>
+        <v>15.5</v>
       </c>
       <c r="I4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -943,7 +943,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -953,22 +953,22 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2182</v>
+        <v>2023</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>KLM + Icelandair</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>12</v>
+        <v>11.2</v>
       </c>
       <c r="I5" t="n">
         <v>2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -995,7 +995,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2571</v>
+        <v>2566</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1037,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2877</v>
+        <v>2843</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1052,7 +1052,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C165"/>
+  <dimension ref="A1:C171"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1539,16 +1539,16 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>371</v>
+        <v>2023</v>
       </c>
     </row>
     <row r="29">
@@ -1559,11 +1559,11 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="30">
@@ -1574,7 +1574,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -1604,7 +1604,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1619,11 +1619,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="34">
@@ -1634,11 +1634,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="35">
@@ -1649,11 +1649,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="36">
@@ -1664,11 +1664,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="37">
@@ -1679,11 +1679,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="38">
@@ -1694,11 +1694,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="39">
@@ -1709,11 +1709,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="40">
@@ -1724,11 +1724,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="41">
@@ -1739,11 +1739,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="42">
@@ -1754,11 +1754,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="43">
@@ -1769,11 +1769,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="44">
@@ -1784,11 +1784,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="45">
@@ -1799,11 +1799,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="46">
@@ -1814,11 +1814,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="47">
@@ -1829,11 +1829,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="48">
@@ -1844,11 +1844,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="49">
@@ -1859,26 +1859,26 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>286</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="51">
@@ -1889,11 +1889,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="52">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -1949,11 +1949,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="56">
@@ -1964,11 +1964,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1674</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="57">
@@ -1979,11 +1979,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1658</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="58">
@@ -1994,11 +1994,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1654</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="59">
@@ -2009,11 +2009,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1668</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="60">
@@ -2024,11 +2024,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1667</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="61">
@@ -2039,11 +2039,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1658</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="62">
@@ -2054,11 +2054,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1661</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="63">
@@ -2069,11 +2069,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1663</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="64">
@@ -2084,11 +2084,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2398</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="65">
@@ -2099,11 +2099,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2410</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="66">
@@ -2114,11 +2114,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="67">
@@ -2129,7 +2129,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -2144,11 +2144,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="69">
@@ -2159,11 +2159,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2329</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="70">
@@ -2174,11 +2174,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="71">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -2204,11 +2204,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="73">
@@ -2219,11 +2219,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2580</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="74">
@@ -2234,11 +2234,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2573</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="75">
@@ -2249,41 +2249,41 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2571</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>228</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1329</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="78">
@@ -2294,11 +2294,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="79">
@@ -2309,7 +2309,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
@@ -2324,7 +2324,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
@@ -2354,11 +2354,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="83">
@@ -2369,11 +2369,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="84">
@@ -2384,11 +2384,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1334</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="85">
@@ -2399,11 +2399,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1345</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="86">
@@ -2414,11 +2414,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1344</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="87">
@@ -2429,11 +2429,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1337</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="88">
@@ -2444,11 +2444,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1340</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2459,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1341</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="90">
@@ -2474,11 +2474,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1337</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="91">
@@ -2489,11 +2489,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1344</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="92">
@@ -2504,11 +2504,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="93">
@@ -2519,11 +2519,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="94">
@@ -2534,7 +2534,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -2549,7 +2549,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -2564,7 +2564,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
@@ -2579,7 +2579,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -2594,11 +2594,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="99">
@@ -2609,11 +2609,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="100">
@@ -2624,11 +2624,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="101">
@@ -2639,56 +2639,56 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>404</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>2353</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>2353</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="105">
@@ -2699,11 +2699,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="106">
@@ -2714,7 +2714,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -2729,11 +2729,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="108">
@@ -2744,11 +2744,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="109">
@@ -2759,11 +2759,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="110">
@@ -2774,11 +2774,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>2238</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="111">
@@ -2789,11 +2789,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>2257</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="112">
@@ -2804,11 +2804,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>2196</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="113">
@@ -2819,11 +2819,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>2185</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="114">
@@ -2834,11 +2834,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>2189</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="115">
@@ -2849,11 +2849,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2191</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="116">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -2879,11 +2879,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>2196</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="118">
@@ -2894,11 +2894,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="119">
@@ -2909,11 +2909,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="120">
@@ -2924,11 +2924,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="121">
@@ -2939,7 +2939,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -2954,7 +2954,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -2969,7 +2969,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -2984,11 +2984,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="125">
@@ -2999,11 +2999,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="126">
@@ -3014,11 +3014,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1679</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="127">
@@ -3029,71 +3029,71 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>2182</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>410</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>2391</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2391</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2391</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="132">
@@ -3104,11 +3104,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="133">
@@ -3119,11 +3119,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="134">
@@ -3134,11 +3134,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="135">
@@ -3149,11 +3149,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="136">
@@ -3164,11 +3164,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="137">
@@ -3179,11 +3179,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="138">
@@ -3194,11 +3194,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="139">
@@ -3209,11 +3209,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="140">
@@ -3224,11 +3224,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="141">
@@ -3239,11 +3239,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="142">
@@ -3254,11 +3254,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="143">
@@ -3269,11 +3269,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="144">
@@ -3284,11 +3284,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="145">
@@ -3299,11 +3299,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="146">
@@ -3314,11 +3314,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="147">
@@ -3329,11 +3329,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="148">
@@ -3344,11 +3344,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="149">
@@ -3359,11 +3359,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="150">
@@ -3374,11 +3374,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="151">
@@ -3389,11 +3389,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="152">
@@ -3404,11 +3404,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2415</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="153">
@@ -3419,86 +3419,86 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>1655</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2704</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2718</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2705</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2705</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2706</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="159">
@@ -3509,11 +3509,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="160">
@@ -3524,11 +3524,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="161">
@@ -3539,11 +3539,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2706</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="162">
@@ -3554,11 +3554,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2704</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="163">
@@ -3569,11 +3569,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2887</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="164">
@@ -3584,11 +3584,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2879</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="165">
@@ -3599,11 +3599,101 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
+          <t>31/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C165" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>31/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C166" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>31/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C167" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>01/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C168" t="n">
+        <v>2887</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>01/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C169" t="n">
+        <v>2879</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
           <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
-      <c r="C165" t="n">
+      <c r="C170" t="n">
         <v>2877</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>02/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>2843</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-06-02 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H8"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1652</v>
+        <v>1651</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1675</v>
+        <v>1674</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -588,31 +588,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>AMS</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Stockholm</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2023</v>
+        <v>2360</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>KLM + Icelandair</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>11.2</v>
+        <v>16.2</v>
       </c>
       <c r="G5" t="n">
         <v>2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2566</v>
+        <v>2553</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -639,14 +639,14 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7</v>
+        <v>22.2</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -686,36 +686,66 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ARN</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Stockholm</t>
-        </is>
-      </c>
+          <t>HEL</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>2915</v>
+        <v>2848</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>15.4</v>
+        <v>7.8</v>
       </c>
       <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>02/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>AMS</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>2855</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>KLM + Air Baltic</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="G9" t="n">
         <v>2</v>
       </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>31/05/2026 20:19 BRT</t>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D8">
+  <conditionalFormatting sqref="D2:D9">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -737,7 +767,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -827,7 +857,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1333</v>
+        <v>1332</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -842,7 +872,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -869,7 +899,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1652</v>
+        <v>1651</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -884,7 +914,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -911,7 +941,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1675</v>
+        <v>1674</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -926,7 +956,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -943,7 +973,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>AMS</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -953,22 +983,22 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2023</v>
+        <v>2360</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>KLM + Icelandair</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>11.2</v>
+        <v>16.2</v>
       </c>
       <c r="I5" t="n">
         <v>2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -995,7 +1025,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2566</v>
+        <v>2553</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1003,14 +1033,14 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>7</v>
+        <v>22.2</v>
       </c>
       <c r="I6" t="n">
         <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1069,7 +1099,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1079,27 +1109,69 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2915</v>
+        <v>2848</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>15.4</v>
+        <v>7.8</v>
       </c>
       <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>02/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>KEF</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>AMS</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="n">
+        <v>2855</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>KLM + Air Baltic</t>
+        </is>
+      </c>
+      <c r="H9" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="I9" t="n">
         <v>2</v>
       </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>31/05/2026 20:19 BRT</t>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F8">
+  <conditionalFormatting sqref="F2:F9">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1121,7 +1193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C171"/>
+  <dimension ref="A1:C178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1554,16 +1626,16 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>371</v>
+        <v>2855</v>
       </c>
     </row>
     <row r="30">
@@ -1574,11 +1646,11 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="31">
@@ -1589,7 +1661,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -1619,7 +1691,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1634,11 +1706,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="35">
@@ -1649,11 +1721,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="36">
@@ -1664,11 +1736,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="37">
@@ -1679,11 +1751,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="38">
@@ -1694,11 +1766,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="39">
@@ -1709,11 +1781,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="40">
@@ -1724,11 +1796,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="41">
@@ -1739,11 +1811,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="42">
@@ -1754,11 +1826,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="43">
@@ -1769,11 +1841,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="44">
@@ -1784,11 +1856,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="45">
@@ -1799,11 +1871,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="46">
@@ -1814,11 +1886,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="47">
@@ -1829,11 +1901,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="48">
@@ -1844,11 +1916,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="49">
@@ -1859,11 +1931,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="50">
@@ -1874,41 +1946,41 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>286</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>1649</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="53">
@@ -1919,11 +1991,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="54">
@@ -1934,7 +2006,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -1949,7 +2021,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -1964,11 +2036,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="57">
@@ -1979,11 +2051,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="58">
@@ -1994,11 +2066,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="59">
@@ -2009,11 +2081,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="60">
@@ -2024,11 +2096,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="61">
@@ -2039,11 +2111,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="62">
@@ -2054,11 +2126,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="63">
@@ -2069,11 +2141,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="64">
@@ -2084,11 +2156,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="65">
@@ -2099,11 +2171,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="66">
@@ -2114,11 +2186,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="67">
@@ -2129,11 +2201,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2575</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="68">
@@ -2144,11 +2216,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="69">
@@ -2159,11 +2231,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="70">
@@ -2174,11 +2246,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="71">
@@ -2189,11 +2261,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2575</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="72">
@@ -2204,11 +2276,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="73">
@@ -2219,11 +2291,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="74">
@@ -2234,11 +2306,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2580</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="75">
@@ -2249,11 +2321,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2573</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="76">
@@ -2264,11 +2336,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2571</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="77">
@@ -2279,56 +2351,56 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2566</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>228</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1329</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1329</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="81">
@@ -2339,11 +2411,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="82">
@@ -2354,7 +2426,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
@@ -2369,7 +2441,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
@@ -2384,11 +2456,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="85">
@@ -2399,11 +2471,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="86">
@@ -2414,11 +2486,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="87">
@@ -2429,11 +2501,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="88">
@@ -2444,11 +2516,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="89">
@@ -2459,11 +2531,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="90">
@@ -2474,11 +2546,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="91">
@@ -2489,11 +2561,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="92">
@@ -2504,7 +2576,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -2519,11 +2591,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="94">
@@ -2534,11 +2606,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1338</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="95">
@@ -2549,11 +2621,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="96">
@@ -2564,11 +2636,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="97">
@@ -2579,7 +2651,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -2594,7 +2666,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -2609,7 +2681,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
@@ -2624,11 +2696,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="101">
@@ -2639,11 +2711,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="102">
@@ -2654,11 +2726,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1336</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="103">
@@ -2669,11 +2741,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="104">
@@ -2684,71 +2756,71 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1333</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>404</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>2353</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>2353</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>2353</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="109">
@@ -2759,11 +2831,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="110">
@@ -2774,11 +2846,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="111">
@@ -2789,11 +2861,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="112">
@@ -2804,11 +2876,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="113">
@@ -2819,11 +2891,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="114">
@@ -2834,11 +2906,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="115">
@@ -2849,11 +2921,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="116">
@@ -2864,11 +2936,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="117">
@@ -2879,11 +2951,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="118">
@@ -2894,11 +2966,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="119">
@@ -2909,11 +2981,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="120">
@@ -2924,11 +2996,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="121">
@@ -2939,11 +3011,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="122">
@@ -2954,11 +3026,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="123">
@@ -2969,11 +3041,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="124">
@@ -2984,11 +3056,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="125">
@@ -2999,7 +3071,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -3014,7 +3086,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -3029,11 +3101,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="128">
@@ -3044,11 +3116,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="129">
@@ -3059,11 +3131,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>1679</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="130">
@@ -3074,11 +3146,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2182</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="131">
@@ -3089,101 +3161,101 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1675</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>410</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2391</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2391</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2391</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>2391</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>2389</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="138">
@@ -3194,11 +3266,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>2402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="139">
@@ -3209,11 +3281,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="140">
@@ -3224,11 +3296,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="141">
@@ -3239,11 +3311,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="142">
@@ -3254,11 +3326,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1660</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="143">
@@ -3269,11 +3341,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1652</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="144">
@@ -3284,11 +3356,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1655</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="145">
@@ -3299,11 +3371,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2411</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="146">
@@ -3314,11 +3386,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2404</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="147">
@@ -3329,11 +3401,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2416</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="148">
@@ -3344,11 +3416,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2405</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="149">
@@ -3359,11 +3431,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="150">
@@ -3374,11 +3446,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2406</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="151">
@@ -3389,11 +3461,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2406</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="152">
@@ -3404,11 +3476,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="153">
@@ -3419,11 +3491,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>1652</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="154">
@@ -3434,11 +3506,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2404</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="155">
@@ -3449,11 +3521,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2422</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="156">
@@ -3464,11 +3536,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2415</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="157">
@@ -3479,11 +3551,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>1655</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="158">
@@ -3494,7 +3566,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -3504,106 +3576,106 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2704</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2718</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2705</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2705</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2706</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2706</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2706</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="166">
@@ -3614,11 +3686,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="167">
@@ -3629,11 +3701,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2704</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="168">
@@ -3644,11 +3716,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="169">
@@ -3659,11 +3731,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2879</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="170">
@@ -3674,11 +3746,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="171">
@@ -3689,10 +3761,115 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
+          <t>30/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C171" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>31/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C172" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>31/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C173" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>31/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C174" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>01/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C175" t="n">
+        <v>2887</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>01/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C176" t="n">
+        <v>2879</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>01/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C177" t="n">
+        <v>2877</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
           <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C171" t="n">
+      <c r="C178" t="n">
         <v>2843</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-06-02 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1332</v>
+        <v>1329</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1651</v>
+        <v>1648</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1674</v>
+        <v>1670</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -588,16 +588,16 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Stockholm</t>
+          <t>Copenhagen</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2360</v>
+        <v>2559</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -605,14 +605,14 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>16.2</v>
+        <v>7</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -622,16 +622,16 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Copenhagen</t>
+          <t>Stockholm</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2553</v>
+        <v>2759</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -639,14 +639,14 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>22.2</v>
+        <v>15.4</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2843</v>
+        <v>2835</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>2848</v>
+        <v>2842</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -706,7 +706,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2855</v>
+        <v>2849</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -740,7 +740,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -857,7 +857,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1332</v>
+        <v>1329</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -872,7 +872,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1651</v>
+        <v>1648</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1674</v>
+        <v>1670</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -956,7 +956,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -973,7 +973,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2360</v>
+        <v>2559</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -991,14 +991,14 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>16.2</v>
+        <v>7</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1025,7 +1025,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2553</v>
+        <v>2759</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1033,14 +1033,14 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>22.2</v>
+        <v>15.4</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2843</v>
+        <v>2835</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1082,7 +1082,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1109,7 +1109,7 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2848</v>
+        <v>2842</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1124,7 +1124,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1151,7 +1151,7 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>2855</v>
+        <v>2849</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1166,7 +1166,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C178"/>
+  <dimension ref="A1:C186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1641,16 +1641,16 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>371</v>
+        <v>2849</v>
       </c>
     </row>
     <row r="31">
@@ -1661,11 +1661,11 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="32">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -1706,7 +1706,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1721,11 +1721,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="36">
@@ -1736,11 +1736,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="37">
@@ -1751,11 +1751,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="38">
@@ -1766,11 +1766,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="39">
@@ -1781,11 +1781,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="40">
@@ -1796,11 +1796,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="41">
@@ -1811,11 +1811,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="42">
@@ -1826,11 +1826,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="43">
@@ -1841,11 +1841,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="44">
@@ -1856,11 +1856,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="45">
@@ -1871,11 +1871,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="46">
@@ -1886,11 +1886,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="47">
@@ -1901,11 +1901,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="48">
@@ -1916,11 +1916,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="49">
@@ -1931,11 +1931,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="50">
@@ -1946,11 +1946,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="51">
@@ -1961,11 +1961,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="52">
@@ -1976,41 +1976,41 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2360</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>286</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>1649</v>
+        <v>2759</v>
       </c>
     </row>
     <row r="55">
@@ -2021,11 +2021,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="56">
@@ -2036,7 +2036,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -2051,7 +2051,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -2066,11 +2066,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="59">
@@ -2081,11 +2081,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="60">
@@ -2096,11 +2096,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="61">
@@ -2111,11 +2111,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="62">
@@ -2126,11 +2126,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="63">
@@ -2141,11 +2141,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="64">
@@ -2156,11 +2156,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="65">
@@ -2171,11 +2171,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="66">
@@ -2186,11 +2186,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="67">
@@ -2201,11 +2201,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="68">
@@ -2216,11 +2216,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="69">
@@ -2231,11 +2231,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2575</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="70">
@@ -2246,11 +2246,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="71">
@@ -2261,11 +2261,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="72">
@@ -2276,11 +2276,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="73">
@@ -2291,11 +2291,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2575</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="74">
@@ -2306,11 +2306,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="75">
@@ -2321,11 +2321,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="76">
@@ -2336,11 +2336,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2580</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="77">
@@ -2351,11 +2351,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2573</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="78">
@@ -2366,11 +2366,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2571</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="79">
@@ -2381,11 +2381,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2566</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="80">
@@ -2396,56 +2396,56 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2553</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>228</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>1329</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>1329</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="84">
@@ -2456,11 +2456,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="85">
@@ -2471,7 +2471,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
@@ -2486,7 +2486,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
@@ -2501,11 +2501,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="88">
@@ -2516,11 +2516,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="89">
@@ -2531,11 +2531,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="90">
@@ -2546,11 +2546,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="91">
@@ -2561,11 +2561,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="92">
@@ -2576,11 +2576,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="93">
@@ -2591,11 +2591,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="94">
@@ -2606,11 +2606,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="95">
@@ -2621,7 +2621,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -2636,11 +2636,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="97">
@@ -2651,11 +2651,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1338</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="98">
@@ -2666,11 +2666,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="99">
@@ -2681,11 +2681,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="100">
@@ -2696,7 +2696,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -2711,7 +2711,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -2726,7 +2726,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
@@ -2741,11 +2741,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="104">
@@ -2756,11 +2756,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="105">
@@ -2771,11 +2771,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1336</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="106">
@@ -2786,11 +2786,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="107">
@@ -2801,11 +2801,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1333</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="108">
@@ -2816,71 +2816,71 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1332</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>404</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>2353</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>2353</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>2353</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="113">
@@ -2891,11 +2891,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="114">
@@ -2906,11 +2906,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="115">
@@ -2921,11 +2921,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="116">
@@ -2936,11 +2936,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="117">
@@ -2951,11 +2951,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="118">
@@ -2966,11 +2966,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="119">
@@ -2981,11 +2981,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="120">
@@ -2996,11 +2996,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="121">
@@ -3011,11 +3011,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="122">
@@ -3026,11 +3026,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="123">
@@ -3041,11 +3041,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="124">
@@ -3056,11 +3056,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="125">
@@ -3071,11 +3071,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="126">
@@ -3086,11 +3086,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="127">
@@ -3101,11 +3101,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="128">
@@ -3116,11 +3116,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="129">
@@ -3131,7 +3131,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -3146,7 +3146,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -3161,11 +3161,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="132">
@@ -3176,11 +3176,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="133">
@@ -3191,11 +3191,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1679</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="134">
@@ -3206,11 +3206,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2182</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="135">
@@ -3221,11 +3221,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1675</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="136">
@@ -3236,116 +3236,116 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1674</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>2848</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>410</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>2391</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>2391</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>2391</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2391</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2389</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="144">
@@ -3356,11 +3356,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>2402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="145">
@@ -3371,11 +3371,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="146">
@@ -3386,11 +3386,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="147">
@@ -3401,11 +3401,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="148">
@@ -3416,11 +3416,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>1660</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="149">
@@ -3431,11 +3431,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>1652</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="150">
@@ -3446,11 +3446,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>1655</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="151">
@@ -3461,11 +3461,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2411</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="152">
@@ -3476,11 +3476,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2404</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="153">
@@ -3491,11 +3491,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2416</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="154">
@@ -3506,11 +3506,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2405</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="155">
@@ -3521,11 +3521,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="156">
@@ -3536,11 +3536,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2406</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="157">
@@ -3551,11 +3551,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2406</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="158">
@@ -3566,11 +3566,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="159">
@@ -3581,11 +3581,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>1652</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="160">
@@ -3596,11 +3596,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2404</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="161">
@@ -3611,11 +3611,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2422</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="162">
@@ -3626,11 +3626,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2415</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="163">
@@ -3641,11 +3641,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>1655</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="164">
@@ -3656,7 +3656,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -3671,116 +3671,116 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>1651</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2704</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2718</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2705</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2705</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2706</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>2706</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>2706</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="173">
@@ -3791,11 +3791,11 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="174">
@@ -3806,11 +3806,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>2704</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="175">
@@ -3821,11 +3821,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="176">
@@ -3836,11 +3836,11 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>2879</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="177">
@@ -3851,11 +3851,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="178">
@@ -3866,11 +3866,131 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
+          <t>30/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C178" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>31/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C179" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>31/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C180" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>31/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C181" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>01/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C182" t="n">
+        <v>2887</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>01/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C183" t="n">
+        <v>2879</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>01/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C184" t="n">
+        <v>2877</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
           <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C178" t="n">
+      <c r="C185" t="n">
         <v>2843</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>02/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>2835</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-06-03 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1329</v>
+        <v>1324</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1648</v>
+        <v>1558</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1670</v>
+        <v>1664</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2559</v>
+        <v>2550</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -631,7 +631,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2759</v>
+        <v>2749</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -656,27 +656,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2835</v>
+        <v>2831</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>11.4</v>
+        <v>7.8</v>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -686,27 +686,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HEL</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>AMS</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
       <c r="D8" t="n">
-        <v>2842</v>
+        <v>2838</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>KLM + Air Baltic</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>7.8</v>
+        <v>11.5</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -716,31 +720,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AMS</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Amsterdam</t>
-        </is>
-      </c>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
-        <v>2849</v>
+        <v>2940</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>KLM + Air Baltic</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="G9" t="n">
         <v>2</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -857,7 +857,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1329</v>
+        <v>1324</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -872,7 +872,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -899,7 +899,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1648</v>
+        <v>1558</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -914,7 +914,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1670</v>
+        <v>1664</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -956,7 +956,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2559</v>
+        <v>2550</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1025,7 +1025,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2759</v>
+        <v>2749</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1057,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1067,22 +1067,22 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2835</v>
+        <v>2831</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>11.4</v>
+        <v>7.8</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1109,22 +1109,22 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2842</v>
+        <v>2838</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>KLM + Air Baltic</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>7.8</v>
+        <v>11.5</v>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AMS</t>
+          <t>ZRH</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1151,22 +1151,22 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>2849</v>
+        <v>2940</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>KLM + Air Baltic</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="I9" t="n">
         <v>2</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1193,7 +1193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C186"/>
+  <dimension ref="A1:C194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1656,16 +1656,16 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>371</v>
+        <v>2838</v>
       </c>
     </row>
     <row r="32">
@@ -1676,11 +1676,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="33">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
@@ -1721,7 +1721,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1736,11 +1736,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="37">
@@ -1751,11 +1751,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="38">
@@ -1766,11 +1766,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="39">
@@ -1781,11 +1781,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="40">
@@ -1796,11 +1796,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="41">
@@ -1811,11 +1811,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="42">
@@ -1826,11 +1826,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="43">
@@ -1841,11 +1841,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="44">
@@ -1856,11 +1856,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="45">
@@ -1871,11 +1871,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="46">
@@ -1886,11 +1886,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="47">
@@ -1901,11 +1901,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="48">
@@ -1916,11 +1916,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="49">
@@ -1931,11 +1931,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="50">
@@ -1946,11 +1946,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="51">
@@ -1961,11 +1961,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="52">
@@ -1976,11 +1976,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="53">
@@ -1991,11 +1991,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2360</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="54">
@@ -2006,41 +2006,41 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2759</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>286</v>
+        <v>2759</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>1649</v>
+        <v>2749</v>
       </c>
     </row>
     <row r="57">
@@ -2051,11 +2051,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="58">
@@ -2066,7 +2066,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -2081,7 +2081,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -2096,11 +2096,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="61">
@@ -2111,11 +2111,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="62">
@@ -2126,11 +2126,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="63">
@@ -2141,11 +2141,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="64">
@@ -2156,11 +2156,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="65">
@@ -2171,11 +2171,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="66">
@@ -2186,11 +2186,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="67">
@@ -2201,11 +2201,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="68">
@@ -2216,11 +2216,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="69">
@@ -2231,11 +2231,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="70">
@@ -2246,11 +2246,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="71">
@@ -2261,11 +2261,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2575</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="72">
@@ -2276,11 +2276,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="73">
@@ -2291,11 +2291,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="74">
@@ -2306,11 +2306,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="75">
@@ -2321,11 +2321,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2575</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="76">
@@ -2336,11 +2336,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="77">
@@ -2351,11 +2351,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="78">
@@ -2366,11 +2366,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2580</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="79">
@@ -2381,11 +2381,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2573</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="80">
@@ -2396,11 +2396,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2571</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="81">
@@ -2411,11 +2411,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2566</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="82">
@@ -2426,11 +2426,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2553</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="83">
@@ -2441,56 +2441,56 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2559</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>228</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>1329</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>1329</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="87">
@@ -2501,11 +2501,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="88">
@@ -2516,7 +2516,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -2531,7 +2531,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
@@ -2546,11 +2546,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="91">
@@ -2561,11 +2561,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="92">
@@ -2576,11 +2576,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="93">
@@ -2591,11 +2591,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="94">
@@ -2606,11 +2606,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="95">
@@ -2621,11 +2621,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="96">
@@ -2636,11 +2636,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="97">
@@ -2651,11 +2651,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="98">
@@ -2666,7 +2666,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -2681,11 +2681,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="100">
@@ -2696,11 +2696,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1338</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="101">
@@ -2711,11 +2711,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="102">
@@ -2726,11 +2726,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="103">
@@ -2741,7 +2741,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -2756,7 +2756,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -2771,7 +2771,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -2786,11 +2786,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="107">
@@ -2801,11 +2801,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="108">
@@ -2816,11 +2816,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1336</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="109">
@@ -2831,11 +2831,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="110">
@@ -2846,11 +2846,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1333</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="111">
@@ -2861,11 +2861,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1332</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="112">
@@ -2876,71 +2876,71 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1329</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>404</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>2353</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>2353</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>2353</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="117">
@@ -2951,11 +2951,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="118">
@@ -2966,11 +2966,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="119">
@@ -2981,11 +2981,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="120">
@@ -2996,11 +2996,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="121">
@@ -3011,11 +3011,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="122">
@@ -3026,11 +3026,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="123">
@@ -3041,11 +3041,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="124">
@@ -3056,11 +3056,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="125">
@@ -3071,11 +3071,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="126">
@@ -3086,11 +3086,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="127">
@@ -3101,11 +3101,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="128">
@@ -3116,11 +3116,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="129">
@@ -3131,11 +3131,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="130">
@@ -3146,11 +3146,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="131">
@@ -3161,11 +3161,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="132">
@@ -3176,11 +3176,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="133">
@@ -3191,7 +3191,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -3206,7 +3206,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -3221,11 +3221,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="136">
@@ -3236,11 +3236,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="137">
@@ -3251,11 +3251,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1679</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="138">
@@ -3266,11 +3266,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>2182</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="139">
@@ -3281,11 +3281,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1675</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="140">
@@ -3296,11 +3296,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1674</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="141">
@@ -3311,131 +3311,131 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1670</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2848</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2842</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>410</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2391</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2391</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2391</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2391</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>2389</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="150">
@@ -3446,11 +3446,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="151">
@@ -3461,11 +3461,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="152">
@@ -3476,11 +3476,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="153">
@@ -3491,11 +3491,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="154">
@@ -3506,11 +3506,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>1660</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="155">
@@ -3521,11 +3521,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>1652</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="156">
@@ -3536,11 +3536,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>1655</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="157">
@@ -3551,11 +3551,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2411</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="158">
@@ -3566,11 +3566,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2404</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="159">
@@ -3581,11 +3581,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2416</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="160">
@@ -3596,11 +3596,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2405</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="161">
@@ -3611,11 +3611,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="162">
@@ -3626,11 +3626,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2406</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="163">
@@ -3641,11 +3641,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2406</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="164">
@@ -3656,11 +3656,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="165">
@@ -3671,11 +3671,11 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>1652</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="166">
@@ -3686,11 +3686,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2404</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="167">
@@ -3701,11 +3701,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2422</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="168">
@@ -3716,11 +3716,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2415</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="169">
@@ -3731,11 +3731,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1655</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="170">
@@ -3746,7 +3746,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -3761,11 +3761,11 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1651</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="172">
@@ -3776,116 +3776,116 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1648</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>2704</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>2718</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>2705</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>2705</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>2706</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>2706</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>2706</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="180">
@@ -3896,11 +3896,11 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="181">
@@ -3911,11 +3911,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>2704</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="182">
@@ -3926,11 +3926,11 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="183">
@@ -3941,11 +3941,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>2879</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="184">
@@ -3956,11 +3956,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="185">
@@ -3971,11 +3971,11 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="186">
@@ -3986,11 +3986,131 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
+          <t>31/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C186" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>31/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C187" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>31/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C188" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>01/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C189" t="n">
+        <v>2887</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>01/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C190" t="n">
+        <v>2879</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>01/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C191" t="n">
+        <v>2877</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>02/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C192" t="n">
+        <v>2843</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
           <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
-      <c r="C186" t="n">
+      <c r="C193" t="n">
         <v>2835</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>2940</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-06-03 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1324</v>
+        <v>1344</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -520,31 +520,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>London Heathrow</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1558</v>
+        <v>1688</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>26.2</v>
+        <v>15.5</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -554,31 +554,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Frankfurt</t>
-        </is>
-      </c>
+          <t>MUC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>1664</v>
+        <v>1692</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.5</v>
+        <v>13.8</v>
       </c>
       <c r="G4" t="n">
         <v>2</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +593,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2550</v>
+        <v>1849</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -605,14 +601,14 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>7</v>
+        <v>15.6</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -622,31 +618,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Stockholm</t>
+          <t>London Heathrow</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2749</v>
+        <v>2428</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>15.4</v>
+        <v>14.2</v>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -656,27 +652,31 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>HEL</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr"/>
+          <t>ARN</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Stockholm</t>
+        </is>
+      </c>
       <c r="D7" t="n">
-        <v>2831</v>
+        <v>2788</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>7.8</v>
+        <v>15.4</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -686,31 +686,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AMS</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Amsterdam</t>
-        </is>
-      </c>
+          <t>HEL</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>2838</v>
+        <v>2872</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>KLM + Air Baltic</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>11.5</v>
+        <v>7.8</v>
       </c>
       <c r="G8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -720,32 +716,66 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ZRH</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>AMS</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
       <c r="D9" t="n">
-        <v>2940</v>
+        <v>2879</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>KLM + Air Baltic</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="G9" t="n">
         <v>2</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>2983</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>SWISS + Lufthansa</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D9">
+  <conditionalFormatting sqref="D2:D10">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -767,7 +797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -857,7 +887,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1324</v>
+        <v>1344</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -872,7 +902,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -889,7 +919,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -899,22 +929,22 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1558</v>
+        <v>1688</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>26.2</v>
+        <v>15.5</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -931,7 +961,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -941,22 +971,22 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1664</v>
+        <v>1692</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>15.5</v>
+        <v>13.8</v>
       </c>
       <c r="I4" t="n">
         <v>2</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -983,7 +1013,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2550</v>
+        <v>1849</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -991,14 +1021,14 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>7</v>
+        <v>15.6</v>
       </c>
       <c r="I5" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1045,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1025,22 +1055,22 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2749</v>
+        <v>2428</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>15.4</v>
+        <v>14.2</v>
       </c>
       <c r="I6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1057,7 +1087,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1067,22 +1097,22 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2831</v>
+        <v>2788</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>7.8</v>
+        <v>15.4</v>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1099,7 +1129,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMS</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1109,22 +1139,22 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2838</v>
+        <v>2872</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>KLM + Air Baltic</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>11.5</v>
+        <v>7.8</v>
       </c>
       <c r="I8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1171,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1151,27 +1181,69 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>2940</v>
+        <v>2879</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>KLM + Air Baltic</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="I9" t="n">
         <v>2</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>KEF</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="n">
+        <v>2983</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>SWISS + Lufthansa</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F9">
+  <conditionalFormatting sqref="F2:F10">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1193,7 +1265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C194"/>
+  <dimension ref="A1:C203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1671,16 +1743,16 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>371</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="33">
@@ -1691,11 +1763,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="34">
@@ -1706,7 +1778,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
@@ -1736,7 +1808,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -1751,11 +1823,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="38">
@@ -1766,11 +1838,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="39">
@@ -1781,11 +1853,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="40">
@@ -1796,11 +1868,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="41">
@@ -1811,11 +1883,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="42">
@@ -1826,11 +1898,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="43">
@@ -1841,11 +1913,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="44">
@@ -1856,11 +1928,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="45">
@@ -1871,11 +1943,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="46">
@@ -1886,11 +1958,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="47">
@@ -1901,11 +1973,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="48">
@@ -1916,11 +1988,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="49">
@@ -1931,11 +2003,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="50">
@@ -1946,11 +2018,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="51">
@@ -1961,11 +2033,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="52">
@@ -1976,11 +2048,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="53">
@@ -1991,11 +2063,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="54">
@@ -2006,11 +2078,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2360</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="55">
@@ -2021,11 +2093,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2759</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="56">
@@ -2036,41 +2108,41 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2749</v>
+        <v>2759</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>286</v>
+        <v>2749</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>1649</v>
+        <v>2788</v>
       </c>
     </row>
     <row r="59">
@@ -2081,11 +2153,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="60">
@@ -2096,7 +2168,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -2111,7 +2183,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -2126,11 +2198,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="63">
@@ -2141,11 +2213,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="64">
@@ -2156,11 +2228,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="65">
@@ -2171,11 +2243,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="66">
@@ -2186,11 +2258,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="67">
@@ -2201,11 +2273,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="68">
@@ -2216,11 +2288,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="69">
@@ -2231,11 +2303,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="70">
@@ -2246,11 +2318,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="71">
@@ -2261,11 +2333,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="72">
@@ -2276,11 +2348,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="73">
@@ -2291,11 +2363,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2575</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="74">
@@ -2306,11 +2378,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="75">
@@ -2321,11 +2393,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="76">
@@ -2336,11 +2408,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="77">
@@ -2351,11 +2423,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2575</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="78">
@@ -2366,11 +2438,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="79">
@@ -2381,11 +2453,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="80">
@@ -2396,11 +2468,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2580</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="81">
@@ -2411,11 +2483,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2573</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="82">
@@ -2426,11 +2498,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2571</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="83">
@@ -2441,11 +2513,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2566</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="84">
@@ -2456,11 +2528,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2553</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="85">
@@ -2471,11 +2543,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2559</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="86">
@@ -2486,56 +2558,56 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2550</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>228</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>1329</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1329</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="90">
@@ -2546,11 +2618,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="91">
@@ -2561,7 +2633,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
@@ -2576,7 +2648,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
@@ -2591,11 +2663,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="94">
@@ -2606,11 +2678,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="95">
@@ -2621,11 +2693,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="96">
@@ -2636,11 +2708,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="97">
@@ -2651,11 +2723,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="98">
@@ -2666,11 +2738,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="99">
@@ -2681,11 +2753,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="100">
@@ -2696,11 +2768,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="101">
@@ -2711,7 +2783,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -2726,11 +2798,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="103">
@@ -2741,11 +2813,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1338</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="104">
@@ -2756,11 +2828,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="105">
@@ -2771,11 +2843,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="106">
@@ -2786,7 +2858,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -2801,7 +2873,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -2816,7 +2888,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -2831,11 +2903,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="110">
@@ -2846,11 +2918,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="111">
@@ -2861,11 +2933,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1336</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="112">
@@ -2876,11 +2948,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="113">
@@ -2891,11 +2963,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1333</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="114">
@@ -2906,11 +2978,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1332</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="115">
@@ -2921,11 +2993,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1329</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="116">
@@ -2936,71 +3008,71 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1324</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>404</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>2353</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>2353</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>2353</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="121">
@@ -3011,11 +3083,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="122">
@@ -3026,11 +3098,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="123">
@@ -3041,11 +3113,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="124">
@@ -3056,11 +3128,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="125">
@@ -3071,11 +3143,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="126">
@@ -3086,11 +3158,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="127">
@@ -3101,11 +3173,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="128">
@@ -3116,11 +3188,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="129">
@@ -3131,11 +3203,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="130">
@@ -3146,11 +3218,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="131">
@@ -3161,11 +3233,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="132">
@@ -3176,11 +3248,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="133">
@@ -3191,11 +3263,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="134">
@@ -3206,11 +3278,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="135">
@@ -3221,11 +3293,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="136">
@@ -3236,11 +3308,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="137">
@@ -3251,7 +3323,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -3266,7 +3338,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -3281,11 +3353,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="140">
@@ -3296,11 +3368,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="141">
@@ -3311,11 +3383,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1679</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="142">
@@ -3326,11 +3398,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2182</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="143">
@@ -3341,11 +3413,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1675</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="144">
@@ -3356,11 +3428,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1674</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="145">
@@ -3371,11 +3443,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1670</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="146">
@@ -3386,146 +3458,146 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>1664</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2848</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2842</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>2831</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>410</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2391</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2391</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2391</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2391</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2389</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="156">
@@ -3536,11 +3608,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="157">
@@ -3551,11 +3623,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="158">
@@ -3566,11 +3638,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="159">
@@ -3581,11 +3653,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="160">
@@ -3596,11 +3668,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>1660</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="161">
@@ -3611,11 +3683,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>1652</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="162">
@@ -3626,11 +3698,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>1655</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="163">
@@ -3641,11 +3713,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2411</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="164">
@@ -3656,11 +3728,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2404</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="165">
@@ -3671,11 +3743,11 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2416</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="166">
@@ -3686,11 +3758,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2405</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="167">
@@ -3701,11 +3773,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="168">
@@ -3716,11 +3788,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2406</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="169">
@@ -3731,11 +3803,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2406</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="170">
@@ -3746,11 +3818,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="171">
@@ -3761,11 +3833,11 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1652</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="172">
@@ -3776,11 +3848,11 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>2404</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="173">
@@ -3791,11 +3863,11 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>2422</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="174">
@@ -3806,11 +3878,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>2415</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="175">
@@ -3821,11 +3893,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1655</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="176">
@@ -3836,7 +3908,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -3851,11 +3923,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>1651</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="178">
@@ -3866,11 +3938,11 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>1648</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="179">
@@ -3881,131 +3953,131 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1558</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>2704</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>2718</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>2705</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>2705</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>2706</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>2706</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2706</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>2706</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="188">
@@ -4016,7 +4088,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -4031,11 +4103,11 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>2887</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="190">
@@ -4046,11 +4118,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>2879</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="191">
@@ -4061,11 +4133,11 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>2877</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="192">
@@ -4076,11 +4148,11 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="193">
@@ -4091,11 +4163,11 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="194">
@@ -4106,11 +4178,146 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
+          <t>31/05/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C194" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>31/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C195" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>31/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C196" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>01/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C197" t="n">
+        <v>2887</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>01/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C198" t="n">
+        <v>2879</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>01/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C199" t="n">
+        <v>2877</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>02/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C200" t="n">
+        <v>2843</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>02/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C201" t="n">
+        <v>2835</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
           <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C194" t="n">
+      <c r="C202" t="n">
         <v>2940</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>2983</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-06-03 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1344</v>
+        <v>1342</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1688</v>
+        <v>1686</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>1692</v>
+        <v>1690</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -574,7 +574,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1849</v>
+        <v>1847</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -608,7 +608,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2428</v>
+        <v>2425</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -661,7 +661,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2788</v>
+        <v>2785</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -676,7 +676,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -686,27 +686,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>HEL</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>AMS</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
       <c r="D8" t="n">
-        <v>2872</v>
+        <v>2875</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>KLM + Air Baltic</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>7.8</v>
+        <v>11.5</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -716,31 +720,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AMS</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Amsterdam</t>
-        </is>
-      </c>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
       <c r="D9" t="n">
-        <v>2879</v>
+        <v>2979</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>KLM + Air Baltic</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="G9" t="n">
         <v>2</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -750,27 +750,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>2983</v>
+        <v>4547</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>11.4</v>
+        <v>7.8</v>
       </c>
       <c r="G10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1344</v>
+        <v>1342</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -902,7 +902,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1688</v>
+        <v>1686</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -944,7 +944,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1692</v>
+        <v>1690</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1849</v>
+        <v>1847</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2428</v>
+        <v>2425</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2788</v>
+        <v>2785</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1139,22 +1139,22 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2872</v>
+        <v>2875</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>KLM + Air Baltic</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>7.8</v>
+        <v>11.5</v>
       </c>
       <c r="I8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AMS</t>
+          <t>ZRH</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1181,22 +1181,22 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>2879</v>
+        <v>2979</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>KLM + Air Baltic</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="I9" t="n">
         <v>2</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1213,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1223,22 +1223,22 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>2983</v>
+        <v>4547</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>11.4</v>
+        <v>7.8</v>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C203"/>
+  <dimension ref="A1:C212"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1758,16 +1758,16 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>371</v>
+        <v>2875</v>
       </c>
     </row>
     <row r="34">
@@ -1778,11 +1778,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="35">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1838,11 +1838,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="39">
@@ -1853,11 +1853,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="40">
@@ -1868,11 +1868,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="41">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="42">
@@ -1898,11 +1898,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="43">
@@ -1913,11 +1913,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="44">
@@ -1928,11 +1928,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="45">
@@ -1943,11 +1943,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="46">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="47">
@@ -1973,11 +1973,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="48">
@@ -1988,11 +1988,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="49">
@@ -2003,11 +2003,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="50">
@@ -2018,11 +2018,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="51">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="52">
@@ -2048,11 +2048,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="53">
@@ -2063,11 +2063,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="54">
@@ -2078,11 +2078,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="55">
@@ -2093,11 +2093,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2360</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="56">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2759</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="57">
@@ -2123,11 +2123,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2749</v>
+        <v>2759</v>
       </c>
     </row>
     <row r="58">
@@ -2138,41 +2138,41 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2788</v>
+        <v>2749</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>286</v>
+        <v>2788</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>1649</v>
+        <v>2785</v>
       </c>
     </row>
     <row r="61">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="62">
@@ -2198,7 +2198,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -2228,11 +2228,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="65">
@@ -2243,11 +2243,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="66">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="67">
@@ -2273,11 +2273,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="68">
@@ -2288,11 +2288,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="69">
@@ -2303,11 +2303,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="70">
@@ -2318,11 +2318,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="71">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="72">
@@ -2348,11 +2348,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="73">
@@ -2363,11 +2363,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="74">
@@ -2378,11 +2378,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="75">
@@ -2393,11 +2393,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2575</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="76">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="77">
@@ -2423,11 +2423,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="78">
@@ -2438,11 +2438,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="79">
@@ -2453,11 +2453,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2575</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="80">
@@ -2468,11 +2468,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="81">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="82">
@@ -2498,11 +2498,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2580</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="83">
@@ -2513,11 +2513,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2573</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="84">
@@ -2528,11 +2528,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2571</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="85">
@@ -2543,11 +2543,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2566</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="86">
@@ -2558,11 +2558,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2553</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="87">
@@ -2573,11 +2573,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2559</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="88">
@@ -2588,11 +2588,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2550</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="89">
@@ -2603,56 +2603,56 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>1849</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>228</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1329</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1329</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="93">
@@ -2663,11 +2663,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="94">
@@ -2678,7 +2678,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
@@ -2693,7 +2693,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="97">
@@ -2723,11 +2723,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="98">
@@ -2738,11 +2738,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="99">
@@ -2753,11 +2753,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="100">
@@ -2768,11 +2768,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="101">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="102">
@@ -2798,11 +2798,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="103">
@@ -2813,11 +2813,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="104">
@@ -2828,7 +2828,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -2843,11 +2843,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="106">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1338</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="107">
@@ -2873,11 +2873,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="108">
@@ -2888,11 +2888,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="109">
@@ -2903,7 +2903,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -2918,7 +2918,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -2948,11 +2948,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="113">
@@ -2963,11 +2963,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="114">
@@ -2978,11 +2978,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1336</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="115">
@@ -2993,11 +2993,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="116">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1333</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="117">
@@ -3023,11 +3023,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1332</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="118">
@@ -3038,11 +3038,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1329</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="119">
@@ -3053,11 +3053,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1324</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="120">
@@ -3068,71 +3068,71 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1344</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>404</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>2353</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>2353</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>2353</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="125">
@@ -3143,11 +3143,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="126">
@@ -3158,11 +3158,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="127">
@@ -3173,11 +3173,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="128">
@@ -3188,11 +3188,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="129">
@@ -3203,11 +3203,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="130">
@@ -3218,11 +3218,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="131">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="132">
@@ -3248,11 +3248,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="133">
@@ -3263,11 +3263,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="134">
@@ -3278,11 +3278,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="135">
@@ -3293,11 +3293,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="136">
@@ -3308,11 +3308,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="137">
@@ -3323,11 +3323,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="138">
@@ -3338,11 +3338,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="139">
@@ -3353,11 +3353,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="140">
@@ -3368,11 +3368,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="141">
@@ -3383,7 +3383,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
@@ -3398,7 +3398,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
@@ -3413,11 +3413,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="144">
@@ -3428,11 +3428,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="145">
@@ -3443,11 +3443,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1679</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="146">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2182</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="147">
@@ -3473,11 +3473,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>1675</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="148">
@@ -3488,11 +3488,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>1674</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="149">
@@ -3503,11 +3503,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>1670</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="150">
@@ -3518,11 +3518,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>1664</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="151">
@@ -3533,17 +3533,17 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>1688</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -3552,13 +3552,13 @@
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2848</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -3567,13 +3567,13 @@
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2842</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -3582,13 +3582,13 @@
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2831</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -3597,97 +3597,97 @@
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2872</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>410</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2391</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2391</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2391</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2391</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2389</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="162">
@@ -3698,11 +3698,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="163">
@@ -3713,11 +3713,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="164">
@@ -3728,11 +3728,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="165">
@@ -3743,11 +3743,11 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="166">
@@ -3758,11 +3758,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>1660</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="167">
@@ -3773,11 +3773,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1652</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="168">
@@ -3788,11 +3788,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>1655</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="169">
@@ -3803,11 +3803,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2411</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="170">
@@ -3818,11 +3818,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2404</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="171">
@@ -3833,11 +3833,11 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>2416</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="172">
@@ -3848,11 +3848,11 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>2405</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="173">
@@ -3863,11 +3863,11 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="174">
@@ -3878,11 +3878,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>2406</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="175">
@@ -3893,11 +3893,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>2406</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="176">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="177">
@@ -3923,11 +3923,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>1652</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="178">
@@ -3938,11 +3938,11 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>2404</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="179">
@@ -3953,11 +3953,11 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>2422</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="180">
@@ -3968,11 +3968,11 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>2415</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="181">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>1655</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="182">
@@ -3998,7 +3998,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -4013,11 +4013,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>1651</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="184">
@@ -4028,11 +4028,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1648</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="185">
@@ -4043,11 +4043,11 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1558</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="186">
@@ -4058,146 +4058,146 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2428</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1692</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>2704</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>2718</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>2705</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>2705</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>2706</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>2706</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>2706</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>2706</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="196">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
@@ -4223,11 +4223,11 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>2887</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="198">
@@ -4238,11 +4238,11 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>2879</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="199">
@@ -4253,11 +4253,11 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>2877</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="200">
@@ -4268,11 +4268,11 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="201">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="202">
@@ -4298,11 +4298,11 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>2940</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="203">
@@ -4313,11 +4313,146 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
+          <t>31/05/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C203" t="n">
+        <v>2706</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>31/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C204" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>01/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C205" t="n">
+        <v>2887</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>01/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C206" t="n">
+        <v>2879</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>01/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C207" t="n">
+        <v>2877</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>02/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C208" t="n">
+        <v>2843</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>02/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C209" t="n">
+        <v>2835</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C210" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
           <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
-      <c r="C203" t="n">
+      <c r="C211" t="n">
         <v>2983</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>2979</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-06-04 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1342</v>
+        <v>1346</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1686</v>
+        <v>1691</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -559,7 +559,7 @@
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>1690</v>
+        <v>1695</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -574,7 +574,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1847</v>
+        <v>1852</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -608,7 +608,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2425</v>
+        <v>2432</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -652,31 +652,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ARN</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>Stockholm</t>
-        </is>
-      </c>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2785</v>
+        <v>2781</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>15.4</v>
+        <v>11.4</v>
       </c>
       <c r="G7" t="n">
         <v>2</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -686,31 +682,31 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>AMS</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Stockholm</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2875</v>
+        <v>2793</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>KLM + Air Baltic</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>11.5</v>
+        <v>15.4</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -720,27 +716,31 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>ZRH</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
+          <t>AMS</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
       <c r="D9" t="n">
-        <v>2979</v>
+        <v>2884</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>KLM + Air Baltic</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="G9" t="n">
         <v>2</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>4547</v>
+        <v>4561</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -770,7 +770,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1342</v>
+        <v>1346</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -902,7 +902,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1686</v>
+        <v>1691</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -944,7 +944,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1690</v>
+        <v>1695</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1013,7 +1013,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1847</v>
+        <v>1852</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2425</v>
+        <v>2432</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>ZRH</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1097,22 +1097,22 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2785</v>
+        <v>2781</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>15.4</v>
+        <v>11.4</v>
       </c>
       <c r="I7" t="n">
         <v>2</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1129,7 +1129,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>AMS</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1139,22 +1139,22 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2875</v>
+        <v>2793</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>KLM + Air Baltic</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>11.5</v>
+        <v>15.4</v>
       </c>
       <c r="I8" t="n">
         <v>2</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1171,7 +1171,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1181,22 +1181,22 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>2979</v>
+        <v>2884</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>KLM + Air Baltic</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>11.4</v>
+        <v>11.5</v>
       </c>
       <c r="I9" t="n">
         <v>2</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>4547</v>
+        <v>4561</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C212"/>
+  <dimension ref="A1:C221"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1773,16 +1773,16 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>371</v>
+        <v>2884</v>
       </c>
     </row>
     <row r="35">
@@ -1793,11 +1793,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="36">
@@ -1808,7 +1808,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -1853,11 +1853,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="40">
@@ -1868,11 +1868,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="41">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="42">
@@ -1898,11 +1898,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="43">
@@ -1913,11 +1913,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="44">
@@ -1928,11 +1928,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="45">
@@ -1943,11 +1943,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="46">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="47">
@@ -1973,11 +1973,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="48">
@@ -1988,11 +1988,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="49">
@@ -2003,11 +2003,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="50">
@@ -2018,11 +2018,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="51">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="52">
@@ -2048,11 +2048,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="53">
@@ -2063,11 +2063,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="54">
@@ -2078,11 +2078,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="55">
@@ -2093,11 +2093,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="56">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2360</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="57">
@@ -2123,11 +2123,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2759</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="58">
@@ -2138,11 +2138,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2749</v>
+        <v>2759</v>
       </c>
     </row>
     <row r="59">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2788</v>
+        <v>2749</v>
       </c>
     </row>
     <row r="60">
@@ -2168,41 +2168,41 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2785</v>
+        <v>2788</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>286</v>
+        <v>2785</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>1649</v>
+        <v>2793</v>
       </c>
     </row>
     <row r="63">
@@ -2213,11 +2213,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="64">
@@ -2228,7 +2228,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -2243,7 +2243,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -2258,11 +2258,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="67">
@@ -2273,11 +2273,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="68">
@@ -2288,11 +2288,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="69">
@@ -2303,11 +2303,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="70">
@@ -2318,11 +2318,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="71">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="72">
@@ -2348,11 +2348,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="73">
@@ -2363,11 +2363,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="74">
@@ -2378,11 +2378,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="75">
@@ -2393,11 +2393,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="76">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="77">
@@ -2423,11 +2423,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2575</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="78">
@@ -2438,11 +2438,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="79">
@@ -2453,11 +2453,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="80">
@@ -2468,11 +2468,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="81">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2575</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="82">
@@ -2498,11 +2498,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="83">
@@ -2513,11 +2513,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="84">
@@ -2528,11 +2528,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2580</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="85">
@@ -2543,11 +2543,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2573</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="86">
@@ -2558,11 +2558,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2571</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="87">
@@ -2573,11 +2573,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2566</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="88">
@@ -2588,11 +2588,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2553</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="89">
@@ -2603,11 +2603,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2559</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="90">
@@ -2618,11 +2618,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2550</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="91">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>1849</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="92">
@@ -2648,56 +2648,56 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>1847</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>228</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1329</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1329</v>
+        <v>1852</v>
       </c>
     </row>
     <row r="96">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="97">
@@ -2723,7 +2723,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
@@ -2738,7 +2738,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
@@ -2753,11 +2753,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="100">
@@ -2768,11 +2768,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="101">
@@ -2783,11 +2783,11 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="102">
@@ -2798,11 +2798,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="103">
@@ -2813,11 +2813,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="104">
@@ -2828,11 +2828,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="105">
@@ -2843,11 +2843,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="106">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="107">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -2888,11 +2888,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="109">
@@ -2903,11 +2903,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1338</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="110">
@@ -2918,11 +2918,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="111">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="112">
@@ -2948,7 +2948,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -2978,7 +2978,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -2993,11 +2993,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="116">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="117">
@@ -3023,11 +3023,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1336</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="118">
@@ -3038,11 +3038,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="119">
@@ -3053,11 +3053,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1333</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="120">
@@ -3068,11 +3068,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1332</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="121">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1329</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="122">
@@ -3098,11 +3098,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1324</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="123">
@@ -3113,11 +3113,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1344</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="124">
@@ -3128,71 +3128,71 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1342</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>404</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>2353</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>2353</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>2353</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="129">
@@ -3203,11 +3203,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="130">
@@ -3218,11 +3218,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="131">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="132">
@@ -3248,11 +3248,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="133">
@@ -3263,11 +3263,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="134">
@@ -3278,11 +3278,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="135">
@@ -3293,11 +3293,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="136">
@@ -3308,11 +3308,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="137">
@@ -3323,11 +3323,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="138">
@@ -3338,11 +3338,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="139">
@@ -3353,11 +3353,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="140">
@@ -3368,11 +3368,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="141">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="142">
@@ -3398,11 +3398,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="143">
@@ -3413,11 +3413,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="144">
@@ -3428,11 +3428,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="145">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -3458,7 +3458,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -3473,11 +3473,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="148">
@@ -3488,11 +3488,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="149">
@@ -3503,11 +3503,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>1679</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="150">
@@ -3518,11 +3518,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2182</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="151">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>1675</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="152">
@@ -3548,11 +3548,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>1674</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="153">
@@ -3563,11 +3563,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>1670</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="154">
@@ -3578,11 +3578,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>1664</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="155">
@@ -3593,11 +3593,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>1688</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="156">
@@ -3608,176 +3608,176 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>1686</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2848</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2842</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2831</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2872</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>4547</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>410</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2391</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2391</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2391</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2391</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2389</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="168">
@@ -3788,11 +3788,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="169">
@@ -3803,11 +3803,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="170">
@@ -3818,11 +3818,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="171">
@@ -3833,11 +3833,11 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="172">
@@ -3848,11 +3848,11 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1660</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="173">
@@ -3863,11 +3863,11 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>1652</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="174">
@@ -3878,11 +3878,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>1655</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="175">
@@ -3893,11 +3893,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>2411</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="176">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>2404</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="177">
@@ -3923,11 +3923,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>2416</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="178">
@@ -3938,11 +3938,11 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>2405</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="179">
@@ -3953,11 +3953,11 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="180">
@@ -3968,11 +3968,11 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>2406</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="181">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>2406</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="182">
@@ -3998,11 +3998,11 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="183">
@@ -4013,11 +4013,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>1652</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="184">
@@ -4028,11 +4028,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>2404</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="185">
@@ -4043,11 +4043,11 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>2422</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="186">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2415</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="187">
@@ -4073,11 +4073,11 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1655</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="188">
@@ -4088,7 +4088,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
@@ -4103,11 +4103,11 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>1651</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="190">
@@ -4118,11 +4118,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1648</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="191">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1558</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="192">
@@ -4148,11 +4148,11 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>2428</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="193">
@@ -4163,161 +4163,161 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>2425</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1692</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1690</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>2704</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>2718</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>2705</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>2705</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>2706</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>2706</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>2706</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>2706</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="204">
@@ -4328,7 +4328,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
@@ -4343,11 +4343,11 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>2887</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="206">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>2879</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="207">
@@ -4373,11 +4373,11 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>2877</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="208">
@@ -4388,11 +4388,11 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="209">
@@ -4403,11 +4403,11 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="210">
@@ -4418,11 +4418,11 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>2940</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="211">
@@ -4433,11 +4433,11 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>2983</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="212">
@@ -4448,11 +4448,146 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
+          <t>31/05/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C212" t="n">
+        <v>2704</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>01/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C213" t="n">
+        <v>2887</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>01/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C214" t="n">
+        <v>2879</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>01/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C215" t="n">
+        <v>2877</v>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>02/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C216" t="n">
+        <v>2843</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>02/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C217" t="n">
+        <v>2835</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C218" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C219" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
           <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
-      <c r="C212" t="n">
+      <c r="C220" t="n">
         <v>2979</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>2781</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-06-04 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1346</v>
+        <v>1345</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -520,31 +520,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>London Heathrow</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1691</v>
+        <v>1581</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>15.5</v>
+        <v>26.2</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -554,27 +554,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MUC</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Frankfurt</t>
+        </is>
+      </c>
       <c r="D4" t="n">
-        <v>1695</v>
+        <v>1689</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Lufthansa</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>13.8</v>
+        <v>15.5</v>
       </c>
       <c r="G4" t="n">
         <v>2</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -584,27 +588,23 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CPH</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Copenhagen</t>
-        </is>
-      </c>
+          <t>MUC</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
-        <v>1852</v>
+        <v>1695</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>15.6</v>
+        <v>13.8</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -618,31 +618,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>London Heathrow</t>
+          <t>Copenhagen</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2432</v>
+        <v>1850</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>14.2</v>
+        <v>15.6</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2781</v>
+        <v>2778</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -672,7 +672,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2793</v>
+        <v>2790</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -706,7 +706,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2884</v>
+        <v>2881</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -740,7 +740,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>4561</v>
+        <v>4557</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -770,7 +770,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1346</v>
+        <v>1345</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -902,7 +902,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -919,7 +919,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -929,22 +929,22 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1691</v>
+        <v>1581</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>15.5</v>
+        <v>26.2</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -961,7 +961,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -971,22 +971,22 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1695</v>
+        <v>1689</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Lufthansa</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>13.8</v>
+        <v>15.5</v>
       </c>
       <c r="I4" t="n">
         <v>2</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1003,7 +1003,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1013,18 +1013,18 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1852</v>
+        <v>1695</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>15.6</v>
+        <v>13.8</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1055,22 +1055,22 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2432</v>
+        <v>1850</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>14.2</v>
+        <v>15.6</v>
       </c>
       <c r="I6" t="n">
         <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2781</v>
+        <v>2778</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2793</v>
+        <v>2790</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>2884</v>
+        <v>2881</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>4561</v>
+        <v>4557</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C221"/>
+  <dimension ref="A1:C229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1788,16 +1788,16 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>371</v>
+        <v>2881</v>
       </c>
     </row>
     <row r="36">
@@ -1808,11 +1808,11 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="37">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -1853,7 +1853,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -1868,11 +1868,11 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="41">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="42">
@@ -1898,11 +1898,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="43">
@@ -1913,11 +1913,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="44">
@@ -1928,11 +1928,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="45">
@@ -1943,11 +1943,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="46">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="47">
@@ -1973,11 +1973,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="48">
@@ -1988,11 +1988,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="49">
@@ -2003,11 +2003,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="50">
@@ -2018,11 +2018,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="51">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="52">
@@ -2048,11 +2048,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="53">
@@ -2063,11 +2063,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="54">
@@ -2078,11 +2078,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="55">
@@ -2093,11 +2093,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="56">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="57">
@@ -2123,11 +2123,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2360</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="58">
@@ -2138,11 +2138,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2759</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="59">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2749</v>
+        <v>2759</v>
       </c>
     </row>
     <row r="60">
@@ -2168,11 +2168,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2788</v>
+        <v>2749</v>
       </c>
     </row>
     <row r="61">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2785</v>
+        <v>2788</v>
       </c>
     </row>
     <row r="62">
@@ -2198,41 +2198,41 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2793</v>
+        <v>2785</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>286</v>
+        <v>2793</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>1649</v>
+        <v>2790</v>
       </c>
     </row>
     <row r="65">
@@ -2243,11 +2243,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="66">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
@@ -2288,11 +2288,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="69">
@@ -2303,11 +2303,11 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="70">
@@ -2318,11 +2318,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="71">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="72">
@@ -2348,11 +2348,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="73">
@@ -2363,11 +2363,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="74">
@@ -2378,11 +2378,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="75">
@@ -2393,11 +2393,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="76">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="77">
@@ -2423,11 +2423,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="78">
@@ -2438,11 +2438,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="79">
@@ -2453,11 +2453,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2575</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="80">
@@ -2468,11 +2468,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="81">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="82">
@@ -2498,11 +2498,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="83">
@@ -2513,11 +2513,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2575</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="84">
@@ -2528,11 +2528,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="85">
@@ -2543,11 +2543,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="86">
@@ -2558,11 +2558,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2580</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="87">
@@ -2573,11 +2573,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2573</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="88">
@@ -2588,11 +2588,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2571</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="89">
@@ -2603,11 +2603,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2566</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="90">
@@ -2618,11 +2618,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2553</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="91">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>2559</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="92">
@@ -2648,11 +2648,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>2550</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="93">
@@ -2663,11 +2663,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>1849</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="94">
@@ -2678,11 +2678,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>1847</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="95">
@@ -2693,56 +2693,56 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1852</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>228</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1329</v>
+        <v>1852</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1329</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="99">
@@ -2753,11 +2753,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="100">
@@ -2768,7 +2768,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
@@ -2783,7 +2783,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
@@ -2798,11 +2798,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="103">
@@ -2813,11 +2813,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="104">
@@ -2828,11 +2828,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="105">
@@ -2843,11 +2843,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="106">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="107">
@@ -2873,11 +2873,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="108">
@@ -2888,11 +2888,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="109">
@@ -2903,11 +2903,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="110">
@@ -2918,7 +2918,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="112">
@@ -2948,11 +2948,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1338</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="113">
@@ -2963,11 +2963,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="114">
@@ -2978,11 +2978,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="115">
@@ -2993,7 +2993,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -3008,7 +3008,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -3023,7 +3023,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -3038,11 +3038,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="119">
@@ -3053,11 +3053,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="120">
@@ -3068,11 +3068,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1336</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="121">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="122">
@@ -3098,11 +3098,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1333</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="123">
@@ -3113,11 +3113,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1332</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="124">
@@ -3128,11 +3128,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1329</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="125">
@@ -3143,11 +3143,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1324</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="126">
@@ -3158,11 +3158,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1344</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="127">
@@ -3173,11 +3173,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1342</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="128">
@@ -3188,71 +3188,71 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1346</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>404</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>2353</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>2353</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>2353</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="133">
@@ -3263,11 +3263,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="134">
@@ -3278,11 +3278,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="135">
@@ -3293,11 +3293,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="136">
@@ -3308,11 +3308,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="137">
@@ -3323,11 +3323,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="138">
@@ -3338,11 +3338,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="139">
@@ -3353,11 +3353,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="140">
@@ -3368,11 +3368,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="141">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="142">
@@ -3398,11 +3398,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="143">
@@ -3413,11 +3413,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="144">
@@ -3428,11 +3428,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="145">
@@ -3443,11 +3443,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="146">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="147">
@@ -3473,11 +3473,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="148">
@@ -3488,11 +3488,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="149">
@@ -3503,7 +3503,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -3518,7 +3518,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="152">
@@ -3548,11 +3548,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="153">
@@ -3563,11 +3563,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>1679</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="154">
@@ -3578,11 +3578,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2182</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="155">
@@ -3593,11 +3593,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>1675</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="156">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>1674</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="157">
@@ -3623,11 +3623,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>1670</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="158">
@@ -3638,11 +3638,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>1664</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="159">
@@ -3653,11 +3653,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>1688</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="160">
@@ -3668,11 +3668,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>1686</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="161">
@@ -3683,86 +3683,86 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>1691</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2848</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2842</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2831</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2872</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>4547</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="167">
@@ -3773,101 +3773,101 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>4561</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>410</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2391</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2391</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>2391</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>2391</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>2389</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="174">
@@ -3878,11 +3878,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>2402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="175">
@@ -3893,11 +3893,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="176">
@@ -3908,11 +3908,11 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="177">
@@ -3923,11 +3923,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="178">
@@ -3938,11 +3938,11 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>1660</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="179">
@@ -3953,11 +3953,11 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1652</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="180">
@@ -3968,11 +3968,11 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>1655</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="181">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>2411</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="182">
@@ -3998,11 +3998,11 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>2404</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="183">
@@ -4013,11 +4013,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>2416</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="184">
@@ -4028,11 +4028,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>2405</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="185">
@@ -4043,11 +4043,11 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="186">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2406</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="187">
@@ -4073,11 +4073,11 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>2406</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="188">
@@ -4088,11 +4088,11 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="189">
@@ -4103,11 +4103,11 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>1652</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="190">
@@ -4118,11 +4118,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>2404</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="191">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>2422</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="192">
@@ -4148,11 +4148,11 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>2415</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="193">
@@ -4163,11 +4163,11 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1655</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="194">
@@ -4178,7 +4178,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
@@ -4193,11 +4193,11 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1651</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="196">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>1648</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="197">
@@ -4223,11 +4223,11 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>1558</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="198">
@@ -4238,11 +4238,11 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>2428</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="199">
@@ -4253,11 +4253,11 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>2425</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="200">
@@ -4268,161 +4268,161 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>2432</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>1692</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>1690</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>1695</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>2704</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>2718</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>2705</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>2705</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2706</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>2706</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>2706</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="211">
@@ -4433,11 +4433,11 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="212">
@@ -4448,11 +4448,11 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>2704</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="213">
@@ -4463,11 +4463,11 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="214">
@@ -4478,11 +4478,11 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>2879</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="215">
@@ -4493,11 +4493,11 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="216">
@@ -4508,11 +4508,11 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="217">
@@ -4523,11 +4523,11 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="218">
@@ -4538,11 +4538,11 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>2940</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="219">
@@ -4553,11 +4553,11 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>2983</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="220">
@@ -4568,11 +4568,11 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>2979</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="221">
@@ -4583,11 +4583,131 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
+          <t>01/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C221" t="n">
+        <v>2879</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>01/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C222" t="n">
+        <v>2877</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>02/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C223" t="n">
+        <v>2843</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>02/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C224" t="n">
+        <v>2835</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C225" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C226" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C227" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
           <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C221" t="n">
+      <c r="C228" t="n">
         <v>2781</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>04/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>2778</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-06-04 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1581</v>
+        <v>1574</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1689</v>
+        <v>1682</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1850</v>
+        <v>1842</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2778</v>
+        <v>2766</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -672,7 +672,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2790</v>
+        <v>2778</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -706,7 +706,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2881</v>
+        <v>2868</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -740,7 +740,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>4557</v>
+        <v>4537</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -770,7 +770,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -887,7 +887,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1345</v>
+        <v>1339</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -902,7 +902,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1581</v>
+        <v>1574</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -944,7 +944,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -971,7 +971,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1689</v>
+        <v>1682</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -986,7 +986,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>1850</v>
+        <v>1842</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1097,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2778</v>
+        <v>2766</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1112,7 +1112,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1139,7 +1139,7 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2790</v>
+        <v>2778</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1154,7 +1154,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1181,7 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>2881</v>
+        <v>2868</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1196,7 +1196,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1223,7 +1223,7 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>4557</v>
+        <v>4537</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1238,7 +1238,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C229"/>
+  <dimension ref="A1:C237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1803,16 +1803,16 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>371</v>
+        <v>2868</v>
       </c>
     </row>
     <row r="37">
@@ -1823,11 +1823,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="38">
@@ -1838,7 +1838,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
@@ -1868,7 +1868,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1883,11 +1883,11 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="42">
@@ -1898,11 +1898,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="43">
@@ -1913,11 +1913,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="44">
@@ -1928,11 +1928,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="45">
@@ -1943,11 +1943,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="46">
@@ -1958,11 +1958,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="47">
@@ -1973,11 +1973,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="48">
@@ -1988,11 +1988,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="49">
@@ -2003,11 +2003,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="50">
@@ -2018,11 +2018,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="51">
@@ -2033,11 +2033,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="52">
@@ -2048,11 +2048,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="53">
@@ -2063,11 +2063,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="54">
@@ -2078,11 +2078,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="55">
@@ -2093,11 +2093,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="56">
@@ -2108,11 +2108,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="57">
@@ -2123,11 +2123,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="58">
@@ -2138,11 +2138,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2360</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="59">
@@ -2153,11 +2153,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2759</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="60">
@@ -2168,11 +2168,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2749</v>
+        <v>2759</v>
       </c>
     </row>
     <row r="61">
@@ -2183,11 +2183,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2788</v>
+        <v>2749</v>
       </c>
     </row>
     <row r="62">
@@ -2198,11 +2198,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2785</v>
+        <v>2788</v>
       </c>
     </row>
     <row r="63">
@@ -2213,11 +2213,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2793</v>
+        <v>2785</v>
       </c>
     </row>
     <row r="64">
@@ -2228,41 +2228,41 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2790</v>
+        <v>2793</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>286</v>
+        <v>2790</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>1649</v>
+        <v>2778</v>
       </c>
     </row>
     <row r="67">
@@ -2273,11 +2273,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="68">
@@ -2288,7 +2288,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
@@ -2303,7 +2303,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -2318,11 +2318,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="71">
@@ -2333,11 +2333,11 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>1674</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="72">
@@ -2348,11 +2348,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1658</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="73">
@@ -2363,11 +2363,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1654</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="74">
@@ -2378,11 +2378,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1668</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="75">
@@ -2393,11 +2393,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1667</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="76">
@@ -2408,11 +2408,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1658</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="77">
@@ -2423,11 +2423,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1661</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="78">
@@ -2438,11 +2438,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1663</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="79">
@@ -2453,11 +2453,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>2398</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="80">
@@ -2468,11 +2468,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>2410</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="81">
@@ -2483,11 +2483,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2575</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="82">
@@ -2498,11 +2498,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="83">
@@ -2513,11 +2513,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="84">
@@ -2528,11 +2528,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>2329</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="85">
@@ -2543,11 +2543,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2575</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="86">
@@ -2558,11 +2558,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="87">
@@ -2573,11 +2573,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="88">
@@ -2588,11 +2588,11 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>2580</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="89">
@@ -2603,11 +2603,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2573</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="90">
@@ -2618,11 +2618,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2571</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="91">
@@ -2633,11 +2633,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>2566</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="92">
@@ -2648,11 +2648,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>2553</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="93">
@@ -2663,11 +2663,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2559</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="94">
@@ -2678,11 +2678,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>2550</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="95">
@@ -2693,11 +2693,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>1849</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="96">
@@ -2708,11 +2708,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>1847</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="97">
@@ -2723,11 +2723,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1852</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="98">
@@ -2738,56 +2738,56 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1850</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>228</v>
+        <v>1852</v>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1329</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>1329</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="102">
@@ -2798,11 +2798,11 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="103">
@@ -2813,7 +2813,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
@@ -2828,7 +2828,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
@@ -2843,11 +2843,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="106">
@@ -2858,11 +2858,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="107">
@@ -2873,11 +2873,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1334</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="108">
@@ -2888,11 +2888,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1345</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="109">
@@ -2903,11 +2903,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="110">
@@ -2918,11 +2918,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1337</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="111">
@@ -2933,11 +2933,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1340</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="112">
@@ -2948,11 +2948,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1341</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="113">
@@ -2963,7 +2963,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -2978,11 +2978,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1344</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="115">
@@ -2993,11 +2993,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1338</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="116">
@@ -3008,11 +3008,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="117">
@@ -3023,11 +3023,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="118">
@@ -3038,7 +3038,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -3053,7 +3053,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -3068,7 +3068,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -3083,11 +3083,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="122">
@@ -3098,11 +3098,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="123">
@@ -3113,11 +3113,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1336</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="124">
@@ -3128,11 +3128,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="125">
@@ -3143,11 +3143,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1333</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="126">
@@ -3158,11 +3158,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1332</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="127">
@@ -3173,11 +3173,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1329</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="128">
@@ -3188,11 +3188,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1324</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="129">
@@ -3203,11 +3203,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>1344</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="130">
@@ -3218,11 +3218,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1342</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="131">
@@ -3233,11 +3233,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1346</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="132">
@@ -3248,71 +3248,71 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1345</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>404</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>2353</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>2353</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>2353</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="137">
@@ -3323,11 +3323,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="138">
@@ -3338,11 +3338,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="139">
@@ -3353,11 +3353,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="140">
@@ -3368,11 +3368,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="141">
@@ -3383,11 +3383,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="142">
@@ -3398,11 +3398,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="143">
@@ -3413,11 +3413,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="144">
@@ -3428,11 +3428,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="145">
@@ -3443,11 +3443,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="146">
@@ -3458,11 +3458,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="147">
@@ -3473,11 +3473,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="148">
@@ -3488,11 +3488,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="149">
@@ -3503,11 +3503,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="150">
@@ -3518,11 +3518,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="151">
@@ -3533,11 +3533,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="152">
@@ -3548,11 +3548,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="153">
@@ -3563,7 +3563,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -3578,7 +3578,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -3593,11 +3593,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="156">
@@ -3608,11 +3608,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="157">
@@ -3623,11 +3623,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>1679</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="158">
@@ -3638,11 +3638,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2182</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="159">
@@ -3653,11 +3653,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>1675</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="160">
@@ -3668,11 +3668,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>1674</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="161">
@@ -3683,11 +3683,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>1670</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="162">
@@ -3698,11 +3698,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>1664</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="163">
@@ -3713,11 +3713,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>1688</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="164">
@@ -3728,11 +3728,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>1686</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="165">
@@ -3743,11 +3743,11 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>1691</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="166">
@@ -3758,86 +3758,86 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>1689</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2848</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2842</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2831</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2872</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>4547</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="172">
@@ -3848,11 +3848,11 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>4561</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="173">
@@ -3863,101 +3863,101 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>4557</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>410</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>2391</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>2391</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>2391</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>2391</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>2389</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="180">
@@ -3968,11 +3968,11 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>2402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="181">
@@ -3983,11 +3983,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="182">
@@ -3998,11 +3998,11 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="183">
@@ -4013,11 +4013,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="184">
@@ -4028,11 +4028,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1660</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="185">
@@ -4043,11 +4043,11 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1652</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="186">
@@ -4058,11 +4058,11 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>1655</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="187">
@@ -4073,11 +4073,11 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>2411</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="188">
@@ -4088,11 +4088,11 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>2404</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="189">
@@ -4103,11 +4103,11 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>2416</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="190">
@@ -4118,11 +4118,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>2405</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="191">
@@ -4133,11 +4133,11 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="192">
@@ -4148,11 +4148,11 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>2406</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="193">
@@ -4163,11 +4163,11 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>2406</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="194">
@@ -4178,11 +4178,11 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="195">
@@ -4193,11 +4193,11 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1652</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="196">
@@ -4208,11 +4208,11 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>2404</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="197">
@@ -4223,11 +4223,11 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>2422</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="198">
@@ -4238,11 +4238,11 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>2415</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="199">
@@ -4253,11 +4253,11 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>1655</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="200">
@@ -4268,7 +4268,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
@@ -4283,11 +4283,11 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>1651</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="202">
@@ -4298,11 +4298,11 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>1648</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="203">
@@ -4313,11 +4313,11 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>1558</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="204">
@@ -4328,11 +4328,11 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>2428</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="205">
@@ -4343,11 +4343,11 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>2425</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="206">
@@ -4358,11 +4358,11 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>2432</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="207">
@@ -4373,161 +4373,161 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>1581</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>1692</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>1690</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>1695</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>2704</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>2718</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>2705</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>2705</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>2706</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2706</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>2706</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="218">
@@ -4538,11 +4538,11 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="219">
@@ -4553,11 +4553,11 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>2704</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="220">
@@ -4568,11 +4568,11 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="221">
@@ -4583,11 +4583,11 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>2879</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="222">
@@ -4598,11 +4598,11 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="223">
@@ -4613,11 +4613,11 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="224">
@@ -4628,11 +4628,11 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="225">
@@ -4643,11 +4643,11 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>2940</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="226">
@@ -4658,11 +4658,11 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>2983</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="227">
@@ -4673,11 +4673,11 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>2979</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="228">
@@ -4688,11 +4688,11 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>2781</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="229">
@@ -4703,11 +4703,131 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
+          <t>01/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C229" t="n">
+        <v>2877</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>02/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C230" t="n">
+        <v>2843</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>02/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C231" t="n">
+        <v>2835</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C232" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C233" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C234" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C235" t="n">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
           <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
-      <c r="C229" t="n">
+      <c r="C236" t="n">
         <v>2778</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>04/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>2766</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-06-05 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -429,14 +429,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H10"/>
+  <dimension ref="A1:H11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="17" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="23" customWidth="1" min="5" max="5"/>
+    <col width="49" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="22" customWidth="1" min="8" max="8"/>
@@ -495,7 +495,7 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1339</v>
+        <v>1343</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -510,7 +510,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1574</v>
+        <v>1579</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1682</v>
+        <v>1687</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1842</v>
+        <v>1848</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -657,7 +657,7 @@
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2766</v>
+        <v>2774</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -672,7 +672,7 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2868</v>
+        <v>2877</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -740,7 +740,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -750,32 +750,62 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>4537</v>
+        <v>3471</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
+          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="G10" t="n">
+        <v>2</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>05/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>HEL</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>4550</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
           <t>Finnair</t>
         </is>
       </c>
-      <c r="F10" t="n">
+      <c r="F11" t="n">
         <v>7.8</v>
       </c>
-      <c r="G10" t="n">
+      <c r="G11" t="n">
         <v>1</v>
       </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>04/06/2026 20:19 BRT</t>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D10">
+  <conditionalFormatting sqref="D2:D11">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -797,7 +827,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -806,7 +836,7 @@
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
-    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="49" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
     <col width="10" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
@@ -887,7 +917,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1339</v>
+        <v>1343</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -902,7 +932,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -929,7 +959,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1574</v>
+        <v>1579</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -944,7 +974,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -971,7 +1001,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1682</v>
+        <v>1687</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -986,7 +1016,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1085,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>1842</v>
+        <v>1848</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1070,7 +1100,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1097,7 +1127,7 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2766</v>
+        <v>2774</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1112,7 +1142,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1181,7 +1211,7 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>2868</v>
+        <v>2877</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -1196,7 +1226,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1213,7 +1243,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1223,27 +1253,69 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>4537</v>
+        <v>3471</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
+          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
+        </is>
+      </c>
+      <c r="H10" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>05/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>DUB</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>KEF</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>HEL</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="n">
+        <v>4550</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
           <t>Finnair</t>
         </is>
       </c>
-      <c r="H10" t="n">
+      <c r="H11" t="n">
         <v>7.8</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I11" t="n">
         <v>1</v>
       </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>04/06/2026 20:19 BRT</t>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F2:F10">
+  <conditionalFormatting sqref="F2:F11">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1265,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C237"/>
+  <dimension ref="A1:C245"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1818,16 +1890,16 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>371</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="38">
@@ -1838,11 +1910,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>2162</v>
+        <v>371</v>
       </c>
     </row>
     <row r="39">
@@ -1853,7 +1925,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C39" t="n">
@@ -1883,7 +1955,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1898,11 +1970,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2161</v>
+        <v>2162</v>
       </c>
     </row>
     <row r="43">
@@ -1913,11 +1985,11 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2172</v>
+        <v>2161</v>
       </c>
     </row>
     <row r="44">
@@ -1928,11 +2000,11 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>2174</v>
+        <v>2172</v>
       </c>
     </row>
     <row r="45">
@@ -1943,11 +2015,11 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2170</v>
+        <v>2174</v>
       </c>
     </row>
     <row r="46">
@@ -1958,11 +2030,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2188</v>
+        <v>2170</v>
       </c>
     </row>
     <row r="47">
@@ -1973,11 +2045,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>2186</v>
+        <v>2188</v>
       </c>
     </row>
     <row r="48">
@@ -1988,11 +2060,11 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>2181</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="49">
@@ -2003,11 +2075,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>2185</v>
+        <v>2181</v>
       </c>
     </row>
     <row r="50">
@@ -2018,11 +2090,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2187</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="51">
@@ -2033,11 +2105,11 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2746</v>
+        <v>2187</v>
       </c>
     </row>
     <row r="52">
@@ -2048,11 +2120,11 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>2771</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="53">
@@ -2063,11 +2135,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>2758</v>
+        <v>2771</v>
       </c>
     </row>
     <row r="54">
@@ -2078,11 +2150,11 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>3175</v>
+        <v>2758</v>
       </c>
     </row>
     <row r="55">
@@ -2093,11 +2165,11 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>2358</v>
+        <v>3175</v>
       </c>
     </row>
     <row r="56">
@@ -2108,11 +2180,11 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>3176</v>
+        <v>2358</v>
       </c>
     </row>
     <row r="57">
@@ -2123,11 +2195,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2917</v>
+        <v>3176</v>
       </c>
     </row>
     <row r="58">
@@ -2138,11 +2210,11 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2915</v>
+        <v>2917</v>
       </c>
     </row>
     <row r="59">
@@ -2153,11 +2225,11 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>2360</v>
+        <v>2915</v>
       </c>
     </row>
     <row r="60">
@@ -2168,11 +2240,11 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>2759</v>
+        <v>2360</v>
       </c>
     </row>
     <row r="61">
@@ -2183,11 +2255,11 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>2749</v>
+        <v>2759</v>
       </c>
     </row>
     <row r="62">
@@ -2198,11 +2270,11 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2788</v>
+        <v>2749</v>
       </c>
     </row>
     <row r="63">
@@ -2213,11 +2285,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>2785</v>
+        <v>2788</v>
       </c>
     </row>
     <row r="64">
@@ -2228,11 +2300,11 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>2793</v>
+        <v>2785</v>
       </c>
     </row>
     <row r="65">
@@ -2243,11 +2315,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>2790</v>
+        <v>2793</v>
       </c>
     </row>
     <row r="66">
@@ -2258,26 +2330,26 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>2778</v>
+        <v>2790</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>286</v>
+        <v>2778</v>
       </c>
     </row>
     <row r="68">
@@ -2288,11 +2360,11 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>1649</v>
+        <v>286</v>
       </c>
     </row>
     <row r="69">
@@ -2303,7 +2375,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C69" t="n">
@@ -2333,7 +2405,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -2348,11 +2420,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>1648</v>
+        <v>1649</v>
       </c>
     </row>
     <row r="73">
@@ -2363,11 +2435,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>1674</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="74">
@@ -2378,11 +2450,11 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>1658</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="75">
@@ -2393,11 +2465,11 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>1654</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="76">
@@ -2408,11 +2480,11 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>1668</v>
+        <v>1654</v>
       </c>
     </row>
     <row r="77">
@@ -2423,11 +2495,11 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>1667</v>
+        <v>1668</v>
       </c>
     </row>
     <row r="78">
@@ -2438,11 +2510,11 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>1658</v>
+        <v>1667</v>
       </c>
     </row>
     <row r="79">
@@ -2453,11 +2525,11 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>1661</v>
+        <v>1658</v>
       </c>
     </row>
     <row r="80">
@@ -2468,11 +2540,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1663</v>
+        <v>1661</v>
       </c>
     </row>
     <row r="81">
@@ -2483,11 +2555,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>2398</v>
+        <v>1663</v>
       </c>
     </row>
     <row r="82">
@@ -2498,11 +2570,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2410</v>
+        <v>2398</v>
       </c>
     </row>
     <row r="83">
@@ -2513,11 +2585,11 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2575</v>
+        <v>2410</v>
       </c>
     </row>
     <row r="84">
@@ -2528,7 +2600,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C84" t="n">
@@ -2543,11 +2615,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="86">
@@ -2558,11 +2630,11 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>2329</v>
+        <v>2576</v>
       </c>
     </row>
     <row r="87">
@@ -2573,11 +2645,11 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>2575</v>
+        <v>2329</v>
       </c>
     </row>
     <row r="88">
@@ -2588,7 +2660,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C88" t="n">
@@ -2603,11 +2675,11 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>2574</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="90">
@@ -2618,11 +2690,11 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>2580</v>
+        <v>2574</v>
       </c>
     </row>
     <row r="91">
@@ -2633,11 +2705,11 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>2573</v>
+        <v>2580</v>
       </c>
     </row>
     <row r="92">
@@ -2648,11 +2720,11 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>2571</v>
+        <v>2573</v>
       </c>
     </row>
     <row r="93">
@@ -2663,11 +2735,11 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>2566</v>
+        <v>2571</v>
       </c>
     </row>
     <row r="94">
@@ -2678,11 +2750,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>2553</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="95">
@@ -2693,11 +2765,11 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>2559</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="96">
@@ -2708,11 +2780,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>2550</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="97">
@@ -2723,11 +2795,11 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>1849</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="98">
@@ -2738,11 +2810,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>1847</v>
+        <v>1849</v>
       </c>
     </row>
     <row r="99">
@@ -2753,11 +2825,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>1852</v>
+        <v>1847</v>
       </c>
     </row>
     <row r="100">
@@ -2768,11 +2840,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>1850</v>
+        <v>1852</v>
       </c>
     </row>
     <row r="101">
@@ -2783,41 +2855,41 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>1842</v>
+        <v>1850</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>228</v>
+        <v>1842</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>1329</v>
+        <v>1848</v>
       </c>
     </row>
     <row r="104">
@@ -2828,11 +2900,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="105">
@@ -2843,7 +2915,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
@@ -2858,7 +2930,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -2873,7 +2945,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -2888,11 +2960,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="109">
@@ -2903,11 +2975,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1337</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="110">
@@ -2918,11 +2990,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1334</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="111">
@@ -2933,11 +3005,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1345</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="112">
@@ -2948,11 +3020,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1344</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="113">
@@ -2963,11 +3035,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1337</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="114">
@@ -2978,11 +3050,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1340</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="115">
@@ -2993,11 +3065,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1341</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="116">
@@ -3008,11 +3080,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1337</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="117">
@@ -3023,11 +3095,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1344</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="118">
@@ -3038,11 +3110,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1338</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="119">
@@ -3053,11 +3125,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="120">
@@ -3068,7 +3140,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -3083,7 +3155,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -3098,7 +3170,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -3113,7 +3185,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -3128,11 +3200,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="125">
@@ -3143,11 +3215,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1340</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="126">
@@ -3158,11 +3230,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1336</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="127">
@@ -3173,11 +3245,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="128">
@@ -3188,11 +3260,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="129">
@@ -3203,11 +3275,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>1332</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="130">
@@ -3218,11 +3290,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1329</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="131">
@@ -3233,11 +3305,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1324</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="132">
@@ -3248,11 +3320,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1344</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="133">
@@ -3263,11 +3335,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1342</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="134">
@@ -3278,11 +3350,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1346</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="135">
@@ -3293,11 +3365,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1345</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="136">
@@ -3308,71 +3380,71 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1339</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>404</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>2353</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>2353</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>2353</v>
+        <v>3471</v>
       </c>
     </row>
     <row r="141">
@@ -3383,11 +3455,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="142">
@@ -3398,11 +3470,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="143">
@@ -3413,11 +3485,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="144">
@@ -3428,11 +3500,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>2367</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="145">
@@ -3443,11 +3515,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2238</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="146">
@@ -3458,11 +3530,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2257</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="147">
@@ -3473,11 +3545,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2196</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="148">
@@ -3488,11 +3560,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2185</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="149">
@@ -3503,11 +3575,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>2189</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="150">
@@ -3518,11 +3590,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2191</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="151">
@@ -3533,11 +3605,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2185</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="152">
@@ -3548,11 +3620,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2196</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="153">
@@ -3563,11 +3635,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2186</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="154">
@@ -3578,11 +3650,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2186</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="155">
@@ -3593,11 +3665,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="156">
@@ -3608,11 +3680,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="157">
@@ -3623,7 +3695,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -3638,7 +3710,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -3653,11 +3725,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="160">
@@ -3668,11 +3740,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="161">
@@ -3683,11 +3755,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>1679</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="162">
@@ -3698,11 +3770,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2182</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="163">
@@ -3713,11 +3785,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>1675</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="164">
@@ -3728,11 +3800,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>1674</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="165">
@@ -3743,11 +3815,11 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>1670</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="166">
@@ -3758,11 +3830,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>1664</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="167">
@@ -3773,11 +3845,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1688</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="168">
@@ -3788,11 +3860,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>1686</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="169">
@@ -3803,11 +3875,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1691</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="170">
@@ -3818,11 +3890,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>1689</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="171">
@@ -3833,86 +3905,86 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1682</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>2848</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>2842</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>2831</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>2872</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>4547</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="177">
@@ -3923,11 +3995,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>4561</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="178">
@@ -3938,11 +4010,11 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>4557</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="179">
@@ -3953,101 +4025,101 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>4537</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>410</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>2391</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>2391</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>2391</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>2391</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>2389</v>
+        <v>4550</v>
       </c>
     </row>
     <row r="186">
@@ -4058,11 +4130,11 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2402</v>
+        <v>410</v>
       </c>
     </row>
     <row r="187">
@@ -4073,11 +4145,11 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="188">
@@ -4088,11 +4160,11 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="189">
@@ -4103,11 +4175,11 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="190">
@@ -4118,11 +4190,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1660</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="191">
@@ -4133,11 +4205,11 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1652</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="192">
@@ -4148,11 +4220,11 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>1655</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="193">
@@ -4163,11 +4235,11 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>2411</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="194">
@@ -4178,11 +4250,11 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>2404</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="195">
@@ -4193,11 +4265,11 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>2416</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="196">
@@ -4208,11 +4280,11 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>2405</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="197">
@@ -4223,11 +4295,11 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="198">
@@ -4238,11 +4310,11 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>2406</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="199">
@@ -4253,11 +4325,11 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>2406</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="200">
@@ -4268,11 +4340,11 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="201">
@@ -4283,11 +4355,11 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>1652</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="202">
@@ -4298,11 +4370,11 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>2404</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="203">
@@ -4313,11 +4385,11 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>2422</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="204">
@@ -4328,11 +4400,11 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>2415</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="205">
@@ -4343,11 +4415,11 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>1655</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="206">
@@ -4358,7 +4430,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -4373,11 +4445,11 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>1651</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="208">
@@ -4388,11 +4460,11 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>1648</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="209">
@@ -4403,11 +4475,11 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>1558</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="210">
@@ -4418,11 +4490,11 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>2428</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="211">
@@ -4433,11 +4505,11 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>2425</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="212">
@@ -4448,11 +4520,11 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>2432</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="213">
@@ -4463,11 +4535,11 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>1581</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="214">
@@ -4478,161 +4550,161 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1574</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>1692</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>1690</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>1695</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>2704</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>2718</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>2705</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>2705</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>2706</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>2706</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>2706</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="225">
@@ -4643,11 +4715,11 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="226">
@@ -4658,11 +4730,11 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>2704</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="227">
@@ -4673,11 +4745,11 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="228">
@@ -4688,11 +4760,11 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>2879</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="229">
@@ -4703,11 +4775,11 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="230">
@@ -4718,11 +4790,11 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="231">
@@ -4733,11 +4805,11 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="232">
@@ -4748,11 +4820,11 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>2940</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="233">
@@ -4763,11 +4835,11 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>2983</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="234">
@@ -4778,11 +4850,11 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>2979</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="235">
@@ -4793,11 +4865,11 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>2781</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="236">
@@ -4808,11 +4880,11 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>2778</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="237">
@@ -4823,11 +4895,131 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
+          <t>02/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C237" t="n">
+        <v>2843</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>02/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C238" t="n">
+        <v>2835</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C239" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C240" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C241" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C242" t="n">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>04/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C243" t="n">
+        <v>2778</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
           <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
-      <c r="C237" t="n">
+      <c r="C244" t="n">
         <v>2766</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>05/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>2774</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Monitor run 2026-06-05 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -490,27 +490,31 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>DIRECT</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>London Heathrow</t>
+        </is>
+      </c>
       <c r="D2" t="n">
-        <v>1343</v>
+        <v>1593</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>2.6</v>
+        <v>26.2</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -520,31 +524,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>London Heathrow</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1579</v>
+        <v>1702</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>26.2</v>
+        <v>15.5</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -554,31 +558,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Frankfurt</t>
-        </is>
-      </c>
+          <t>MUC</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>1687</v>
+        <v>1706</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>15.5</v>
+        <v>13.8</v>
       </c>
       <c r="G4" t="n">
         <v>2</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -588,27 +588,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>MUC</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>CPH</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Copenhagen</t>
+        </is>
+      </c>
       <c r="D5" t="n">
-        <v>1695</v>
+        <v>1864</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Lufthansa</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>13.8</v>
+        <v>15.6</v>
       </c>
       <c r="G5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -618,31 +622,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CPH</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Copenhagen</t>
-        </is>
-      </c>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>1848</v>
+        <v>2009</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>15.6</v>
+        <v>2.6</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>4550</v>
+        <v>4590</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -800,7 +800,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -917,22 +917,22 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1343</v>
+        <v>1593</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>2.6</v>
+        <v>26.2</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -959,22 +959,22 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1579</v>
+        <v>1702</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>26.2</v>
+        <v>15.5</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1001,22 +1001,22 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1687</v>
+        <v>1706</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>15.5</v>
+        <v>13.8</v>
       </c>
       <c r="I4" t="n">
         <v>2</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1695</v>
+        <v>1864</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Lufthansa</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>13.8</v>
+        <v>15.6</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1085,22 +1085,22 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>1848</v>
+        <v>2009</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>15.6</v>
+        <v>2.6</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>4550</v>
+        <v>4590</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C245"/>
+  <dimension ref="A1:C251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2895,16 +2895,16 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>228</v>
+        <v>1864</v>
       </c>
     </row>
     <row r="105">
@@ -2915,11 +2915,11 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="106">
@@ -2930,7 +2930,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -2990,11 +2990,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="111">
@@ -3005,11 +3005,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="112">
@@ -3020,11 +3020,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1334</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="113">
@@ -3035,11 +3035,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1345</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="114">
@@ -3050,11 +3050,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="115">
@@ -3065,11 +3065,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="116">
@@ -3080,11 +3080,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="117">
@@ -3095,11 +3095,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="118">
@@ -3110,11 +3110,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1337</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="119">
@@ -3125,11 +3125,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="120">
@@ -3140,11 +3140,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="121">
@@ -3155,7 +3155,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -3230,11 +3230,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="127">
@@ -3245,11 +3245,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="128">
@@ -3260,11 +3260,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="129">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -3290,11 +3290,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="131">
@@ -3305,11 +3305,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="132">
@@ -3320,11 +3320,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1329</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="133">
@@ -3335,11 +3335,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1324</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="134">
@@ -3350,11 +3350,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1344</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="135">
@@ -3365,11 +3365,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1342</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="136">
@@ -3380,11 +3380,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1346</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="137">
@@ -3395,11 +3395,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="138">
@@ -3410,11 +3410,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1339</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="139">
@@ -3425,17 +3425,17 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1343</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -3444,37 +3444,37 @@
         </is>
       </c>
       <c r="C140" t="n">
-        <v>3471</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>404</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2353</v>
+        <v>3471</v>
       </c>
     </row>
     <row r="143">
@@ -3485,11 +3485,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="144">
@@ -3500,7 +3500,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -3530,11 +3530,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="147">
@@ -3545,11 +3545,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="148">
@@ -3560,11 +3560,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2367</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="149">
@@ -3575,11 +3575,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>2238</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="150">
@@ -3590,11 +3590,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2257</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="151">
@@ -3605,11 +3605,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2196</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="152">
@@ -3620,11 +3620,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2185</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="153">
@@ -3635,11 +3635,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2189</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="154">
@@ -3650,11 +3650,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2191</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="155">
@@ -3665,11 +3665,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2185</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="156">
@@ -3680,11 +3680,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2196</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="157">
@@ -3695,11 +3695,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="158">
@@ -3710,11 +3710,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="159">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -3755,7 +3755,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -3785,11 +3785,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="164">
@@ -3800,11 +3800,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="165">
@@ -3815,11 +3815,11 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="166">
@@ -3830,11 +3830,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2182</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="167">
@@ -3845,11 +3845,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1675</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="168">
@@ -3860,11 +3860,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>1674</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="169">
@@ -3875,11 +3875,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1670</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="170">
@@ -3890,11 +3890,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>1664</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="171">
@@ -3905,11 +3905,11 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1688</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="172">
@@ -3920,11 +3920,11 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1686</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="173">
@@ -3935,11 +3935,11 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>1691</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="174">
@@ -3950,11 +3950,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>1689</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="175">
@@ -3965,11 +3965,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1682</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="176">
@@ -3980,56 +3980,56 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>1687</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>2848</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>2842</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>2831</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="180">
@@ -4040,11 +4040,11 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>2872</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="181">
@@ -4055,11 +4055,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>4547</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="182">
@@ -4070,11 +4070,11 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>4561</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="183">
@@ -4085,11 +4085,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>4557</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="184">
@@ -4100,11 +4100,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>4537</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="185">
@@ -4115,71 +4115,71 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>4550</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>410</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>2391</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>2391</v>
+        <v>4550</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>2391</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="190">
@@ -4190,11 +4190,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="191">
@@ -4205,11 +4205,11 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="192">
@@ -4220,11 +4220,11 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="193">
@@ -4235,11 +4235,11 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="194">
@@ -4250,11 +4250,11 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="195">
@@ -4265,11 +4265,11 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="196">
@@ -4280,11 +4280,11 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="197">
@@ -4295,11 +4295,11 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="198">
@@ -4310,11 +4310,11 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="199">
@@ -4325,11 +4325,11 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="200">
@@ -4340,11 +4340,11 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="201">
@@ -4355,11 +4355,11 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="202">
@@ -4370,11 +4370,11 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="203">
@@ -4385,11 +4385,11 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="204">
@@ -4400,11 +4400,11 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="205">
@@ -4415,11 +4415,11 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="206">
@@ -4430,11 +4430,11 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="207">
@@ -4445,11 +4445,11 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="208">
@@ -4460,11 +4460,11 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="209">
@@ -4475,11 +4475,11 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="210">
@@ -4490,11 +4490,11 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>2415</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="211">
@@ -4505,11 +4505,11 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>1655</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="212">
@@ -4520,11 +4520,11 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="213">
@@ -4535,11 +4535,11 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>1651</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="214">
@@ -4550,11 +4550,11 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1648</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="215">
@@ -4565,11 +4565,11 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>1558</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="216">
@@ -4580,11 +4580,11 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2428</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="217">
@@ -4595,11 +4595,11 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>2425</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="218">
@@ -4610,11 +4610,11 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>2432</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="219">
@@ -4625,11 +4625,11 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1581</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="220">
@@ -4640,11 +4640,11 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>1574</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="221">
@@ -4655,146 +4655,146 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>1579</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>1692</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1690</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>1695</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>2704</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>2718</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>2705</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>2705</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>2706</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>2706</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="231">
@@ -4805,11 +4805,11 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="232">
@@ -4820,11 +4820,11 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="233">
@@ -4835,11 +4835,11 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>2704</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="234">
@@ -4850,11 +4850,11 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="235">
@@ -4865,11 +4865,11 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>2879</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="236">
@@ -4880,11 +4880,11 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="237">
@@ -4895,11 +4895,11 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="238">
@@ -4910,11 +4910,11 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="239">
@@ -4925,11 +4925,11 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>2940</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="240">
@@ -4940,11 +4940,11 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>2983</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="241">
@@ -4955,11 +4955,11 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>2979</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="242">
@@ -4970,11 +4970,11 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2781</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="243">
@@ -4985,11 +4985,11 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>2778</v>
+        <v>2843</v>
       </c>
     </row>
     <row r="244">
@@ -5000,11 +5000,11 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>2766</v>
+        <v>2835</v>
       </c>
     </row>
     <row r="245">
@@ -5015,10 +5015,100 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C245" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C246" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C247" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C248" t="n">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>04/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C249" t="n">
+        <v>2778</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>04/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C250" t="n">
+        <v>2766</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
           <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C245" t="n">
+      <c r="C251" t="n">
         <v>2774</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-06-05 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1593</v>
+        <v>1596</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1702</v>
+        <v>1705</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -548,7 +548,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>1706</v>
+        <v>1709</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1864</v>
+        <v>1868</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>2009</v>
+        <v>2013</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>4590</v>
+        <v>4600</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -800,7 +800,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1593</v>
+        <v>1596</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -932,7 +932,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1702</v>
+        <v>1705</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -974,7 +974,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1706</v>
+        <v>1709</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1864</v>
+        <v>1868</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1085,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2009</v>
+        <v>2013</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>4590</v>
+        <v>4600</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C251"/>
+  <dimension ref="A1:C257"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2910,16 +2910,16 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C105" t="n">
-        <v>228</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="106">
@@ -2930,11 +2930,11 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="107">
@@ -2945,7 +2945,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -3005,11 +3005,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="112">
@@ -3020,11 +3020,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="113">
@@ -3035,11 +3035,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1334</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="114">
@@ -3050,11 +3050,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1345</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="115">
@@ -3065,11 +3065,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="116">
@@ -3080,11 +3080,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="117">
@@ -3095,11 +3095,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="118">
@@ -3110,11 +3110,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="119">
@@ -3125,11 +3125,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1337</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="120">
@@ -3140,11 +3140,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="121">
@@ -3155,11 +3155,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="122">
@@ -3170,7 +3170,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -3245,11 +3245,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="128">
@@ -3260,11 +3260,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="129">
@@ -3275,11 +3275,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="130">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -3305,11 +3305,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="132">
@@ -3320,11 +3320,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="133">
@@ -3335,11 +3335,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1329</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="134">
@@ -3350,11 +3350,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1324</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="135">
@@ -3365,11 +3365,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1344</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="136">
@@ -3380,11 +3380,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1342</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="137">
@@ -3395,11 +3395,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1346</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="138">
@@ -3410,11 +3410,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="139">
@@ -3425,11 +3425,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1339</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="140">
@@ -3440,11 +3440,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1343</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="141">
@@ -3455,56 +3455,56 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>2009</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>3471</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>404</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>2353</v>
+        <v>3471</v>
       </c>
     </row>
     <row r="145">
@@ -3515,11 +3515,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="146">
@@ -3530,7 +3530,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -3560,11 +3560,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="149">
@@ -3575,11 +3575,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="150">
@@ -3590,11 +3590,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2367</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="151">
@@ -3605,11 +3605,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2238</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="152">
@@ -3620,11 +3620,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2257</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="153">
@@ -3635,11 +3635,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2196</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="154">
@@ -3650,11 +3650,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2185</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="155">
@@ -3665,11 +3665,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2189</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="156">
@@ -3680,11 +3680,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2191</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="157">
@@ -3695,11 +3695,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2185</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="158">
@@ -3710,11 +3710,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2196</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="159">
@@ -3725,11 +3725,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="160">
@@ -3740,11 +3740,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="161">
@@ -3755,7 +3755,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -3785,7 +3785,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -3800,7 +3800,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -3815,11 +3815,11 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="166">
@@ -3830,11 +3830,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="167">
@@ -3845,11 +3845,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="168">
@@ -3860,11 +3860,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2182</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="169">
@@ -3875,11 +3875,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1675</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="170">
@@ -3890,11 +3890,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>1674</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="171">
@@ -3905,11 +3905,11 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1670</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="172">
@@ -3920,11 +3920,11 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1664</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="173">
@@ -3935,11 +3935,11 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>1688</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="174">
@@ -3950,11 +3950,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>1686</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="175">
@@ -3965,11 +3965,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1691</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="176">
@@ -3980,11 +3980,11 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>1689</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="177">
@@ -3995,11 +3995,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>1682</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="178">
@@ -4010,11 +4010,11 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>1687</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="179">
@@ -4025,56 +4025,56 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1702</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>2848</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>2842</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>2831</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="183">
@@ -4085,11 +4085,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>2872</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="184">
@@ -4100,11 +4100,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>4547</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="185">
@@ -4115,11 +4115,11 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>4561</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="186">
@@ -4130,11 +4130,11 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>4557</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="187">
@@ -4145,11 +4145,11 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>4537</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="188">
@@ -4160,11 +4160,11 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>4550</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="189">
@@ -4175,71 +4175,71 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>4590</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>410</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>2391</v>
+        <v>4550</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>2391</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>2391</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="194">
@@ -4250,11 +4250,11 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="195">
@@ -4265,11 +4265,11 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="196">
@@ -4280,11 +4280,11 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="197">
@@ -4295,11 +4295,11 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="198">
@@ -4310,11 +4310,11 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="199">
@@ -4325,11 +4325,11 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="200">
@@ -4340,11 +4340,11 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="201">
@@ -4355,11 +4355,11 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="202">
@@ -4370,11 +4370,11 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="203">
@@ -4385,11 +4385,11 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="204">
@@ -4400,11 +4400,11 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="205">
@@ -4415,11 +4415,11 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="206">
@@ -4430,11 +4430,11 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="207">
@@ -4445,11 +4445,11 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="208">
@@ -4460,11 +4460,11 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="209">
@@ -4475,11 +4475,11 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="210">
@@ -4490,11 +4490,11 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="211">
@@ -4505,11 +4505,11 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="212">
@@ -4520,11 +4520,11 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="213">
@@ -4535,11 +4535,11 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="214">
@@ -4550,11 +4550,11 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>2415</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="215">
@@ -4565,11 +4565,11 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>1655</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="216">
@@ -4580,11 +4580,11 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="217">
@@ -4595,11 +4595,11 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>1651</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="218">
@@ -4610,11 +4610,11 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>1648</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="219">
@@ -4625,11 +4625,11 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1558</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="220">
@@ -4640,11 +4640,11 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>2428</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="221">
@@ -4655,11 +4655,11 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>2425</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="222">
@@ -4670,11 +4670,11 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>2432</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="223">
@@ -4685,11 +4685,11 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1581</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="224">
@@ -4700,11 +4700,11 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>1574</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="225">
@@ -4715,11 +4715,11 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>1579</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="226">
@@ -4730,62 +4730,62 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>1593</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>1692</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>1690</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>1695</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
@@ -4794,97 +4794,97 @@
         </is>
       </c>
       <c r="C230" t="n">
-        <v>1706</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>2704</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>2718</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>2705</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>2705</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>2706</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>2706</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="237">
@@ -4895,11 +4895,11 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="238">
@@ -4910,11 +4910,11 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="239">
@@ -4925,11 +4925,11 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>2704</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="240">
@@ -4940,11 +4940,11 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="241">
@@ -4955,11 +4955,11 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>2879</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="242">
@@ -4970,11 +4970,11 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="243">
@@ -4985,11 +4985,11 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="244">
@@ -5000,11 +5000,11 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="245">
@@ -5015,11 +5015,11 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>2940</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="246">
@@ -5030,11 +5030,11 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>2983</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="247">
@@ -5045,11 +5045,11 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>2979</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="248">
@@ -5060,11 +5060,11 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>2781</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="249">
@@ -5075,11 +5075,11 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>2778</v>
+        <v>2843</v>
       </c>
     </row>
     <row r="250">
@@ -5090,11 +5090,11 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C250" t="n">
-        <v>2766</v>
+        <v>2835</v>
       </c>
     </row>
     <row r="251">
@@ -5105,10 +5105,100 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C253" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C254" t="n">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>04/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C255" t="n">
+        <v>2778</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>04/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C256" t="n">
+        <v>2766</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
           <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C251" t="n">
+      <c r="C257" t="n">
         <v>2774</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-06-06 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1705</v>
+        <v>1706</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -548,7 +548,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1705</v>
+        <v>1706</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -974,7 +974,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1709</v>
+        <v>1710</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C257"/>
+  <dimension ref="A1:C263"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2925,16 +2925,16 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C106" t="n">
-        <v>228</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="107">
@@ -2945,11 +2945,11 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="108">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -3020,11 +3020,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="113">
@@ -3035,11 +3035,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="114">
@@ -3050,11 +3050,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1334</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="115">
@@ -3065,11 +3065,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1345</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="116">
@@ -3080,11 +3080,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="117">
@@ -3095,11 +3095,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="118">
@@ -3110,11 +3110,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="119">
@@ -3125,11 +3125,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="120">
@@ -3140,11 +3140,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1337</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="121">
@@ -3155,11 +3155,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="122">
@@ -3170,11 +3170,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="123">
@@ -3185,7 +3185,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -3260,11 +3260,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="129">
@@ -3275,11 +3275,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="130">
@@ -3290,11 +3290,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="131">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -3320,11 +3320,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="133">
@@ -3335,11 +3335,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="134">
@@ -3350,11 +3350,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1329</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="135">
@@ -3365,11 +3365,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1324</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="136">
@@ -3380,11 +3380,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1344</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="137">
@@ -3395,11 +3395,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1342</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="138">
@@ -3410,11 +3410,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1346</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="139">
@@ -3425,11 +3425,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="140">
@@ -3440,11 +3440,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1339</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="141">
@@ -3455,11 +3455,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1343</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="142">
@@ -3470,11 +3470,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>2009</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="143">
@@ -3485,56 +3485,56 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2013</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>3471</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>404</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2353</v>
+        <v>3471</v>
       </c>
     </row>
     <row r="147">
@@ -3545,11 +3545,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="148">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -3575,7 +3575,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -3590,11 +3590,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="151">
@@ -3605,11 +3605,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="152">
@@ -3620,11 +3620,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2367</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="153">
@@ -3635,11 +3635,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2238</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="154">
@@ -3650,11 +3650,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2257</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="155">
@@ -3665,11 +3665,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2196</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="156">
@@ -3680,11 +3680,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2185</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="157">
@@ -3695,11 +3695,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2189</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="158">
@@ -3710,11 +3710,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2191</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="159">
@@ -3725,11 +3725,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2185</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="160">
@@ -3740,11 +3740,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2196</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="161">
@@ -3755,11 +3755,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="162">
@@ -3770,11 +3770,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="163">
@@ -3785,7 +3785,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -3800,7 +3800,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -3815,7 +3815,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -3830,7 +3830,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -3845,11 +3845,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="168">
@@ -3860,11 +3860,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="169">
@@ -3875,11 +3875,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="170">
@@ -3890,11 +3890,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2182</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="171">
@@ -3905,11 +3905,11 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1675</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="172">
@@ -3920,11 +3920,11 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1674</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="173">
@@ -3935,11 +3935,11 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>1670</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="174">
@@ -3950,11 +3950,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>1664</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="175">
@@ -3965,11 +3965,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1688</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="176">
@@ -3980,11 +3980,11 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>1686</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="177">
@@ -3995,11 +3995,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>1691</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="178">
@@ -4010,11 +4010,11 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>1689</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="179">
@@ -4025,11 +4025,11 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1682</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="180">
@@ -4040,11 +4040,11 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>1687</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="181">
@@ -4055,11 +4055,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>1702</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="182">
@@ -4070,56 +4070,56 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>1705</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>2848</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>2842</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>2831</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="186">
@@ -4130,11 +4130,11 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2872</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="187">
@@ -4145,11 +4145,11 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>4547</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="188">
@@ -4160,11 +4160,11 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>4561</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="189">
@@ -4175,11 +4175,11 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>4557</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="190">
@@ -4190,11 +4190,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>4537</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="191">
@@ -4205,11 +4205,11 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>4550</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="192">
@@ -4220,11 +4220,11 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>4590</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="193">
@@ -4235,71 +4235,71 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>4600</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>410</v>
+        <v>4550</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>2391</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>2391</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>2391</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="198">
@@ -4310,11 +4310,11 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="199">
@@ -4325,11 +4325,11 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="200">
@@ -4340,11 +4340,11 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="201">
@@ -4355,11 +4355,11 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="202">
@@ -4370,11 +4370,11 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="203">
@@ -4385,11 +4385,11 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="204">
@@ -4400,11 +4400,11 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="205">
@@ -4415,11 +4415,11 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="206">
@@ -4430,11 +4430,11 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="207">
@@ -4445,11 +4445,11 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="208">
@@ -4460,11 +4460,11 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="209">
@@ -4475,11 +4475,11 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="210">
@@ -4490,11 +4490,11 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="211">
@@ -4505,11 +4505,11 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="212">
@@ -4520,11 +4520,11 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="213">
@@ -4535,11 +4535,11 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="214">
@@ -4550,11 +4550,11 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="215">
@@ -4565,11 +4565,11 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="216">
@@ -4580,11 +4580,11 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="217">
@@ -4595,11 +4595,11 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="218">
@@ -4610,11 +4610,11 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>2415</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="219">
@@ -4625,11 +4625,11 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1655</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="220">
@@ -4640,11 +4640,11 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="221">
@@ -4655,11 +4655,11 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>1651</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="222">
@@ -4670,11 +4670,11 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>1648</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="223">
@@ -4685,11 +4685,11 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1558</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="224">
@@ -4700,11 +4700,11 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>2428</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="225">
@@ -4715,11 +4715,11 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>2425</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="226">
@@ -4730,11 +4730,11 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>2432</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="227">
@@ -4745,11 +4745,11 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>1581</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="228">
@@ -4760,11 +4760,11 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>1574</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="229">
@@ -4775,11 +4775,11 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>1579</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="230">
@@ -4790,11 +4790,11 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>1593</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="231">
@@ -4805,176 +4805,176 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>1596</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>1692</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>1690</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>1695</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1706</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>1709</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>2704</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2718</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>2705</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>2705</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>2706</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2706</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="243">
@@ -4985,11 +4985,11 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="244">
@@ -5000,11 +5000,11 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="245">
@@ -5015,11 +5015,11 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>2704</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="246">
@@ -5030,11 +5030,11 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="247">
@@ -5045,11 +5045,11 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>2879</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="248">
@@ -5060,11 +5060,11 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="249">
@@ -5075,11 +5075,11 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="250">
@@ -5090,11 +5090,11 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C250" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="251">
@@ -5105,11 +5105,11 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C251" t="n">
-        <v>2940</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="252">
@@ -5120,11 +5120,11 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C252" t="n">
-        <v>2983</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="253">
@@ -5135,11 +5135,11 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C253" t="n">
-        <v>2979</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="254">
@@ -5150,11 +5150,11 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C254" t="n">
-        <v>2781</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="255">
@@ -5165,11 +5165,11 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C255" t="n">
-        <v>2778</v>
+        <v>2843</v>
       </c>
     </row>
     <row r="256">
@@ -5180,11 +5180,11 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C256" t="n">
-        <v>2766</v>
+        <v>2835</v>
       </c>
     </row>
     <row r="257">
@@ -5195,10 +5195,100 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C257" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C258" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C259" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C260" t="n">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>04/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C261" t="n">
+        <v>2778</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>04/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C262" t="n">
+        <v>2766</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
           <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C257" t="n">
+      <c r="C263" t="n">
         <v>2774</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-06-06 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C263"/>
+  <dimension ref="A1:C269"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2940,16 +2940,16 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C107" t="n">
-        <v>228</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="108">
@@ -2960,11 +2960,11 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="109">
@@ -2975,7 +2975,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -3035,11 +3035,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="114">
@@ -3050,11 +3050,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="115">
@@ -3065,11 +3065,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1334</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="116">
@@ -3080,11 +3080,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1345</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="117">
@@ -3095,11 +3095,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="118">
@@ -3110,11 +3110,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="119">
@@ -3125,11 +3125,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="120">
@@ -3140,11 +3140,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="121">
@@ -3155,11 +3155,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1337</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="122">
@@ -3170,11 +3170,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="123">
@@ -3185,11 +3185,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="124">
@@ -3200,7 +3200,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -3260,7 +3260,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -3275,11 +3275,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="130">
@@ -3290,11 +3290,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="131">
@@ -3305,11 +3305,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="132">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -3335,11 +3335,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="134">
@@ -3350,11 +3350,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="135">
@@ -3365,11 +3365,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1329</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="136">
@@ -3380,11 +3380,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1324</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="137">
@@ -3395,11 +3395,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1344</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="138">
@@ -3410,11 +3410,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1342</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="139">
@@ -3425,11 +3425,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1346</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="140">
@@ -3440,11 +3440,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="141">
@@ -3455,11 +3455,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1339</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="142">
@@ -3470,11 +3470,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1343</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="143">
@@ -3485,11 +3485,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>2009</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="144">
@@ -3500,11 +3500,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>2013</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="145">
@@ -3515,7 +3515,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
@@ -3525,46 +3525,46 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>3471</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>404</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2353</v>
+        <v>3471</v>
       </c>
     </row>
     <row r="149">
@@ -3575,11 +3575,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="150">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -3620,11 +3620,11 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="153">
@@ -3635,11 +3635,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="154">
@@ -3650,11 +3650,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2367</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="155">
@@ -3665,11 +3665,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2238</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="156">
@@ -3680,11 +3680,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2257</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="157">
@@ -3695,11 +3695,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2196</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="158">
@@ -3710,11 +3710,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2185</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="159">
@@ -3725,11 +3725,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2189</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="160">
@@ -3740,11 +3740,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2191</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="161">
@@ -3755,11 +3755,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2185</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="162">
@@ -3770,11 +3770,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2196</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="163">
@@ -3785,11 +3785,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="164">
@@ -3800,11 +3800,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="165">
@@ -3815,7 +3815,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -3830,7 +3830,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -3860,7 +3860,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -3875,11 +3875,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="170">
@@ -3890,11 +3890,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="171">
@@ -3905,11 +3905,11 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="172">
@@ -3920,11 +3920,11 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>2182</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="173">
@@ -3935,11 +3935,11 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>1675</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="174">
@@ -3950,11 +3950,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>1674</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="175">
@@ -3965,11 +3965,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1670</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="176">
@@ -3980,11 +3980,11 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>1664</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="177">
@@ -3995,11 +3995,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>1688</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="178">
@@ -4010,11 +4010,11 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>1686</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="179">
@@ -4025,11 +4025,11 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1691</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="180">
@@ -4040,11 +4040,11 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>1689</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="181">
@@ -4055,11 +4055,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>1682</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="182">
@@ -4070,11 +4070,11 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>1687</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="183">
@@ -4085,11 +4085,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>1702</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="184">
@@ -4100,11 +4100,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1705</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="185">
@@ -4115,56 +4115,56 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1706</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2848</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>2842</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>2831</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="189">
@@ -4175,11 +4175,11 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>2872</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="190">
@@ -4190,11 +4190,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>4547</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="191">
@@ -4205,11 +4205,11 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>4561</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="192">
@@ -4220,11 +4220,11 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>4557</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="193">
@@ -4235,11 +4235,11 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>4537</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="194">
@@ -4250,11 +4250,11 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>4550</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="195">
@@ -4265,11 +4265,11 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>4590</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="196">
@@ -4280,11 +4280,11 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>4600</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="197">
@@ -4295,71 +4295,71 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>4600</v>
+        <v>4550</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>410</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>2391</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>2391</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>2391</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="202">
@@ -4370,11 +4370,11 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="203">
@@ -4385,11 +4385,11 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="204">
@@ -4400,11 +4400,11 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="205">
@@ -4415,11 +4415,11 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="206">
@@ -4430,11 +4430,11 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="207">
@@ -4445,11 +4445,11 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="208">
@@ -4460,11 +4460,11 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="209">
@@ -4475,11 +4475,11 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="210">
@@ -4490,11 +4490,11 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="211">
@@ -4505,11 +4505,11 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="212">
@@ -4520,11 +4520,11 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="213">
@@ -4535,11 +4535,11 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="214">
@@ -4550,11 +4550,11 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="215">
@@ -4565,11 +4565,11 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="216">
@@ -4580,11 +4580,11 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="217">
@@ -4595,11 +4595,11 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="218">
@@ -4610,11 +4610,11 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="219">
@@ -4625,11 +4625,11 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="220">
@@ -4640,11 +4640,11 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="221">
@@ -4655,11 +4655,11 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="222">
@@ -4670,11 +4670,11 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>2415</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="223">
@@ -4685,11 +4685,11 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1655</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="224">
@@ -4700,11 +4700,11 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="225">
@@ -4715,11 +4715,11 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>1651</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="226">
@@ -4730,11 +4730,11 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>1648</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="227">
@@ -4745,11 +4745,11 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>1558</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="228">
@@ -4760,11 +4760,11 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>2428</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="229">
@@ -4775,11 +4775,11 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>2425</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="230">
@@ -4790,11 +4790,11 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>2432</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="231">
@@ -4805,11 +4805,11 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>1581</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="232">
@@ -4820,11 +4820,11 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>1574</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="233">
@@ -4835,11 +4835,11 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>1579</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="234">
@@ -4850,11 +4850,11 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>1593</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="235">
@@ -4865,11 +4865,11 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1596</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="236">
@@ -4880,86 +4880,86 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>1596</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>1692</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>1690</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1695</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>1706</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>1709</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="242">
@@ -4970,101 +4970,101 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>1710</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>2704</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>2718</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>2705</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>2705</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>2706</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>2706</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="249">
@@ -5075,11 +5075,11 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="250">
@@ -5090,11 +5090,11 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C250" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="251">
@@ -5105,11 +5105,11 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C251" t="n">
-        <v>2704</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="252">
@@ -5120,11 +5120,11 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C252" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="253">
@@ -5135,11 +5135,11 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C253" t="n">
-        <v>2879</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="254">
@@ -5150,11 +5150,11 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C254" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="255">
@@ -5165,11 +5165,11 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C255" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="256">
@@ -5180,11 +5180,11 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C256" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="257">
@@ -5195,11 +5195,11 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C257" t="n">
-        <v>2940</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="258">
@@ -5210,11 +5210,11 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C258" t="n">
-        <v>2983</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="259">
@@ -5225,11 +5225,11 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C259" t="n">
-        <v>2979</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="260">
@@ -5240,11 +5240,11 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C260" t="n">
-        <v>2781</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="261">
@@ -5255,11 +5255,11 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C261" t="n">
-        <v>2778</v>
+        <v>2843</v>
       </c>
     </row>
     <row r="262">
@@ -5270,11 +5270,11 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C262" t="n">
-        <v>2766</v>
+        <v>2835</v>
       </c>
     </row>
     <row r="263">
@@ -5285,10 +5285,100 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C263" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C264" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C265" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C266" t="n">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>04/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C267" t="n">
+        <v>2778</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>04/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C268" t="n">
+        <v>2766</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
           <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C263" t="n">
+      <c r="C269" t="n">
         <v>2774</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-06-06 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -490,31 +490,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LHR</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>London Heathrow</t>
-        </is>
-      </c>
+          <t>MUC</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>1596</v>
+        <v>1710</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>26.2</v>
+        <v>13.8</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -524,31 +520,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Frankfurt</t>
+          <t>Copenhagen</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1706</v>
+        <v>1868</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>15.5</v>
+        <v>15.6</v>
       </c>
       <c r="G3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -558,27 +554,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>1710</v>
+        <v>2013</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Lufthansa</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>13.8</v>
+        <v>2.6</v>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -588,31 +584,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Copenhagen</t>
+          <t>London Heathrow</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1868</v>
+        <v>2453</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>15.6</v>
+        <v>14.2</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -622,27 +618,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DIRECT</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>FRA</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Frankfurt</t>
+        </is>
+      </c>
       <c r="D6" t="n">
-        <v>2013</v>
+        <v>2632</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.6</v>
+        <v>12.1</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -800,7 +800,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -917,22 +917,22 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1596</v>
+        <v>1710</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>26.2</v>
+        <v>13.8</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -959,22 +959,22 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1706</v>
+        <v>1868</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>15.5</v>
+        <v>15.6</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1001,22 +1001,22 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1710</v>
+        <v>2013</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Lufthansa</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>13.8</v>
+        <v>2.6</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1868</v>
+        <v>2453</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>15.6</v>
+        <v>14.2</v>
       </c>
       <c r="I5" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1085,22 +1085,22 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2013</v>
+        <v>2632</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>2.6</v>
+        <v>12.1</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C269"/>
+  <dimension ref="A1:C277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2955,16 +2955,16 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C108" t="n">
-        <v>228</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="109">
@@ -2975,11 +2975,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="110">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -3050,11 +3050,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="115">
@@ -3065,11 +3065,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="116">
@@ -3080,11 +3080,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1334</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="117">
@@ -3095,11 +3095,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1345</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="118">
@@ -3110,11 +3110,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="119">
@@ -3125,11 +3125,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="120">
@@ -3140,11 +3140,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="121">
@@ -3155,11 +3155,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="122">
@@ -3170,11 +3170,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1337</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="123">
@@ -3185,11 +3185,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="124">
@@ -3200,11 +3200,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="125">
@@ -3215,7 +3215,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -3260,7 +3260,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -3290,11 +3290,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="131">
@@ -3305,11 +3305,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="132">
@@ -3320,11 +3320,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="133">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -3350,11 +3350,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="135">
@@ -3365,11 +3365,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="136">
@@ -3380,11 +3380,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1329</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="137">
@@ -3395,11 +3395,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1324</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="138">
@@ -3410,11 +3410,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1344</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="139">
@@ -3425,11 +3425,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1342</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="140">
@@ -3440,11 +3440,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1346</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="141">
@@ -3455,11 +3455,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="142">
@@ -3470,11 +3470,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1339</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="143">
@@ -3485,11 +3485,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1343</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="144">
@@ -3500,11 +3500,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>2009</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="145">
@@ -3515,11 +3515,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2013</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="146">
@@ -3530,7 +3530,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -3555,46 +3555,46 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>3471</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>404</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2353</v>
+        <v>3471</v>
       </c>
     </row>
     <row r="151">
@@ -3605,11 +3605,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="152">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -3650,11 +3650,11 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="155">
@@ -3665,11 +3665,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="156">
@@ -3680,11 +3680,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2367</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="157">
@@ -3695,11 +3695,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2238</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="158">
@@ -3710,11 +3710,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2257</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="159">
@@ -3725,11 +3725,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2196</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="160">
@@ -3740,11 +3740,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2185</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="161">
@@ -3755,11 +3755,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2189</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="162">
@@ -3770,11 +3770,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2191</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="163">
@@ -3785,11 +3785,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2185</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="164">
@@ -3800,11 +3800,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2196</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="165">
@@ -3815,11 +3815,11 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="166">
@@ -3830,11 +3830,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="167">
@@ -3845,7 +3845,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
@@ -3860,7 +3860,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -3890,7 +3890,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -3905,11 +3905,11 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="172">
@@ -3920,11 +3920,11 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="173">
@@ -3935,11 +3935,11 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="174">
@@ -3950,11 +3950,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>2182</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="175">
@@ -3965,11 +3965,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1675</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="176">
@@ -3980,11 +3980,11 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>1674</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="177">
@@ -3995,11 +3995,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>1670</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="178">
@@ -4010,11 +4010,11 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>1664</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="179">
@@ -4025,11 +4025,11 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1688</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="180">
@@ -4040,11 +4040,11 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>1686</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="181">
@@ -4055,11 +4055,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>1691</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="182">
@@ -4070,11 +4070,11 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>1689</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="183">
@@ -4085,11 +4085,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>1682</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="184">
@@ -4100,11 +4100,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1687</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="185">
@@ -4115,11 +4115,11 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1702</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="186">
@@ -4130,11 +4130,11 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>1705</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="187">
@@ -4145,11 +4145,11 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1706</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="188">
@@ -4160,71 +4160,71 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>1706</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>2848</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>2842</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>2831</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>2872</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="193">
@@ -4235,11 +4235,11 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>4547</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="194">
@@ -4250,11 +4250,11 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>4561</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="195">
@@ -4265,11 +4265,11 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>4557</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="196">
@@ -4280,11 +4280,11 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>4537</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="197">
@@ -4295,11 +4295,11 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>4550</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="198">
@@ -4310,11 +4310,11 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>4590</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="199">
@@ -4325,11 +4325,11 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>4600</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="200">
@@ -4340,11 +4340,11 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>4600</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="201">
@@ -4355,86 +4355,86 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>4600</v>
+        <v>4550</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>410</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>2391</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>2391</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>2391</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>2391</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="207">
@@ -4445,11 +4445,11 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>2389</v>
+        <v>410</v>
       </c>
     </row>
     <row r="208">
@@ -4460,11 +4460,11 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="209">
@@ -4475,11 +4475,11 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="210">
@@ -4490,11 +4490,11 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="211">
@@ -4505,11 +4505,11 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>2419</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="212">
@@ -4520,11 +4520,11 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>1660</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="213">
@@ -4535,11 +4535,11 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>1652</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="214">
@@ -4550,11 +4550,11 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>1655</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="215">
@@ -4565,11 +4565,11 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>2411</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="216">
@@ -4580,11 +4580,11 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2404</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="217">
@@ -4595,11 +4595,11 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>2416</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="218">
@@ -4610,11 +4610,11 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>2405</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="219">
@@ -4625,11 +4625,11 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="220">
@@ -4640,11 +4640,11 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>2406</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="221">
@@ -4655,11 +4655,11 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="222">
@@ -4670,11 +4670,11 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>1652</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="223">
@@ -4685,11 +4685,11 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="224">
@@ -4700,11 +4700,11 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>2404</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="225">
@@ -4715,11 +4715,11 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="226">
@@ -4730,11 +4730,11 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>2415</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="227">
@@ -4745,11 +4745,11 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>1655</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="228">
@@ -4760,7 +4760,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C228" t="n">
@@ -4775,11 +4775,11 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>1651</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="230">
@@ -4790,11 +4790,11 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>1648</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="231">
@@ -4805,11 +4805,11 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>1558</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="232">
@@ -4820,11 +4820,11 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>2428</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="233">
@@ -4835,11 +4835,11 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>2425</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="234">
@@ -4850,11 +4850,11 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>2432</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="235">
@@ -4865,11 +4865,11 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1581</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="236">
@@ -4880,11 +4880,11 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>1574</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="237">
@@ -4895,11 +4895,11 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>1579</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="238">
@@ -4910,11 +4910,11 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>1593</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="239">
@@ -4925,11 +4925,11 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1596</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="240">
@@ -4940,11 +4940,11 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>1596</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="241">
@@ -4955,236 +4955,236 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>1596</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>1692</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>1690</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1695</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>1706</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>1709</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>1710</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>1710</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>2704</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C250" t="n">
-        <v>2718</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C251" t="n">
-        <v>2705</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C252" t="n">
-        <v>2705</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C253" t="n">
-        <v>2706</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C254" t="n">
-        <v>2706</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C255" t="n">
-        <v>2706</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C256" t="n">
-        <v>2706</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="257">
@@ -5195,7 +5195,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -5210,11 +5210,11 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C258" t="n">
-        <v>2887</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="259">
@@ -5225,11 +5225,11 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C259" t="n">
-        <v>2879</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="260">
@@ -5240,11 +5240,11 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C260" t="n">
-        <v>2877</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="261">
@@ -5255,11 +5255,11 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C261" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="262">
@@ -5270,11 +5270,11 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C262" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="263">
@@ -5285,11 +5285,11 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C263" t="n">
-        <v>2940</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="264">
@@ -5300,11 +5300,11 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C264" t="n">
-        <v>2983</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="265">
@@ -5315,11 +5315,11 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C265" t="n">
-        <v>2979</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="266">
@@ -5330,11 +5330,11 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C266" t="n">
-        <v>2781</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="267">
@@ -5345,11 +5345,11 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C267" t="n">
-        <v>2778</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="268">
@@ -5360,11 +5360,11 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C268" t="n">
-        <v>2766</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="269">
@@ -5375,10 +5375,130 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
+          <t>02/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C269" t="n">
+        <v>2843</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>02/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C270" t="n">
+        <v>2835</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C271" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C272" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C273" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C274" t="n">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>04/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C275" t="n">
+        <v>2778</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>04/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C276" t="n">
+        <v>2766</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
           <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C269" t="n">
+      <c r="C277" t="n">
         <v>2774</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-06-07 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -490,27 +490,31 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>MUC</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>London Heathrow</t>
+        </is>
+      </c>
       <c r="D2" t="n">
-        <v>1710</v>
+        <v>1596</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Lufthansa</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>13.8</v>
+        <v>26.2</v>
       </c>
       <c r="G2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -520,31 +524,31 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Copenhagen</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1868</v>
+        <v>1705</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>15.6</v>
+        <v>15.5</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -554,27 +558,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>2013</v>
+        <v>1709</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2.6</v>
+        <v>13.8</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -584,31 +588,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>London Heathrow</t>
+          <t>Copenhagen</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>2453</v>
+        <v>1868</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>14.2</v>
+        <v>15.6</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -618,31 +622,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>Frankfurt</t>
-        </is>
-      </c>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>2632</v>
+        <v>2013</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Lufthansa</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>12.1</v>
+        <v>2.6</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -750,27 +750,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>3471</v>
+        <v>3407</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>9.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="G10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -780,27 +780,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>4600</v>
+        <v>3471</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>7.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -917,22 +917,22 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1710</v>
+        <v>1596</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Lufthansa</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>13.8</v>
+        <v>26.2</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -959,22 +959,22 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1868</v>
+        <v>1705</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>15.6</v>
+        <v>15.5</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1001,22 +1001,22 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>2013</v>
+        <v>1709</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>2.6</v>
+        <v>13.8</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2453</v>
+        <v>1868</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>14.2</v>
+        <v>15.6</v>
       </c>
       <c r="I5" t="n">
         <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1085,22 +1085,22 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2632</v>
+        <v>2013</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Lufthansa</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>12.1</v>
+        <v>2.6</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1253,22 +1253,22 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>3471</v>
+        <v>3407</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>9.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1295,22 +1295,22 @@
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>4600</v>
+        <v>3471</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>7.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C277"/>
+  <dimension ref="A1:C283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2970,16 +2970,16 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>228</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="110">
@@ -2990,11 +2990,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="111">
@@ -3005,7 +3005,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -3065,11 +3065,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="116">
@@ -3080,11 +3080,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="117">
@@ -3095,11 +3095,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1334</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="118">
@@ -3110,11 +3110,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1345</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="119">
@@ -3125,11 +3125,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="120">
@@ -3140,11 +3140,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="121">
@@ -3155,11 +3155,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="122">
@@ -3170,11 +3170,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="123">
@@ -3185,11 +3185,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1337</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="124">
@@ -3200,11 +3200,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="125">
@@ -3215,11 +3215,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="126">
@@ -3230,7 +3230,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -3260,7 +3260,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -3305,11 +3305,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="132">
@@ -3320,11 +3320,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="133">
@@ -3335,11 +3335,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="134">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -3365,11 +3365,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="136">
@@ -3380,11 +3380,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="137">
@@ -3395,11 +3395,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1329</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="138">
@@ -3410,11 +3410,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1324</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="139">
@@ -3425,11 +3425,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1344</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="140">
@@ -3440,11 +3440,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1342</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="141">
@@ -3455,11 +3455,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1346</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="142">
@@ -3470,11 +3470,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="143">
@@ -3485,11 +3485,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1339</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="144">
@@ -3500,11 +3500,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1343</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="145">
@@ -3515,11 +3515,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>2009</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="146">
@@ -3530,11 +3530,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2013</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="147">
@@ -3545,7 +3545,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -3575,7 +3575,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -3585,46 +3585,46 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>3471</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>404</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>2353</v>
+        <v>3471</v>
       </c>
     </row>
     <row r="153">
@@ -3635,11 +3635,11 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="154">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -3680,11 +3680,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="157">
@@ -3695,11 +3695,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="158">
@@ -3710,11 +3710,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2367</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="159">
@@ -3725,11 +3725,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2238</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="160">
@@ -3740,11 +3740,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2257</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="161">
@@ -3755,11 +3755,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2196</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="162">
@@ -3770,11 +3770,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2185</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="163">
@@ -3785,11 +3785,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2189</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="164">
@@ -3800,11 +3800,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2191</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="165">
@@ -3815,11 +3815,11 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2185</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="166">
@@ -3830,11 +3830,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2196</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="167">
@@ -3845,11 +3845,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="168">
@@ -3860,11 +3860,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="169">
@@ -3875,7 +3875,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
@@ -3890,7 +3890,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
@@ -3905,7 +3905,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -3935,11 +3935,11 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="174">
@@ -3950,11 +3950,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="175">
@@ -3965,11 +3965,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="176">
@@ -3980,11 +3980,11 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>2182</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="177">
@@ -3995,11 +3995,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>1675</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="178">
@@ -4010,11 +4010,11 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>1674</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="179">
@@ -4025,11 +4025,11 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1670</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="180">
@@ -4040,11 +4040,11 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>1664</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="181">
@@ -4055,11 +4055,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>1688</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="182">
@@ -4070,11 +4070,11 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>1686</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="183">
@@ -4085,11 +4085,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>1691</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="184">
@@ -4100,11 +4100,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1689</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="185">
@@ -4115,11 +4115,11 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1682</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="186">
@@ -4130,11 +4130,11 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>1687</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="187">
@@ -4145,11 +4145,11 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1702</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="188">
@@ -4160,11 +4160,11 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>1705</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="189">
@@ -4175,11 +4175,11 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>1706</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="190">
@@ -4190,11 +4190,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1706</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="191">
@@ -4205,7 +4205,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
@@ -4220,56 +4220,56 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>2632</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>2848</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>2842</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>2831</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="196">
@@ -4280,11 +4280,11 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>2872</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="197">
@@ -4295,11 +4295,11 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>4547</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="198">
@@ -4310,11 +4310,11 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>4561</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="199">
@@ -4325,11 +4325,11 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>4557</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="200">
@@ -4340,11 +4340,11 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>4537</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="201">
@@ -4355,11 +4355,11 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>4550</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="202">
@@ -4370,11 +4370,11 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>4590</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="203">
@@ -4385,11 +4385,11 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>4600</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="204">
@@ -4400,11 +4400,11 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>4600</v>
+        <v>4550</v>
       </c>
     </row>
     <row r="205">
@@ -4415,11 +4415,11 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>4600</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="206">
@@ -4430,7 +4430,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
@@ -4440,61 +4440,61 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>410</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2391</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>2391</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>2391</v>
+        <v>3407</v>
       </c>
     </row>
     <row r="211">
@@ -4505,11 +4505,11 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="212">
@@ -4520,11 +4520,11 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="213">
@@ -4535,11 +4535,11 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="214">
@@ -4550,11 +4550,11 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="215">
@@ -4565,11 +4565,11 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="216">
@@ -4580,11 +4580,11 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="217">
@@ -4595,11 +4595,11 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="218">
@@ -4610,11 +4610,11 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="219">
@@ -4625,11 +4625,11 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="220">
@@ -4640,11 +4640,11 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="221">
@@ -4655,11 +4655,11 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="222">
@@ -4670,11 +4670,11 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="223">
@@ -4685,11 +4685,11 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="224">
@@ -4700,11 +4700,11 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="225">
@@ -4715,11 +4715,11 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="226">
@@ -4730,11 +4730,11 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="227">
@@ -4745,11 +4745,11 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="228">
@@ -4760,11 +4760,11 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="229">
@@ -4775,11 +4775,11 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="230">
@@ -4790,11 +4790,11 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="231">
@@ -4805,11 +4805,11 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>2415</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="232">
@@ -4820,11 +4820,11 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>1655</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="233">
@@ -4835,11 +4835,11 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="234">
@@ -4850,11 +4850,11 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>1651</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="235">
@@ -4865,11 +4865,11 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1648</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="236">
@@ -4880,11 +4880,11 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>1558</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="237">
@@ -4895,11 +4895,11 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>2428</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="238">
@@ -4910,11 +4910,11 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2425</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="239">
@@ -4925,11 +4925,11 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>2432</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="240">
@@ -4940,11 +4940,11 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>1581</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="241">
@@ -4955,11 +4955,11 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>1574</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="242">
@@ -4970,11 +4970,11 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>1579</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="243">
@@ -4985,11 +4985,11 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>1593</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="244">
@@ -5000,11 +5000,11 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1596</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="245">
@@ -5015,11 +5015,11 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>1596</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="246">
@@ -5030,11 +5030,11 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>1596</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="247">
@@ -5045,11 +5045,11 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>1596</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="248">
@@ -5060,86 +5060,86 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>2453</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>1692</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C250" t="n">
-        <v>1690</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C251" t="n">
-        <v>1695</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C252" t="n">
-        <v>1706</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C253" t="n">
-        <v>1709</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="254">
@@ -5150,11 +5150,11 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C254" t="n">
-        <v>1710</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="255">
@@ -5165,11 +5165,11 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C255" t="n">
-        <v>1710</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="256">
@@ -5180,101 +5180,101 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C256" t="n">
-        <v>1710</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C257" t="n">
-        <v>2704</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C258" t="n">
-        <v>2718</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C259" t="n">
-        <v>2705</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C260" t="n">
-        <v>2705</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C261" t="n">
-        <v>2706</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C262" t="n">
-        <v>2706</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="263">
@@ -5285,11 +5285,11 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C263" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="264">
@@ -5300,11 +5300,11 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C264" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="265">
@@ -5315,11 +5315,11 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C265" t="n">
-        <v>2704</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="266">
@@ -5330,11 +5330,11 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C266" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="267">
@@ -5345,11 +5345,11 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C267" t="n">
-        <v>2879</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="268">
@@ -5360,11 +5360,11 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C268" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="269">
@@ -5375,11 +5375,11 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C269" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="270">
@@ -5390,11 +5390,11 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C270" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="271">
@@ -5405,11 +5405,11 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C271" t="n">
-        <v>2940</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="272">
@@ -5420,11 +5420,11 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C272" t="n">
-        <v>2983</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="273">
@@ -5435,11 +5435,11 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C273" t="n">
-        <v>2979</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="274">
@@ -5450,11 +5450,11 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C274" t="n">
-        <v>2781</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="275">
@@ -5465,11 +5465,11 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C275" t="n">
-        <v>2778</v>
+        <v>2843</v>
       </c>
     </row>
     <row r="276">
@@ -5480,11 +5480,11 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C276" t="n">
-        <v>2766</v>
+        <v>2835</v>
       </c>
     </row>
     <row r="277">
@@ -5495,10 +5495,100 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C277" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C278" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C279" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C280" t="n">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>04/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C281" t="n">
+        <v>2778</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>04/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C282" t="n">
+        <v>2766</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
           <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C277" t="n">
+      <c r="C283" t="n">
         <v>2774</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-06-07 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -642,7 +642,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -750,27 +750,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>3407</v>
+        <v>3471</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>7.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -780,27 +780,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>3471</v>
+        <v>4599</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>9.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="G11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -974,7 +974,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1253,22 +1253,22 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>3407</v>
+        <v>3471</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>7.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1295,22 +1295,22 @@
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>3471</v>
+        <v>4599</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>9.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="I11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C283"/>
+  <dimension ref="A1:C289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -2985,16 +2985,16 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>228</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="111">
@@ -3005,11 +3005,11 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="112">
@@ -3020,7 +3020,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -3080,11 +3080,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="117">
@@ -3095,11 +3095,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="118">
@@ -3110,11 +3110,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1334</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="119">
@@ -3125,11 +3125,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1345</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="120">
@@ -3140,11 +3140,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="121">
@@ -3155,11 +3155,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="122">
@@ -3170,11 +3170,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="123">
@@ -3185,11 +3185,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="124">
@@ -3200,11 +3200,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1337</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="125">
@@ -3215,11 +3215,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="126">
@@ -3230,11 +3230,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="127">
@@ -3245,7 +3245,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
@@ -3260,7 +3260,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -3320,11 +3320,11 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="133">
@@ -3335,11 +3335,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="134">
@@ -3350,11 +3350,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="135">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -3380,11 +3380,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="137">
@@ -3395,11 +3395,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="138">
@@ -3410,11 +3410,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1329</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="139">
@@ -3425,11 +3425,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1324</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="140">
@@ -3440,11 +3440,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1344</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="141">
@@ -3455,11 +3455,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1342</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="142">
@@ -3470,11 +3470,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1346</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="143">
@@ -3485,11 +3485,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="144">
@@ -3500,11 +3500,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1339</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="145">
@@ -3515,11 +3515,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1343</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="146">
@@ -3530,11 +3530,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>2009</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="147">
@@ -3545,11 +3545,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2013</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="148">
@@ -3560,7 +3560,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
@@ -3575,7 +3575,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -3615,46 +3615,46 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
-        <v>3471</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
-        <v>404</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>2353</v>
+        <v>3471</v>
       </c>
     </row>
     <row r="155">
@@ -3665,11 +3665,11 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="156">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -3695,7 +3695,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
@@ -3710,11 +3710,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="159">
@@ -3725,11 +3725,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="160">
@@ -3740,11 +3740,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2367</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="161">
@@ -3755,11 +3755,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2238</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="162">
@@ -3770,11 +3770,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2257</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="163">
@@ -3785,11 +3785,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2196</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="164">
@@ -3800,11 +3800,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2185</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="165">
@@ -3815,11 +3815,11 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2189</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="166">
@@ -3830,11 +3830,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2191</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="167">
@@ -3845,11 +3845,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2185</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="168">
@@ -3860,11 +3860,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2196</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="169">
@@ -3875,11 +3875,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="170">
@@ -3890,11 +3890,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="171">
@@ -3905,7 +3905,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
@@ -3920,7 +3920,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -3965,11 +3965,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="176">
@@ -3980,11 +3980,11 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="177">
@@ -3995,11 +3995,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="178">
@@ -4010,11 +4010,11 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>2182</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="179">
@@ -4025,11 +4025,11 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1675</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="180">
@@ -4040,11 +4040,11 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>1674</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="181">
@@ -4055,11 +4055,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>1670</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="182">
@@ -4070,11 +4070,11 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>1664</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="183">
@@ -4085,11 +4085,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>1688</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="184">
@@ -4100,11 +4100,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1686</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="185">
@@ -4115,11 +4115,11 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1691</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="186">
@@ -4130,11 +4130,11 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>1689</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="187">
@@ -4145,11 +4145,11 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1682</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="188">
@@ -4160,11 +4160,11 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>1687</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="189">
@@ -4175,11 +4175,11 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>1702</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="190">
@@ -4190,11 +4190,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1705</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="191">
@@ -4205,11 +4205,11 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1706</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="192">
@@ -4220,11 +4220,11 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>1706</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="193">
@@ -4235,7 +4235,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
@@ -4250,11 +4250,11 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>2632</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="195">
@@ -4265,56 +4265,56 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1705</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>2848</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>2842</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>2831</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="199">
@@ -4325,11 +4325,11 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>2872</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="200">
@@ -4340,11 +4340,11 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>4547</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="201">
@@ -4355,11 +4355,11 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>4561</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="202">
@@ -4370,11 +4370,11 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>4557</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="203">
@@ -4385,11 +4385,11 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>4537</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="204">
@@ -4400,11 +4400,11 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>4550</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="205">
@@ -4415,11 +4415,11 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>4590</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="206">
@@ -4430,11 +4430,11 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>4600</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="207">
@@ -4445,11 +4445,11 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>4600</v>
+        <v>4550</v>
       </c>
     </row>
     <row r="208">
@@ -4460,11 +4460,11 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>4600</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="209">
@@ -4475,7 +4475,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
@@ -4490,71 +4490,71 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>3407</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>410</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>2391</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>2391</v>
+        <v>3407</v>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>2391</v>
+        <v>4599</v>
       </c>
     </row>
     <row r="215">
@@ -4565,11 +4565,11 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="216">
@@ -4580,11 +4580,11 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="217">
@@ -4595,11 +4595,11 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="218">
@@ -4610,11 +4610,11 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="219">
@@ -4625,11 +4625,11 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="220">
@@ -4640,11 +4640,11 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="221">
@@ -4655,11 +4655,11 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="222">
@@ -4670,11 +4670,11 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="223">
@@ -4685,11 +4685,11 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="224">
@@ -4700,11 +4700,11 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="225">
@@ -4715,11 +4715,11 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="226">
@@ -4730,11 +4730,11 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="227">
@@ -4745,11 +4745,11 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="228">
@@ -4760,11 +4760,11 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="229">
@@ -4775,11 +4775,11 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="230">
@@ -4790,11 +4790,11 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="231">
@@ -4805,11 +4805,11 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="232">
@@ -4820,11 +4820,11 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="233">
@@ -4835,11 +4835,11 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="234">
@@ -4850,11 +4850,11 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="235">
@@ -4865,11 +4865,11 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>2415</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="236">
@@ -4880,11 +4880,11 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>1655</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="237">
@@ -4895,11 +4895,11 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="238">
@@ -4910,11 +4910,11 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>1651</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="239">
@@ -4925,11 +4925,11 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1648</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="240">
@@ -4940,11 +4940,11 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>1558</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="241">
@@ -4955,11 +4955,11 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>2428</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="242">
@@ -4970,11 +4970,11 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2425</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="243">
@@ -4985,11 +4985,11 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>2432</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="244">
@@ -5000,11 +5000,11 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1581</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="245">
@@ -5015,11 +5015,11 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>1574</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="246">
@@ -5030,11 +5030,11 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>1579</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="247">
@@ -5045,11 +5045,11 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>1593</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="248">
@@ -5060,11 +5060,11 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>1596</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="249">
@@ -5075,11 +5075,11 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>1596</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="250">
@@ -5090,11 +5090,11 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C250" t="n">
-        <v>1596</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="251">
@@ -5105,11 +5105,11 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C251" t="n">
-        <v>1596</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="252">
@@ -5120,11 +5120,11 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C252" t="n">
-        <v>2453</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="253">
@@ -5135,7 +5135,7 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C253" t="n">
@@ -5145,76 +5145,76 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C254" t="n">
-        <v>1692</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C255" t="n">
-        <v>1690</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C256" t="n">
-        <v>1695</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C257" t="n">
-        <v>1706</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C258" t="n">
-        <v>1709</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="259">
@@ -5225,11 +5225,11 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C259" t="n">
-        <v>1710</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="260">
@@ -5240,11 +5240,11 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C260" t="n">
-        <v>1710</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="261">
@@ -5255,11 +5255,11 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C261" t="n">
-        <v>1710</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="262">
@@ -5270,101 +5270,101 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C262" t="n">
-        <v>1709</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C263" t="n">
-        <v>2704</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C264" t="n">
-        <v>2718</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C265" t="n">
-        <v>2705</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C266" t="n">
-        <v>2705</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C267" t="n">
-        <v>2706</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C268" t="n">
-        <v>2706</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="269">
@@ -5375,11 +5375,11 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C269" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="270">
@@ -5390,11 +5390,11 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C270" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="271">
@@ -5405,11 +5405,11 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C271" t="n">
-        <v>2704</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="272">
@@ -5420,11 +5420,11 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C272" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="273">
@@ -5435,11 +5435,11 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C273" t="n">
-        <v>2879</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="274">
@@ -5450,11 +5450,11 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C274" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="275">
@@ -5465,11 +5465,11 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C275" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="276">
@@ -5480,11 +5480,11 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C276" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="277">
@@ -5495,11 +5495,11 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C277" t="n">
-        <v>2940</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="278">
@@ -5510,11 +5510,11 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C278" t="n">
-        <v>2983</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="279">
@@ -5525,11 +5525,11 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C279" t="n">
-        <v>2979</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="280">
@@ -5540,11 +5540,11 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C280" t="n">
-        <v>2781</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="281">
@@ -5555,11 +5555,11 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C281" t="n">
-        <v>2778</v>
+        <v>2843</v>
       </c>
     </row>
     <row r="282">
@@ -5570,11 +5570,11 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C282" t="n">
-        <v>2766</v>
+        <v>2835</v>
       </c>
     </row>
     <row r="283">
@@ -5585,10 +5585,100 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C283" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C284" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C285" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C286" t="n">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>04/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C287" t="n">
+        <v>2778</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>04/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C288" t="n">
+        <v>2766</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
           <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C283" t="n">
+      <c r="C289" t="n">
         <v>2774</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-06-07 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1596</v>
+        <v>1682</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -548,7 +548,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1868</v>
+        <v>1867</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>4599</v>
+        <v>4597</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -800,7 +800,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1596</v>
+        <v>1682</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -932,7 +932,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1705</v>
+        <v>1704</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -974,7 +974,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1868</v>
+        <v>1867</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1085,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2013</v>
+        <v>2012</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>4599</v>
+        <v>4597</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C289"/>
+  <dimension ref="A1:C295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3000,16 +3000,16 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>228</v>
+        <v>1867</v>
       </c>
     </row>
     <row r="112">
@@ -3020,11 +3020,11 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="113">
@@ -3035,7 +3035,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -3080,7 +3080,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -3095,11 +3095,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="118">
@@ -3110,11 +3110,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="119">
@@ -3125,11 +3125,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1334</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="120">
@@ -3140,11 +3140,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1345</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="121">
@@ -3155,11 +3155,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="122">
@@ -3170,11 +3170,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="123">
@@ -3185,11 +3185,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="124">
@@ -3200,11 +3200,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="125">
@@ -3215,11 +3215,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1337</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="126">
@@ -3230,11 +3230,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="127">
@@ -3245,11 +3245,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="128">
@@ -3260,7 +3260,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -3335,11 +3335,11 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="134">
@@ -3350,11 +3350,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="135">
@@ -3365,11 +3365,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="136">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -3395,11 +3395,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="138">
@@ -3410,11 +3410,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="139">
@@ -3425,11 +3425,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1329</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="140">
@@ -3440,11 +3440,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1324</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="141">
@@ -3455,11 +3455,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1344</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="142">
@@ -3470,11 +3470,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1342</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="143">
@@ -3485,11 +3485,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1346</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="144">
@@ -3500,11 +3500,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="145">
@@ -3515,11 +3515,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1339</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="146">
@@ -3530,11 +3530,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>1343</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="147">
@@ -3545,11 +3545,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>2009</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="148">
@@ -3560,11 +3560,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2013</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="149">
@@ -3575,7 +3575,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -3645,46 +3645,46 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
-        <v>3471</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>404</v>
+        <v>2012</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2353</v>
+        <v>3471</v>
       </c>
     </row>
     <row r="157">
@@ -3695,11 +3695,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="158">
@@ -3710,7 +3710,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
@@ -3725,7 +3725,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
@@ -3740,11 +3740,11 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="161">
@@ -3755,11 +3755,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="162">
@@ -3770,11 +3770,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2367</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="163">
@@ -3785,11 +3785,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2238</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="164">
@@ -3800,11 +3800,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2257</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="165">
@@ -3815,11 +3815,11 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2196</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="166">
@@ -3830,11 +3830,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2185</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="167">
@@ -3845,11 +3845,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2189</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="168">
@@ -3860,11 +3860,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2191</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="169">
@@ -3875,11 +3875,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2185</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="170">
@@ -3890,11 +3890,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2196</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="171">
@@ -3905,11 +3905,11 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="172">
@@ -3920,11 +3920,11 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="173">
@@ -3935,7 +3935,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
@@ -3950,7 +3950,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
@@ -3965,7 +3965,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -3980,7 +3980,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -3995,11 +3995,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="178">
@@ -4010,11 +4010,11 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="179">
@@ -4025,11 +4025,11 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="180">
@@ -4040,11 +4040,11 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>2182</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="181">
@@ -4055,11 +4055,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>1675</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="182">
@@ -4070,11 +4070,11 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>1674</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="183">
@@ -4085,11 +4085,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>1670</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="184">
@@ -4100,11 +4100,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1664</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="185">
@@ -4115,11 +4115,11 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1688</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="186">
@@ -4130,11 +4130,11 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>1686</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="187">
@@ -4145,11 +4145,11 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1691</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="188">
@@ -4160,11 +4160,11 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>1689</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="189">
@@ -4175,11 +4175,11 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>1682</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="190">
@@ -4190,11 +4190,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1687</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="191">
@@ -4205,11 +4205,11 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1702</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="192">
@@ -4220,11 +4220,11 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>1705</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="193">
@@ -4235,11 +4235,11 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1706</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="194">
@@ -4250,11 +4250,11 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1706</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="195">
@@ -4265,7 +4265,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
@@ -4280,11 +4280,11 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>2632</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="197">
@@ -4295,11 +4295,11 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>1705</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="198">
@@ -4310,56 +4310,56 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>1705</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>2848</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>2842</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>2831</v>
+        <v>1704</v>
       </c>
     </row>
     <row r="202">
@@ -4370,11 +4370,11 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>2872</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="203">
@@ -4385,11 +4385,11 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>4547</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="204">
@@ -4400,11 +4400,11 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>4561</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="205">
@@ -4415,11 +4415,11 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>4557</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="206">
@@ -4430,11 +4430,11 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>4537</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="207">
@@ -4445,11 +4445,11 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>4550</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="208">
@@ -4460,11 +4460,11 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>4590</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="209">
@@ -4475,11 +4475,11 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>4600</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="210">
@@ -4490,11 +4490,11 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>4600</v>
+        <v>4550</v>
       </c>
     </row>
     <row r="211">
@@ -4505,11 +4505,11 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>4600</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="212">
@@ -4520,7 +4520,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
@@ -4535,11 +4535,11 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>3407</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="214">
@@ -4550,71 +4550,71 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>4599</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>410</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>2391</v>
+        <v>3407</v>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>2391</v>
+        <v>4599</v>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>2391</v>
+        <v>4597</v>
       </c>
     </row>
     <row r="219">
@@ -4625,11 +4625,11 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="220">
@@ -4640,11 +4640,11 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="221">
@@ -4655,11 +4655,11 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="222">
@@ -4670,11 +4670,11 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="223">
@@ -4685,11 +4685,11 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="224">
@@ -4700,11 +4700,11 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="225">
@@ -4715,11 +4715,11 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="226">
@@ -4730,11 +4730,11 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="227">
@@ -4745,11 +4745,11 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="228">
@@ -4760,11 +4760,11 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="229">
@@ -4775,11 +4775,11 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="230">
@@ -4790,11 +4790,11 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="231">
@@ -4805,11 +4805,11 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="232">
@@ -4820,11 +4820,11 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="233">
@@ -4835,11 +4835,11 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="234">
@@ -4850,11 +4850,11 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="235">
@@ -4865,11 +4865,11 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="236">
@@ -4880,11 +4880,11 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="237">
@@ -4895,11 +4895,11 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="238">
@@ -4910,11 +4910,11 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="239">
@@ -4925,11 +4925,11 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>2415</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="240">
@@ -4940,11 +4940,11 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>1655</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="241">
@@ -4955,11 +4955,11 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="242">
@@ -4970,11 +4970,11 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>1651</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="243">
@@ -4985,11 +4985,11 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>1648</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="244">
@@ -5000,11 +5000,11 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1558</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="245">
@@ -5015,11 +5015,11 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>2428</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="246">
@@ -5030,11 +5030,11 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>2425</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="247">
@@ -5045,11 +5045,11 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>2432</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="248">
@@ -5060,11 +5060,11 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>1581</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="249">
@@ -5075,11 +5075,11 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>1574</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="250">
@@ -5090,11 +5090,11 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C250" t="n">
-        <v>1579</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="251">
@@ -5105,11 +5105,11 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C251" t="n">
-        <v>1593</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="252">
@@ -5120,11 +5120,11 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C252" t="n">
-        <v>1596</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="253">
@@ -5135,11 +5135,11 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C253" t="n">
-        <v>1596</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="254">
@@ -5150,11 +5150,11 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C254" t="n">
-        <v>1596</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="255">
@@ -5165,11 +5165,11 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C255" t="n">
-        <v>1596</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="256">
@@ -5180,11 +5180,11 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C256" t="n">
-        <v>2453</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="257">
@@ -5195,7 +5195,7 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C257" t="n">
@@ -5210,7 +5210,7 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C258" t="n">
@@ -5220,76 +5220,76 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C259" t="n">
-        <v>1692</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C260" t="n">
-        <v>1690</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C261" t="n">
-        <v>1695</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C262" t="n">
-        <v>1706</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C263" t="n">
-        <v>1709</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="264">
@@ -5300,11 +5300,11 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C264" t="n">
-        <v>1710</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="265">
@@ -5315,11 +5315,11 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C265" t="n">
-        <v>1710</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="266">
@@ -5330,11 +5330,11 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C266" t="n">
-        <v>1710</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="267">
@@ -5345,11 +5345,11 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C267" t="n">
-        <v>1709</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="268">
@@ -5360,7 +5360,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -5370,91 +5370,91 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C269" t="n">
-        <v>2704</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C270" t="n">
-        <v>2718</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C271" t="n">
-        <v>2705</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C272" t="n">
-        <v>2705</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C273" t="n">
-        <v>2706</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C274" t="n">
-        <v>2706</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="275">
@@ -5465,11 +5465,11 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C275" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="276">
@@ -5480,11 +5480,11 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C276" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="277">
@@ -5495,11 +5495,11 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C277" t="n">
-        <v>2704</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="278">
@@ -5510,11 +5510,11 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C278" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="279">
@@ -5525,11 +5525,11 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C279" t="n">
-        <v>2879</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="280">
@@ -5540,11 +5540,11 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C280" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="281">
@@ -5555,11 +5555,11 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C281" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="282">
@@ -5570,11 +5570,11 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C282" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="283">
@@ -5585,11 +5585,11 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C283" t="n">
-        <v>2940</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="284">
@@ -5600,11 +5600,11 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C284" t="n">
-        <v>2983</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="285">
@@ -5615,11 +5615,11 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C285" t="n">
-        <v>2979</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="286">
@@ -5630,11 +5630,11 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C286" t="n">
-        <v>2781</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="287">
@@ -5645,11 +5645,11 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C287" t="n">
-        <v>2778</v>
+        <v>2843</v>
       </c>
     </row>
     <row r="288">
@@ -5660,11 +5660,11 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C288" t="n">
-        <v>2766</v>
+        <v>2835</v>
       </c>
     </row>
     <row r="289">
@@ -5675,10 +5675,100 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C289" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C290" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C291" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C292" t="n">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>04/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C293" t="n">
+        <v>2778</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>04/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C294" t="n">
+        <v>2766</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
           <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C289" t="n">
+      <c r="C295" t="n">
         <v>2774</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-06-08 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -490,31 +490,31 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>London Heathrow</t>
+          <t>Frankfurt</t>
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1682</v>
+        <v>1706</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>26.2</v>
+        <v>15.5</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -524,31 +524,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>FRA</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Frankfurt</t>
-        </is>
-      </c>
+          <t>MUC</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
-        <v>1704</v>
+        <v>1710</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>15.5</v>
+        <v>13.8</v>
       </c>
       <c r="G3" t="n">
         <v>2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -558,27 +554,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MUC</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr"/>
+          <t>CPH</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Copenhagen</t>
+        </is>
+      </c>
       <c r="D4" t="n">
-        <v>1709</v>
+        <v>1868</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Lufthansa</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>13.8</v>
+        <v>15.6</v>
       </c>
       <c r="G4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -588,31 +588,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CPH</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>Copenhagen</t>
-        </is>
-      </c>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
-        <v>1867</v>
+        <v>2323</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>15.6</v>
+        <v>2.6</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -622,27 +618,31 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>DIRECT</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr"/>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>London Heathrow</t>
+        </is>
+      </c>
       <c r="D6" t="n">
-        <v>2012</v>
+        <v>2453</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>2.6</v>
+        <v>14.2</v>
       </c>
       <c r="G6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -785,7 +785,7 @@
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>4597</v>
+        <v>4601</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -800,7 +800,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -907,7 +907,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -917,22 +917,22 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1682</v>
+        <v>1706</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Lufthansa + Austrian</t>
         </is>
       </c>
       <c r="H2" t="n">
-        <v>26.2</v>
+        <v>15.5</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -949,7 +949,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -959,22 +959,22 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1704</v>
+        <v>1710</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Lufthansa + Austrian</t>
+          <t>Lufthansa</t>
         </is>
       </c>
       <c r="H3" t="n">
-        <v>15.5</v>
+        <v>13.8</v>
       </c>
       <c r="I3" t="n">
         <v>2</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -991,7 +991,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1001,22 +1001,22 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1709</v>
+        <v>1868</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Lufthansa</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H4" t="n">
-        <v>13.8</v>
+        <v>15.6</v>
       </c>
       <c r="I4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>CPH</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1867</v>
+        <v>2323</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>15.6</v>
+        <v>2.6</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1085,22 +1085,22 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2012</v>
+        <v>2453</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>2.6</v>
+        <v>14.2</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1295,7 +1295,7 @@
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>4597</v>
+        <v>4601</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -1310,7 +1310,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C295"/>
+  <dimension ref="A1:C301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3015,16 +3015,16 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>228</v>
+        <v>1868</v>
       </c>
     </row>
     <row r="113">
@@ -3035,11 +3035,11 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="114">
@@ -3050,7 +3050,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
@@ -3080,7 +3080,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -3110,11 +3110,11 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="119">
@@ -3125,11 +3125,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="120">
@@ -3140,11 +3140,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1334</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="121">
@@ -3155,11 +3155,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1345</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="122">
@@ -3170,11 +3170,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="123">
@@ -3185,11 +3185,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="124">
@@ -3200,11 +3200,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="125">
@@ -3215,11 +3215,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="126">
@@ -3230,11 +3230,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1337</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="127">
@@ -3245,11 +3245,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="128">
@@ -3260,11 +3260,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="129">
@@ -3275,7 +3275,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -3350,11 +3350,11 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="135">
@@ -3365,11 +3365,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="136">
@@ -3380,11 +3380,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="137">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
@@ -3410,11 +3410,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="139">
@@ -3425,11 +3425,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="140">
@@ -3440,11 +3440,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1329</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="141">
@@ -3455,11 +3455,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1324</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="142">
@@ -3470,11 +3470,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1344</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="143">
@@ -3485,11 +3485,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1342</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="144">
@@ -3500,11 +3500,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1346</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="145">
@@ -3515,11 +3515,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="146">
@@ -3530,11 +3530,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>1339</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="147">
@@ -3545,11 +3545,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>1343</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="148">
@@ -3560,11 +3560,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>2009</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="149">
@@ -3575,11 +3575,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>2013</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="150">
@@ -3590,7 +3590,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -3665,56 +3665,56 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>3471</v>
+        <v>2012</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>404</v>
+        <v>2323</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2353</v>
+        <v>3471</v>
       </c>
     </row>
     <row r="159">
@@ -3725,11 +3725,11 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="160">
@@ -3740,7 +3740,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
@@ -3755,7 +3755,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
@@ -3770,11 +3770,11 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="163">
@@ -3785,11 +3785,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="164">
@@ -3800,11 +3800,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2367</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="165">
@@ -3815,11 +3815,11 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2238</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="166">
@@ -3830,11 +3830,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2257</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="167">
@@ -3845,11 +3845,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2196</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="168">
@@ -3860,11 +3860,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2185</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="169">
@@ -3875,11 +3875,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2189</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="170">
@@ -3890,11 +3890,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2191</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="171">
@@ -3905,11 +3905,11 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>2185</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="172">
@@ -3920,11 +3920,11 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>2196</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="173">
@@ -3935,11 +3935,11 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="174">
@@ -3950,11 +3950,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="175">
@@ -3965,7 +3965,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
@@ -3980,7 +3980,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -4025,11 +4025,11 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="180">
@@ -4040,11 +4040,11 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="181">
@@ -4055,11 +4055,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="182">
@@ -4070,11 +4070,11 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>2182</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="183">
@@ -4085,11 +4085,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>1675</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="184">
@@ -4100,11 +4100,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1674</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="185">
@@ -4115,11 +4115,11 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1670</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="186">
@@ -4130,11 +4130,11 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>1664</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="187">
@@ -4145,11 +4145,11 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1688</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="188">
@@ -4160,11 +4160,11 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>1686</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="189">
@@ -4175,11 +4175,11 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>1691</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="190">
@@ -4190,11 +4190,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1689</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="191">
@@ -4205,11 +4205,11 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1682</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="192">
@@ -4220,11 +4220,11 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>1687</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="193">
@@ -4235,11 +4235,11 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1702</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="194">
@@ -4250,11 +4250,11 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1705</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="195">
@@ -4265,11 +4265,11 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1706</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="196">
@@ -4280,11 +4280,11 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>1706</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="197">
@@ -4295,7 +4295,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
@@ -4310,11 +4310,11 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>2632</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="199">
@@ -4325,11 +4325,11 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>1705</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="200">
@@ -4340,11 +4340,11 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>1705</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="201">
@@ -4355,56 +4355,56 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>1704</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>2848</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>2842</v>
+        <v>1704</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>2831</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="205">
@@ -4415,11 +4415,11 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>2872</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="206">
@@ -4430,11 +4430,11 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>4547</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="207">
@@ -4445,11 +4445,11 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>4561</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="208">
@@ -4460,11 +4460,11 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>4557</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="209">
@@ -4475,11 +4475,11 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>4537</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="210">
@@ -4490,11 +4490,11 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>4550</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="211">
@@ -4505,11 +4505,11 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>4590</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="212">
@@ -4520,11 +4520,11 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>4600</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="213">
@@ -4535,11 +4535,11 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>4600</v>
+        <v>4550</v>
       </c>
     </row>
     <row r="214">
@@ -4550,11 +4550,11 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>4600</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="215">
@@ -4565,7 +4565,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
@@ -4580,11 +4580,11 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>3407</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="217">
@@ -4595,11 +4595,11 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>4599</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="218">
@@ -4610,71 +4610,71 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>4597</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>410</v>
+        <v>3407</v>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>2391</v>
+        <v>4599</v>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>2391</v>
+        <v>4597</v>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>2391</v>
+        <v>4601</v>
       </c>
     </row>
     <row r="223">
@@ -4685,11 +4685,11 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="224">
@@ -4700,11 +4700,11 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="225">
@@ -4715,11 +4715,11 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="226">
@@ -4730,11 +4730,11 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="227">
@@ -4745,11 +4745,11 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="228">
@@ -4760,11 +4760,11 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="229">
@@ -4775,11 +4775,11 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="230">
@@ -4790,11 +4790,11 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="231">
@@ -4805,11 +4805,11 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="232">
@@ -4820,11 +4820,11 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="233">
@@ -4835,11 +4835,11 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="234">
@@ -4850,11 +4850,11 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="235">
@@ -4865,11 +4865,11 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="236">
@@ -4880,11 +4880,11 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="237">
@@ -4895,11 +4895,11 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="238">
@@ -4910,11 +4910,11 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="239">
@@ -4925,11 +4925,11 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="240">
@@ -4940,11 +4940,11 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="241">
@@ -4955,11 +4955,11 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="242">
@@ -4970,11 +4970,11 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="243">
@@ -4985,11 +4985,11 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>2415</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="244">
@@ -5000,11 +5000,11 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1655</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="245">
@@ -5015,11 +5015,11 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="246">
@@ -5030,11 +5030,11 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>1651</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="247">
@@ -5045,11 +5045,11 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>1648</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="248">
@@ -5060,11 +5060,11 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>1558</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="249">
@@ -5075,11 +5075,11 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>2428</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="250">
@@ -5090,11 +5090,11 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C250" t="n">
-        <v>2425</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="251">
@@ -5105,11 +5105,11 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C251" t="n">
-        <v>2432</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="252">
@@ -5120,11 +5120,11 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C252" t="n">
-        <v>1581</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="253">
@@ -5135,11 +5135,11 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C253" t="n">
-        <v>1574</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="254">
@@ -5150,11 +5150,11 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C254" t="n">
-        <v>1579</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="255">
@@ -5165,11 +5165,11 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C255" t="n">
-        <v>1593</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="256">
@@ -5180,11 +5180,11 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C256" t="n">
-        <v>1596</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="257">
@@ -5195,11 +5195,11 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C257" t="n">
-        <v>1596</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="258">
@@ -5210,11 +5210,11 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C258" t="n">
-        <v>1596</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="259">
@@ -5225,11 +5225,11 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C259" t="n">
-        <v>1596</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="260">
@@ -5240,11 +5240,11 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C260" t="n">
-        <v>2453</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="261">
@@ -5255,7 +5255,7 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C261" t="n">
@@ -5270,7 +5270,7 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C262" t="n">
@@ -5285,86 +5285,86 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C263" t="n">
-        <v>1682</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C264" t="n">
-        <v>1692</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C265" t="n">
-        <v>1690</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C266" t="n">
-        <v>1695</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C267" t="n">
-        <v>1706</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C268" t="n">
-        <v>1709</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="269">
@@ -5375,11 +5375,11 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C269" t="n">
-        <v>1710</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="270">
@@ -5390,11 +5390,11 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C270" t="n">
-        <v>1710</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="271">
@@ -5405,11 +5405,11 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C271" t="n">
-        <v>1710</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="272">
@@ -5420,11 +5420,11 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C272" t="n">
-        <v>1709</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="273">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C273" t="n">
@@ -5450,101 +5450,101 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C274" t="n">
-        <v>1709</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C275" t="n">
-        <v>2704</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C276" t="n">
-        <v>2718</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C277" t="n">
-        <v>2705</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C278" t="n">
-        <v>2705</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C279" t="n">
-        <v>2706</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C280" t="n">
-        <v>2706</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="281">
@@ -5555,11 +5555,11 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C281" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="282">
@@ -5570,11 +5570,11 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C282" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="283">
@@ -5585,11 +5585,11 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C283" t="n">
-        <v>2704</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="284">
@@ -5600,11 +5600,11 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C284" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="285">
@@ -5615,11 +5615,11 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C285" t="n">
-        <v>2879</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="286">
@@ -5630,11 +5630,11 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C286" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="287">
@@ -5645,11 +5645,11 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C287" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="288">
@@ -5660,11 +5660,11 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C288" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="289">
@@ -5675,11 +5675,11 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C289" t="n">
-        <v>2940</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="290">
@@ -5690,11 +5690,11 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C290" t="n">
-        <v>2983</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="291">
@@ -5705,11 +5705,11 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C291" t="n">
-        <v>2979</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="292">
@@ -5720,11 +5720,11 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C292" t="n">
-        <v>2781</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="293">
@@ -5735,11 +5735,11 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C293" t="n">
-        <v>2778</v>
+        <v>2843</v>
       </c>
     </row>
     <row r="294">
@@ -5750,11 +5750,11 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C294" t="n">
-        <v>2766</v>
+        <v>2835</v>
       </c>
     </row>
     <row r="295">
@@ -5765,10 +5765,100 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C295" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C296" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C297" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C298" t="n">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>04/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C299" t="n">
+        <v>2778</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>04/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C300" t="n">
+        <v>2766</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
           <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C295" t="n">
+      <c r="C301" t="n">
         <v>2774</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-06-08 23:19 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1706</v>
+        <v>1718</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
-        <v>1710</v>
+        <v>1722</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1868</v>
+        <v>1881</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -593,7 +593,7 @@
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
-        <v>2323</v>
+        <v>2340</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -608,7 +608,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>2453</v>
+        <v>2470</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -750,27 +750,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>3471</v>
+        <v>3432</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>9.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="G10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -780,27 +780,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>4601</v>
+        <v>3471</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>7.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1706</v>
+        <v>1718</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -932,7 +932,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1710</v>
+        <v>1722</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -974,7 +974,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1868</v>
+        <v>1881</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2323</v>
+        <v>2340</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1085,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2453</v>
+        <v>2470</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1253,22 +1253,22 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>3471</v>
+        <v>3432</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>9.199999999999999</v>
+        <v>7.8</v>
       </c>
       <c r="I10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1285,7 +1285,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1295,22 +1295,22 @@
       </c>
       <c r="E11" t="inlineStr"/>
       <c r="F11" t="n">
-        <v>4601</v>
+        <v>3471</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>Eurowings + Lufthansa City Airlines + Lufthansa</t>
         </is>
       </c>
       <c r="H11" t="n">
-        <v>7.8</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="I11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C301"/>
+  <dimension ref="A1:C307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3030,16 +3030,16 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C113" t="n">
-        <v>228</v>
+        <v>1881</v>
       </c>
     </row>
     <row r="114">
@@ -3050,11 +3050,11 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="115">
@@ -3065,7 +3065,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -3125,11 +3125,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="120">
@@ -3140,11 +3140,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="121">
@@ -3155,11 +3155,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1334</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="122">
@@ -3170,11 +3170,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1345</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="123">
@@ -3185,11 +3185,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="124">
@@ -3200,11 +3200,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="125">
@@ -3215,11 +3215,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="126">
@@ -3230,11 +3230,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="127">
@@ -3245,11 +3245,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1337</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="128">
@@ -3260,11 +3260,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="129">
@@ -3275,11 +3275,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="130">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -3365,11 +3365,11 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="136">
@@ -3380,11 +3380,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="137">
@@ -3395,11 +3395,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="138">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
@@ -3425,11 +3425,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="140">
@@ -3440,11 +3440,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="141">
@@ -3455,11 +3455,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1329</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="142">
@@ -3470,11 +3470,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1324</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="143">
@@ -3485,11 +3485,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1344</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="144">
@@ -3500,11 +3500,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1342</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="145">
@@ -3515,11 +3515,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1346</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="146">
@@ -3530,11 +3530,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="147">
@@ -3545,11 +3545,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>1339</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="148">
@@ -3560,11 +3560,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>1343</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="149">
@@ -3575,11 +3575,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>2009</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="150">
@@ -3590,11 +3590,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2013</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="151">
@@ -3605,7 +3605,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -3680,11 +3680,11 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="157">
@@ -3695,56 +3695,56 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2323</v>
+        <v>2012</v>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>3471</v>
+        <v>2323</v>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>404</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>2353</v>
+        <v>3471</v>
       </c>
     </row>
     <row r="161">
@@ -3755,11 +3755,11 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="162">
@@ -3770,7 +3770,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
@@ -3785,7 +3785,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
@@ -3800,11 +3800,11 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="165">
@@ -3815,11 +3815,11 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="166">
@@ -3830,11 +3830,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2367</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="167">
@@ -3845,11 +3845,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2238</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="168">
@@ -3860,11 +3860,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2257</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="169">
@@ -3875,11 +3875,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2196</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="170">
@@ -3890,11 +3890,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2185</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="171">
@@ -3905,11 +3905,11 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>2189</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="172">
@@ -3920,11 +3920,11 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>2191</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="173">
@@ -3935,11 +3935,11 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>2185</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="174">
@@ -3950,11 +3950,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>2196</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="175">
@@ -3965,11 +3965,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="176">
@@ -3980,11 +3980,11 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="177">
@@ -3995,7 +3995,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
@@ -4010,7 +4010,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -4055,11 +4055,11 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="182">
@@ -4070,11 +4070,11 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="183">
@@ -4085,11 +4085,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="184">
@@ -4100,11 +4100,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>2182</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="185">
@@ -4115,11 +4115,11 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1675</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="186">
@@ -4130,11 +4130,11 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>1674</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="187">
@@ -4145,11 +4145,11 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1670</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="188">
@@ -4160,11 +4160,11 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>1664</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="189">
@@ -4175,11 +4175,11 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>1688</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="190">
@@ -4190,11 +4190,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1686</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="191">
@@ -4205,11 +4205,11 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1691</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="192">
@@ -4220,11 +4220,11 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>1689</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="193">
@@ -4235,11 +4235,11 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1682</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="194">
@@ -4250,11 +4250,11 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1687</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="195">
@@ -4265,11 +4265,11 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1702</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="196">
@@ -4280,11 +4280,11 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>1705</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="197">
@@ -4295,11 +4295,11 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>1706</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="198">
@@ -4310,11 +4310,11 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>1706</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="199">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
@@ -4340,11 +4340,11 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>2632</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="201">
@@ -4355,11 +4355,11 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
-        <v>1705</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="202">
@@ -4370,11 +4370,11 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>1705</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="203">
@@ -4385,11 +4385,11 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>1704</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="204">
@@ -4400,56 +4400,56 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>1706</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>2848</v>
+        <v>1704</v>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>2842</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>2831</v>
+        <v>1718</v>
       </c>
     </row>
     <row r="208">
@@ -4460,11 +4460,11 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2872</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="209">
@@ -4475,11 +4475,11 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>4547</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="210">
@@ -4490,11 +4490,11 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>4561</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="211">
@@ -4505,11 +4505,11 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>4557</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="212">
@@ -4520,11 +4520,11 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>4537</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="213">
@@ -4535,11 +4535,11 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>4550</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="214">
@@ -4550,11 +4550,11 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>4590</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="215">
@@ -4565,11 +4565,11 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>4600</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="216">
@@ -4580,11 +4580,11 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>4600</v>
+        <v>4550</v>
       </c>
     </row>
     <row r="217">
@@ -4595,11 +4595,11 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>4600</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="218">
@@ -4610,7 +4610,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
@@ -4625,11 +4625,11 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>3407</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="220">
@@ -4640,11 +4640,11 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>4599</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="221">
@@ -4655,11 +4655,11 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C221" t="n">
-        <v>4597</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="222">
@@ -4670,71 +4670,71 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>4601</v>
+        <v>3407</v>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>410</v>
+        <v>4599</v>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>2391</v>
+        <v>4597</v>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>2391</v>
+        <v>4601</v>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>2391</v>
+        <v>3432</v>
       </c>
     </row>
     <row r="227">
@@ -4745,11 +4745,11 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="228">
@@ -4760,11 +4760,11 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="229">
@@ -4775,11 +4775,11 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="230">
@@ -4790,11 +4790,11 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="231">
@@ -4805,11 +4805,11 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="232">
@@ -4820,11 +4820,11 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="233">
@@ -4835,11 +4835,11 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="234">
@@ -4850,11 +4850,11 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="235">
@@ -4865,11 +4865,11 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="236">
@@ -4880,11 +4880,11 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="237">
@@ -4895,11 +4895,11 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="238">
@@ -4910,11 +4910,11 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="239">
@@ -4925,11 +4925,11 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="240">
@@ -4940,11 +4940,11 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="241">
@@ -4955,11 +4955,11 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="242">
@@ -4970,11 +4970,11 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="243">
@@ -4985,11 +4985,11 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="244">
@@ -5000,11 +5000,11 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="245">
@@ -5015,11 +5015,11 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="246">
@@ -5030,11 +5030,11 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="247">
@@ -5045,11 +5045,11 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>2415</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="248">
@@ -5060,11 +5060,11 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>1655</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="249">
@@ -5075,11 +5075,11 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="250">
@@ -5090,11 +5090,11 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C250" t="n">
-        <v>1651</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="251">
@@ -5105,11 +5105,11 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C251" t="n">
-        <v>1648</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="252">
@@ -5120,11 +5120,11 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C252" t="n">
-        <v>1558</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="253">
@@ -5135,11 +5135,11 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C253" t="n">
-        <v>2428</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="254">
@@ -5150,11 +5150,11 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C254" t="n">
-        <v>2425</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="255">
@@ -5165,11 +5165,11 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C255" t="n">
-        <v>2432</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="256">
@@ -5180,11 +5180,11 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C256" t="n">
-        <v>1581</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="257">
@@ -5195,11 +5195,11 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C257" t="n">
-        <v>1574</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="258">
@@ -5210,11 +5210,11 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C258" t="n">
-        <v>1579</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="259">
@@ -5225,11 +5225,11 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C259" t="n">
-        <v>1593</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="260">
@@ -5240,11 +5240,11 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C260" t="n">
-        <v>1596</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="261">
@@ -5255,11 +5255,11 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C261" t="n">
-        <v>1596</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="262">
@@ -5270,11 +5270,11 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C262" t="n">
-        <v>1596</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="263">
@@ -5285,11 +5285,11 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C263" t="n">
-        <v>1596</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="264">
@@ -5300,11 +5300,11 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C264" t="n">
-        <v>2453</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="265">
@@ -5315,7 +5315,7 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C265" t="n">
@@ -5330,7 +5330,7 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C266" t="n">
@@ -5345,11 +5345,11 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C267" t="n">
-        <v>1682</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="268">
@@ -5360,7 +5360,7 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C268" t="n">
@@ -5370,76 +5370,76 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C269" t="n">
-        <v>1692</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C270" t="n">
-        <v>1690</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C271" t="n">
-        <v>1695</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C272" t="n">
-        <v>1706</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C273" t="n">
-        <v>1709</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="274">
@@ -5450,11 +5450,11 @@
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C274" t="n">
-        <v>1710</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="275">
@@ -5465,11 +5465,11 @@
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C275" t="n">
-        <v>1710</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="276">
@@ -5480,11 +5480,11 @@
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C276" t="n">
-        <v>1710</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="277">
@@ -5495,11 +5495,11 @@
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C277" t="n">
-        <v>1709</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="278">
@@ -5510,7 +5510,7 @@
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C278" t="n">
@@ -5525,11 +5525,11 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C279" t="n">
-        <v>1709</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="280">
@@ -5540,7 +5540,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C280" t="n">
@@ -5550,91 +5550,91 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C281" t="n">
-        <v>2704</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C282" t="n">
-        <v>2718</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C283" t="n">
-        <v>2705</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C284" t="n">
-        <v>2705</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C285" t="n">
-        <v>2706</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C286" t="n">
-        <v>2706</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="287">
@@ -5645,11 +5645,11 @@
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C287" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="288">
@@ -5660,11 +5660,11 @@
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C288" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="289">
@@ -5675,11 +5675,11 @@
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C289" t="n">
-        <v>2704</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="290">
@@ -5690,11 +5690,11 @@
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C290" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="291">
@@ -5705,11 +5705,11 @@
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C291" t="n">
-        <v>2879</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="292">
@@ -5720,11 +5720,11 @@
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C292" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="293">
@@ -5735,11 +5735,11 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C293" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="294">
@@ -5750,11 +5750,11 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C294" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="295">
@@ -5765,11 +5765,11 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C295" t="n">
-        <v>2940</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="296">
@@ -5780,11 +5780,11 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C296" t="n">
-        <v>2983</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="297">
@@ -5795,11 +5795,11 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C297" t="n">
-        <v>2979</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="298">
@@ -5810,11 +5810,11 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C298" t="n">
-        <v>2781</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="299">
@@ -5825,11 +5825,11 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C299" t="n">
-        <v>2778</v>
+        <v>2843</v>
       </c>
     </row>
     <row r="300">
@@ -5840,11 +5840,11 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C300" t="n">
-        <v>2766</v>
+        <v>2835</v>
       </c>
     </row>
     <row r="301">
@@ -5855,10 +5855,100 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C301" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C302" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C303" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C304" t="n">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>04/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C305" t="n">
+        <v>2778</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>04/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C306" t="n">
+        <v>2766</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
           <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C301" t="n">
+      <c r="C307" t="n">
         <v>2774</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-06-09 11:17 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
-        <v>1722</v>
+        <v>1724</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1881</v>
+        <v>1883</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -588,27 +588,31 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>DIRECT</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr"/>
+          <t>LHR</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>London Heathrow</t>
+        </is>
+      </c>
       <c r="D5" t="n">
-        <v>2340</v>
+        <v>1951</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2.6</v>
+        <v>26.2</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -618,31 +622,27 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>LHR</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>London Heathrow</t>
-        </is>
-      </c>
+          <t>DIRECT</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>2470</v>
+        <v>2342</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>14.2</v>
+        <v>2.6</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="n">
-        <v>3432</v>
+        <v>3436</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -770,7 +770,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1718</v>
+        <v>1719</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -932,7 +932,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1722</v>
+        <v>1724</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -974,7 +974,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1881</v>
+        <v>1883</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1033,7 +1033,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1043,22 +1043,22 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>2340</v>
+        <v>1951</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Icelandair</t>
+          <t>British Airways</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>2.6</v>
+        <v>26.2</v>
       </c>
       <c r="I5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1075,7 +1075,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1085,22 +1085,22 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2470</v>
+        <v>2342</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>British Airways</t>
+          <t>Icelandair</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>14.2</v>
+        <v>2.6</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1253,7 +1253,7 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>3432</v>
+        <v>3436</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -1268,7 +1268,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C307"/>
+  <dimension ref="A1:C313"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3045,16 +3045,16 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>228</v>
+        <v>1883</v>
       </c>
     </row>
     <row r="115">
@@ -3065,11 +3065,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="116">
@@ -3080,7 +3080,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
@@ -3110,7 +3110,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C118" t="n">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -3140,11 +3140,11 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="121">
@@ -3155,11 +3155,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="122">
@@ -3170,11 +3170,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1334</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="123">
@@ -3185,11 +3185,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1345</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="124">
@@ -3200,11 +3200,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="125">
@@ -3215,11 +3215,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="126">
@@ -3230,11 +3230,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="127">
@@ -3245,11 +3245,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="128">
@@ -3260,11 +3260,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1337</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="129">
@@ -3275,11 +3275,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="130">
@@ -3290,11 +3290,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="131">
@@ -3305,7 +3305,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -3380,11 +3380,11 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="137">
@@ -3395,11 +3395,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="138">
@@ -3410,11 +3410,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="139">
@@ -3425,7 +3425,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
@@ -3440,11 +3440,11 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="141">
@@ -3455,11 +3455,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="142">
@@ -3470,11 +3470,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1329</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="143">
@@ -3485,11 +3485,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1324</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="144">
@@ -3500,11 +3500,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1344</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="145">
@@ -3515,11 +3515,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1342</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="146">
@@ -3530,11 +3530,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>1346</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="147">
@@ -3545,11 +3545,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C147" t="n">
-        <v>1345</v>
+        <v>1346</v>
       </c>
     </row>
     <row r="148">
@@ -3560,11 +3560,11 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C148" t="n">
-        <v>1339</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="149">
@@ -3575,11 +3575,11 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C149" t="n">
-        <v>1343</v>
+        <v>1339</v>
       </c>
     </row>
     <row r="150">
@@ -3590,11 +3590,11 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C150" t="n">
-        <v>2009</v>
+        <v>1343</v>
       </c>
     </row>
     <row r="151">
@@ -3605,11 +3605,11 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C151" t="n">
-        <v>2013</v>
+        <v>2009</v>
       </c>
     </row>
     <row r="152">
@@ -3620,7 +3620,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C152" t="n">
@@ -3635,7 +3635,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C153" t="n">
@@ -3650,7 +3650,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C154" t="n">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C155" t="n">
@@ -3680,7 +3680,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C156" t="n">
@@ -3695,11 +3695,11 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C157" t="n">
-        <v>2012</v>
+        <v>2013</v>
       </c>
     </row>
     <row r="158">
@@ -3710,11 +3710,11 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C158" t="n">
-        <v>2323</v>
+        <v>2012</v>
       </c>
     </row>
     <row r="159">
@@ -3725,56 +3725,56 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C159" t="n">
-        <v>2340</v>
+        <v>2323</v>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>DUS</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C160" t="n">
-        <v>3471</v>
+        <v>2340</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DIRECT</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C161" t="n">
-        <v>404</v>
+        <v>2342</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>FRA</t>
+          <t>DUS</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C162" t="n">
-        <v>2353</v>
+        <v>3471</v>
       </c>
     </row>
     <row r="163">
@@ -3785,11 +3785,11 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C163" t="n">
-        <v>2353</v>
+        <v>404</v>
       </c>
     </row>
     <row r="164">
@@ -3800,7 +3800,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C164" t="n">
@@ -3815,7 +3815,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C165" t="n">
@@ -3830,11 +3830,11 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C166" t="n">
-        <v>2352</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="167">
@@ -3845,11 +3845,11 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C167" t="n">
-        <v>2364</v>
+        <v>2353</v>
       </c>
     </row>
     <row r="168">
@@ -3860,11 +3860,11 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C168" t="n">
-        <v>2367</v>
+        <v>2352</v>
       </c>
     </row>
     <row r="169">
@@ -3875,11 +3875,11 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C169" t="n">
-        <v>2238</v>
+        <v>2364</v>
       </c>
     </row>
     <row r="170">
@@ -3890,11 +3890,11 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C170" t="n">
-        <v>2257</v>
+        <v>2367</v>
       </c>
     </row>
     <row r="171">
@@ -3905,11 +3905,11 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C171" t="n">
-        <v>2196</v>
+        <v>2238</v>
       </c>
     </row>
     <row r="172">
@@ -3920,11 +3920,11 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C172" t="n">
-        <v>2185</v>
+        <v>2257</v>
       </c>
     </row>
     <row r="173">
@@ -3935,11 +3935,11 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C173" t="n">
-        <v>2189</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="174">
@@ -3950,11 +3950,11 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C174" t="n">
-        <v>2191</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="175">
@@ -3965,11 +3965,11 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C175" t="n">
-        <v>2185</v>
+        <v>2189</v>
       </c>
     </row>
     <row r="176">
@@ -3980,11 +3980,11 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C176" t="n">
-        <v>2196</v>
+        <v>2191</v>
       </c>
     </row>
     <row r="177">
@@ -3995,11 +3995,11 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C177" t="n">
-        <v>2186</v>
+        <v>2185</v>
       </c>
     </row>
     <row r="178">
@@ -4010,11 +4010,11 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C178" t="n">
-        <v>2186</v>
+        <v>2196</v>
       </c>
     </row>
     <row r="179">
@@ -4025,7 +4025,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C179" t="n">
@@ -4040,7 +4040,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C180" t="n">
@@ -4055,7 +4055,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C181" t="n">
@@ -4070,7 +4070,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C182" t="n">
@@ -4085,11 +4085,11 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C183" t="n">
-        <v>1680</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="184">
@@ -4100,11 +4100,11 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C184" t="n">
-        <v>1684</v>
+        <v>2186</v>
       </c>
     </row>
     <row r="185">
@@ -4115,11 +4115,11 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C185" t="n">
-        <v>1679</v>
+        <v>1680</v>
       </c>
     </row>
     <row r="186">
@@ -4130,11 +4130,11 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C186" t="n">
-        <v>2182</v>
+        <v>1684</v>
       </c>
     </row>
     <row r="187">
@@ -4145,11 +4145,11 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C187" t="n">
-        <v>1675</v>
+        <v>1679</v>
       </c>
     </row>
     <row r="188">
@@ -4160,11 +4160,11 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C188" t="n">
-        <v>1674</v>
+        <v>2182</v>
       </c>
     </row>
     <row r="189">
@@ -4175,11 +4175,11 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C189" t="n">
-        <v>1670</v>
+        <v>1675</v>
       </c>
     </row>
     <row r="190">
@@ -4190,11 +4190,11 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C190" t="n">
-        <v>1664</v>
+        <v>1674</v>
       </c>
     </row>
     <row r="191">
@@ -4205,11 +4205,11 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C191" t="n">
-        <v>1688</v>
+        <v>1670</v>
       </c>
     </row>
     <row r="192">
@@ -4220,11 +4220,11 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C192" t="n">
-        <v>1686</v>
+        <v>1664</v>
       </c>
     </row>
     <row r="193">
@@ -4235,11 +4235,11 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C193" t="n">
-        <v>1691</v>
+        <v>1688</v>
       </c>
     </row>
     <row r="194">
@@ -4250,11 +4250,11 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C194" t="n">
-        <v>1689</v>
+        <v>1686</v>
       </c>
     </row>
     <row r="195">
@@ -4265,11 +4265,11 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C195" t="n">
-        <v>1682</v>
+        <v>1691</v>
       </c>
     </row>
     <row r="196">
@@ -4280,11 +4280,11 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C196" t="n">
-        <v>1687</v>
+        <v>1689</v>
       </c>
     </row>
     <row r="197">
@@ -4295,11 +4295,11 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C197" t="n">
-        <v>1702</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="198">
@@ -4310,11 +4310,11 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C198" t="n">
-        <v>1705</v>
+        <v>1687</v>
       </c>
     </row>
     <row r="199">
@@ -4325,11 +4325,11 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C199" t="n">
-        <v>1706</v>
+        <v>1702</v>
       </c>
     </row>
     <row r="200">
@@ -4340,11 +4340,11 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C200" t="n">
-        <v>1706</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="201">
@@ -4355,7 +4355,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C201" t="n">
@@ -4370,11 +4370,11 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C202" t="n">
-        <v>2632</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="203">
@@ -4385,11 +4385,11 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C203" t="n">
-        <v>1705</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="204">
@@ -4400,11 +4400,11 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C204" t="n">
-        <v>1705</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="205">
@@ -4415,11 +4415,11 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C205" t="n">
-        <v>1704</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="206">
@@ -4430,11 +4430,11 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C206" t="n">
-        <v>1706</v>
+        <v>1705</v>
       </c>
     </row>
     <row r="207">
@@ -4445,56 +4445,56 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C207" t="n">
-        <v>1718</v>
+        <v>1704</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C208" t="n">
-        <v>2848</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C209" t="n">
-        <v>2842</v>
+        <v>1718</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>FRA</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C210" t="n">
-        <v>2831</v>
+        <v>1719</v>
       </c>
     </row>
     <row r="211">
@@ -4505,11 +4505,11 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C211" t="n">
-        <v>2872</v>
+        <v>2848</v>
       </c>
     </row>
     <row r="212">
@@ -4520,11 +4520,11 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C212" t="n">
-        <v>4547</v>
+        <v>2842</v>
       </c>
     </row>
     <row r="213">
@@ -4535,11 +4535,11 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C213" t="n">
-        <v>4561</v>
+        <v>2831</v>
       </c>
     </row>
     <row r="214">
@@ -4550,11 +4550,11 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C214" t="n">
-        <v>4557</v>
+        <v>2872</v>
       </c>
     </row>
     <row r="215">
@@ -4565,11 +4565,11 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C215" t="n">
-        <v>4537</v>
+        <v>4547</v>
       </c>
     </row>
     <row r="216">
@@ -4580,11 +4580,11 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C216" t="n">
-        <v>4550</v>
+        <v>4561</v>
       </c>
     </row>
     <row r="217">
@@ -4595,11 +4595,11 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C217" t="n">
-        <v>4590</v>
+        <v>4557</v>
       </c>
     </row>
     <row r="218">
@@ -4610,11 +4610,11 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C218" t="n">
-        <v>4600</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="219">
@@ -4625,11 +4625,11 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C219" t="n">
-        <v>4600</v>
+        <v>4550</v>
       </c>
     </row>
     <row r="220">
@@ -4640,11 +4640,11 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C220" t="n">
-        <v>4600</v>
+        <v>4590</v>
       </c>
     </row>
     <row r="221">
@@ -4655,7 +4655,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C221" t="n">
@@ -4670,11 +4670,11 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C222" t="n">
-        <v>3407</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="223">
@@ -4685,11 +4685,11 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C223" t="n">
-        <v>4599</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="224">
@@ -4700,11 +4700,11 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C224" t="n">
-        <v>4597</v>
+        <v>4600</v>
       </c>
     </row>
     <row r="225">
@@ -4715,11 +4715,11 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C225" t="n">
-        <v>4601</v>
+        <v>3407</v>
       </c>
     </row>
     <row r="226">
@@ -4730,71 +4730,71 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C226" t="n">
-        <v>3432</v>
+        <v>4599</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C227" t="n">
-        <v>410</v>
+        <v>4597</v>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C228" t="n">
-        <v>2391</v>
+        <v>4601</v>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C229" t="n">
-        <v>2391</v>
+        <v>3432</v>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>LHR</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C230" t="n">
-        <v>2391</v>
+        <v>3436</v>
       </c>
     </row>
     <row r="231">
@@ -4805,11 +4805,11 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C231" t="n">
-        <v>2391</v>
+        <v>410</v>
       </c>
     </row>
     <row r="232">
@@ -4820,11 +4820,11 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C232" t="n">
-        <v>2389</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="233">
@@ -4835,11 +4835,11 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C233" t="n">
-        <v>2402</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="234">
@@ -4850,11 +4850,11 @@
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C234" t="n">
-        <v>2404</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="235">
@@ -4865,11 +4865,11 @@
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C235" t="n">
-        <v>2399</v>
+        <v>2391</v>
       </c>
     </row>
     <row r="236">
@@ -4880,11 +4880,11 @@
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C236" t="n">
-        <v>2419</v>
+        <v>2389</v>
       </c>
     </row>
     <row r="237">
@@ -4895,11 +4895,11 @@
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C237" t="n">
-        <v>1660</v>
+        <v>2402</v>
       </c>
     </row>
     <row r="238">
@@ -4910,11 +4910,11 @@
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C238" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="239">
@@ -4925,11 +4925,11 @@
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C239" t="n">
-        <v>1655</v>
+        <v>2399</v>
       </c>
     </row>
     <row r="240">
@@ -4940,11 +4940,11 @@
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C240" t="n">
-        <v>2411</v>
+        <v>2419</v>
       </c>
     </row>
     <row r="241">
@@ -4955,11 +4955,11 @@
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C241" t="n">
-        <v>2404</v>
+        <v>1660</v>
       </c>
     </row>
     <row r="242">
@@ -4970,11 +4970,11 @@
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C242" t="n">
-        <v>2416</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="243">
@@ -4985,11 +4985,11 @@
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C243" t="n">
-        <v>2405</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="244">
@@ -5000,11 +5000,11 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>2405</v>
+        <v>2411</v>
       </c>
     </row>
     <row r="245">
@@ -5015,11 +5015,11 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>2406</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="246">
@@ -5030,11 +5030,11 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C246" t="n">
-        <v>2406</v>
+        <v>2416</v>
       </c>
     </row>
     <row r="247">
@@ -5045,11 +5045,11 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C247" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="248">
@@ -5060,11 +5060,11 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C248" t="n">
-        <v>1652</v>
+        <v>2405</v>
       </c>
     </row>
     <row r="249">
@@ -5075,11 +5075,11 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C249" t="n">
-        <v>2404</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="250">
@@ -5090,11 +5090,11 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C250" t="n">
-        <v>2422</v>
+        <v>2406</v>
       </c>
     </row>
     <row r="251">
@@ -5105,11 +5105,11 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C251" t="n">
-        <v>2415</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="252">
@@ -5120,11 +5120,11 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C252" t="n">
-        <v>1655</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="253">
@@ -5135,11 +5135,11 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C253" t="n">
-        <v>1652</v>
+        <v>2404</v>
       </c>
     </row>
     <row r="254">
@@ -5150,11 +5150,11 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C254" t="n">
-        <v>1651</v>
+        <v>2422</v>
       </c>
     </row>
     <row r="255">
@@ -5165,11 +5165,11 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C255" t="n">
-        <v>1648</v>
+        <v>2415</v>
       </c>
     </row>
     <row r="256">
@@ -5180,11 +5180,11 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C256" t="n">
-        <v>1558</v>
+        <v>1655</v>
       </c>
     </row>
     <row r="257">
@@ -5195,11 +5195,11 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C257" t="n">
-        <v>2428</v>
+        <v>1652</v>
       </c>
     </row>
     <row r="258">
@@ -5210,11 +5210,11 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C258" t="n">
-        <v>2425</v>
+        <v>1651</v>
       </c>
     </row>
     <row r="259">
@@ -5225,11 +5225,11 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C259" t="n">
-        <v>2432</v>
+        <v>1648</v>
       </c>
     </row>
     <row r="260">
@@ -5240,11 +5240,11 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C260" t="n">
-        <v>1581</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="261">
@@ -5255,11 +5255,11 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C261" t="n">
-        <v>1574</v>
+        <v>2428</v>
       </c>
     </row>
     <row r="262">
@@ -5270,11 +5270,11 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C262" t="n">
-        <v>1579</v>
+        <v>2425</v>
       </c>
     </row>
     <row r="263">
@@ -5285,11 +5285,11 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C263" t="n">
-        <v>1593</v>
+        <v>2432</v>
       </c>
     </row>
     <row r="264">
@@ -5300,11 +5300,11 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>04/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C264" t="n">
-        <v>1596</v>
+        <v>1581</v>
       </c>
     </row>
     <row r="265">
@@ -5315,11 +5315,11 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C265" t="n">
-        <v>1596</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="266">
@@ -5330,11 +5330,11 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C266" t="n">
-        <v>1596</v>
+        <v>1579</v>
       </c>
     </row>
     <row r="267">
@@ -5345,11 +5345,11 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C267" t="n">
-        <v>1596</v>
+        <v>1593</v>
       </c>
     </row>
     <row r="268">
@@ -5360,11 +5360,11 @@
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C268" t="n">
-        <v>2453</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="269">
@@ -5375,7 +5375,7 @@
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C269" t="n">
@@ -5390,7 +5390,7 @@
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C270" t="n">
@@ -5405,11 +5405,11 @@
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C271" t="n">
-        <v>1682</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="272">
@@ -5420,7 +5420,7 @@
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C272" t="n">
@@ -5435,86 +5435,86 @@
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C273" t="n">
-        <v>2470</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C274" t="n">
-        <v>1692</v>
+        <v>1596</v>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C275" t="n">
-        <v>1690</v>
+        <v>1682</v>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C276" t="n">
-        <v>1695</v>
+        <v>2453</v>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>05/06/2026 14:23 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C277" t="n">
-        <v>1706</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>MUC</t>
+          <t>LHR</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>05/06/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C278" t="n">
-        <v>1709</v>
+        <v>1951</v>
       </c>
     </row>
     <row r="279">
@@ -5525,11 +5525,11 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>06/06/2026 08:17 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C279" t="n">
-        <v>1710</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="280">
@@ -5540,11 +5540,11 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>06/06/2026 14:23 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C280" t="n">
-        <v>1710</v>
+        <v>1690</v>
       </c>
     </row>
     <row r="281">
@@ -5555,11 +5555,11 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>06/06/2026 20:19 BRT</t>
+          <t>04/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C281" t="n">
-        <v>1710</v>
+        <v>1695</v>
       </c>
     </row>
     <row r="282">
@@ -5570,11 +5570,11 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>07/06/2026 08:17 BRT</t>
+          <t>05/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C282" t="n">
-        <v>1709</v>
+        <v>1706</v>
       </c>
     </row>
     <row r="283">
@@ -5585,7 +5585,7 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>07/06/2026 14:23 BRT</t>
+          <t>05/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C283" t="n">
@@ -5600,11 +5600,11 @@
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>07/06/2026 20:19 BRT</t>
+          <t>06/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C284" t="n">
-        <v>1709</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="285">
@@ -5615,7 +5615,7 @@
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>08/06/2026 08:17 BRT</t>
+          <t>06/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C285" t="n">
@@ -5630,101 +5630,101 @@
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>08/06/2026 20:19 BRT</t>
+          <t>06/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C286" t="n">
-        <v>1722</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>07/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C287" t="n">
-        <v>2704</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>07/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C288" t="n">
-        <v>2718</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>07/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C289" t="n">
-        <v>2705</v>
+        <v>1709</v>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>08/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C290" t="n">
-        <v>2705</v>
+        <v>1710</v>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>08/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C291" t="n">
-        <v>2706</v>
+        <v>1722</v>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>MUC</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>09/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C292" t="n">
-        <v>2706</v>
+        <v>1724</v>
       </c>
     </row>
     <row r="293">
@@ -5735,11 +5735,11 @@
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C293" t="n">
-        <v>2706</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="294">
@@ -5750,11 +5750,11 @@
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C294" t="n">
-        <v>2706</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="295">
@@ -5765,11 +5765,11 @@
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C295" t="n">
-        <v>2704</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="296">
@@ -5780,11 +5780,11 @@
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C296" t="n">
-        <v>2887</v>
+        <v>2705</v>
       </c>
     </row>
     <row r="297">
@@ -5795,11 +5795,11 @@
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C297" t="n">
-        <v>2879</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="298">
@@ -5810,11 +5810,11 @@
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C298" t="n">
-        <v>2877</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="299">
@@ -5825,11 +5825,11 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C299" t="n">
-        <v>2843</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="300">
@@ -5840,11 +5840,11 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C300" t="n">
-        <v>2835</v>
+        <v>2706</v>
       </c>
     </row>
     <row r="301">
@@ -5855,11 +5855,11 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C301" t="n">
-        <v>2940</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="302">
@@ -5870,11 +5870,11 @@
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C302" t="n">
-        <v>2983</v>
+        <v>2887</v>
       </c>
     </row>
     <row r="303">
@@ -5885,11 +5885,11 @@
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C303" t="n">
-        <v>2979</v>
+        <v>2879</v>
       </c>
     </row>
     <row r="304">
@@ -5900,11 +5900,11 @@
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C304" t="n">
-        <v>2781</v>
+        <v>2877</v>
       </c>
     </row>
     <row r="305">
@@ -5915,11 +5915,11 @@
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>04/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C305" t="n">
-        <v>2778</v>
+        <v>2843</v>
       </c>
     </row>
     <row r="306">
@@ -5930,11 +5930,11 @@
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C306" t="n">
-        <v>2766</v>
+        <v>2835</v>
       </c>
     </row>
     <row r="307">
@@ -5945,10 +5945,100 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
+          <t>03/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C307" t="n">
+        <v>2940</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>03/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C308" t="n">
+        <v>2983</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>03/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C309" t="n">
+        <v>2979</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>04/06/2026 08:17 BRT</t>
+        </is>
+      </c>
+      <c r="C310" t="n">
+        <v>2781</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>04/06/2026 14:23 BRT</t>
+        </is>
+      </c>
+      <c r="C311" t="n">
+        <v>2778</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>04/06/2026 20:19 BRT</t>
+        </is>
+      </c>
+      <c r="C312" t="n">
+        <v>2766</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
           <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
-      <c r="C307" t="n">
+      <c r="C313" t="n">
         <v>2774</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Monitor run 2026-06-09 17:23 UTC
</commit_message>
<xml_diff>
--- a/docs/flights.xlsx
+++ b/docs/flights.xlsx
@@ -499,7 +499,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>1719</v>
+        <v>1715</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>09/06/2026 08:17 BRT</t>
+          <t>09/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -529,7 +529,7 @@
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
-        <v>1724</v>
+        <v>1719</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -544,7 +544,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>09/06/2026 08:17 BRT</t>
+          <t>09/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -563,7 +563,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1883</v>
+        <v>1878</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -578,7 +578,7 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>09/06/2026 08:17 BRT</t>
+          <t>09/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1951</v>
+        <v>1946</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -612,7 +612,7 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>09/06/2026 08:17 BRT</t>
+          <t>09/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>2342</v>
+        <v>2336</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -642,7 +642,7 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>09/06/2026 08:17 BRT</t>
+          <t>09/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -652,27 +652,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>2774</v>
+        <v>2690</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>11.4</v>
+        <v>7.8</v>
       </c>
       <c r="G7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>09/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -682,31 +682,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ARN</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>Stockholm</t>
-        </is>
-      </c>
+          <t>ZRH</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>2778</v>
+        <v>2774</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>15.4</v>
+        <v>11.4</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -716,31 +712,31 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>AMS</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Amsterdam</t>
+          <t>Stockholm</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>2877</v>
+        <v>2778</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>KLM + Air Baltic</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>11.5</v>
+        <v>15.4</v>
       </c>
       <c r="G9" t="n">
         <v>2</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -750,27 +746,31 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>HEL</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
+          <t>AMS</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Amsterdam</t>
+        </is>
+      </c>
       <c r="D10" t="n">
-        <v>3436</v>
+        <v>2877</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>KLM + Air Baltic</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>7.8</v>
+        <v>11.5</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>09/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -917,7 +917,7 @@
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="n">
-        <v>1719</v>
+        <v>1715</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -932,7 +932,7 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>09/06/2026 08:17 BRT</t>
+          <t>09/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -959,7 +959,7 @@
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
-        <v>1724</v>
+        <v>1719</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -974,7 +974,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>09/06/2026 08:17 BRT</t>
+          <t>09/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1001,7 +1001,7 @@
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
-        <v>1883</v>
+        <v>1878</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -1016,7 +1016,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>09/06/2026 08:17 BRT</t>
+          <t>09/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1043,7 +1043,7 @@
       </c>
       <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
-        <v>1951</v>
+        <v>1946</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -1058,7 +1058,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>09/06/2026 08:17 BRT</t>
+          <t>09/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1085,7 +1085,7 @@
       </c>
       <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
-        <v>2342</v>
+        <v>2336</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1100,7 +1100,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>09/06/2026 08:17 BRT</t>
+          <t>09/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1117,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>ZRH</t>
+          <t>HEL</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1127,22 +1127,22 @@
       </c>
       <c r="E7" t="inlineStr"/>
       <c r="F7" t="n">
-        <v>2774</v>
+        <v>2690</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>SWISS + Lufthansa</t>
+          <t>Finnair</t>
         </is>
       </c>
       <c r="H7" t="n">
-        <v>11.4</v>
+        <v>7.8</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>09/06/2026 14:23 BRT</t>
         </is>
       </c>
     </row>
@@ -1159,7 +1159,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>ARN</t>
+          <t>ZRH</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1169,22 +1169,22 @@
       </c>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="n">
-        <v>2778</v>
+        <v>2774</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Scandinavian Airlines</t>
+          <t>SWISS + Lufthansa</t>
         </is>
       </c>
       <c r="H8" t="n">
-        <v>15.4</v>
+        <v>11.4</v>
       </c>
       <c r="I8" t="n">
         <v>2</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>04/06/2026 20:19 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>AMS</t>
+          <t>ARN</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1211,22 +1211,22 @@
       </c>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
-        <v>2877</v>
+        <v>2778</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>KLM + Air Baltic</t>
+          <t>Scandinavian Airlines</t>
         </is>
       </c>
       <c r="H9" t="n">
-        <v>11.5</v>
+        <v>15.4</v>
       </c>
       <c r="I9" t="n">
         <v>2</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>05/06/2026 08:17 BRT</t>
+          <t>04/06/2026 20:19 BRT</t>
         </is>
       </c>
     </row>
@@ -1243,7 +1243,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>HEL</t>
+          <t>AMS</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1253,22 +1253,22 @@
       </c>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
-        <v>3436</v>
+        <v>2877</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Finnair</t>
+          <t>KLM + Air Baltic</t>
         </is>
       </c>
       <c r="H10" t="n">
-        <v>7.8</v>
+        <v>11.5</v>
       </c>
       <c r="I10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>09/06/2026 08:17 BRT</t>
+          <t>05/06/2026 08:17 BRT</t>
         </is>
       </c>
     </row>
@@ -1337,7 +1337,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C313"/>
+  <dimension ref="A1:C319"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -3060,16 +3060,16 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>DIRECT</t>
+          <t>CPH</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>23/05/2026 09:17 BRT</t>
+          <t>09/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>228</v>
+        <v>1878</v>
       </c>
     </row>
     <row r="116">
@@ -3080,11 +3080,11 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>25/05/2026 15:34 BRT</t>
+          <t>23/05/2026 09:17 BRT</t>
         </is>
       </c>
       <c r="C116" t="n">
-        <v>1329</v>
+        <v>228</v>
       </c>
     </row>
     <row r="117">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>25/05/2026 15:35 BRT</t>
+          <t>25/05/2026 15:34 BRT</t>
         </is>
       </c>
       <c r="C117" t="n">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>25/05/2026 15:57 BRT</t>
+          <t>25/05/2026 15:35 BRT</t>
         </is>
       </c>
       <c r="C119" t="n">
@@ -3140,7 +3140,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>25/05/2026 20:19 BRT</t>
+          <t>25/05/2026 15:57 BRT</t>
         </is>
       </c>
       <c r="C120" t="n">
@@ -3155,11 +3155,11 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>26/05/2026 14:23 BRT</t>
+          <t>25/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C121" t="n">
-        <v>1336</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="122">
@@ -3170,11 +3170,11 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>26/05/2026 20:19 BRT</t>
+          <t>26/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C122" t="n">
-        <v>1337</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="123">
@@ -3185,11 +3185,11 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>27/05/2026 08:17 BRT</t>
+          <t>26/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C123" t="n">
-        <v>1334</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="124">
@@ -3200,11 +3200,11 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>27/05/2026 14:23 BRT</t>
+          <t>27/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C124" t="n">
-        <v>1345</v>
+        <v>1334</v>
       </c>
     </row>
     <row r="125">
@@ -3215,11 +3215,11 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>27/05/2026 20:19 BRT</t>
+          <t>27/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C125" t="n">
-        <v>1344</v>
+        <v>1345</v>
       </c>
     </row>
     <row r="126">
@@ -3230,11 +3230,11 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>28/05/2026 08:17 BRT</t>
+          <t>27/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C126" t="n">
-        <v>1337</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="127">
@@ -3245,11 +3245,11 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>28/05/2026 14:23 BRT</t>
+          <t>28/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C127" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="128">
@@ -3260,11 +3260,11 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>28/05/2026 20:19 BRT</t>
+          <t>28/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C128" t="n">
-        <v>1341</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="129">
@@ -3275,11 +3275,11 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>29/05/2026 08:17 BRT</t>
+          <t>28/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C129" t="n">
-        <v>1337</v>
+        <v>1341</v>
       </c>
     </row>
     <row r="130">
@@ -3290,11 +3290,11 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>29/05/2026 14:23 BRT</t>
+          <t>29/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C130" t="n">
-        <v>1344</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="131">
@@ -3305,11 +3305,11 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>29/05/2026 20:19 BRT</t>
+          <t>29/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C131" t="n">
-        <v>1338</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="132">
@@ -3320,7 +3320,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>30/05/2026 08:17 BRT</t>
+          <t>29/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C132" t="n">
@@ -3335,7 +3335,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>30/05/2026 14:23 BRT</t>
+          <t>30/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C133" t="n">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>30/05/2026 20:19 BRT</t>
+          <t>30/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C134" t="n">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>31/05/2026 08:17 BRT</t>
+          <t>30/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C135" t="n">
@@ -3380,7 +3380,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>31/05/2026 14:23 BRT</t>
+          <t>31/05/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C136" t="n">
@@ -3395,11 +3395,11 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>31/05/2026 20:19 BRT</t>
+          <t>31/05/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C137" t="n">
-        <v>1337</v>
+        <v>1338</v>
       </c>
     </row>
     <row r="138">
@@ -3410,11 +3410,11 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>01/06/2026 08:17 BRT</t>
+          <t>31/05/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C138" t="n">
-        <v>1340</v>
+        <v>1337</v>
       </c>
     </row>
     <row r="139">
@@ -3425,11 +3425,11 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>01/06/2026 14:23 BRT</t>
+          <t>01/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C139" t="n">
-        <v>1336</v>
+        <v>1340</v>
       </c>
     </row>
     <row r="140">
@@ -3440,7 +3440,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>01/06/2026 20:19 BRT</t>
+          <t>01/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C140" t="n">
@@ -3455,11 +3455,11 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>02/06/2026 08:17 BRT</t>
+          <t>01/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C141" t="n">
-        <v>1333</v>
+        <v>1336</v>
       </c>
     </row>
     <row r="142">
@@ -3470,11 +3470,11 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>02/06/2026 14:23 BRT</t>
+          <t>02/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C142" t="n">
-        <v>1332</v>
+        <v>1333</v>
       </c>
     </row>
     <row r="143">
@@ -3485,11 +3485,11 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>02/06/2026 20:19 BRT</t>
+          <t>02/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C143" t="n">
-        <v>1329</v>
+        <v>1332</v>
       </c>
     </row>
     <row r="144">
@@ -3500,11 +3500,11 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>03/06/2026 08:17 BRT</t>
+          <t>02/06/2026 20:19 BRT</t>
         </is>
       </c>
       <c r="C144" t="n">
-        <v>1324</v>
+        <v>1329</v>
       </c>
     </row>
     <row r="145">
@@ -3515,11 +3515,11 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>03/06/2026 14:23 BRT</t>
+          <t>03/06/2026 08:17 BRT</t>
         </is>
       </c>
       <c r="C145" t="n">
-        <v>1344</v>
+        <v>1324</v>
       </c>
     </row>
     <row r="146">
@@ -3530,11 +3530,11 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>03/06/2026 20:19 BRT</t>
+          <t>03/06/2026 14:23 BRT</t>
         </is>
       </c>
       <c r="C146" t="n">
-        <v>1342</v>
+        <v>1344</v>
       </c>
     </row>
     <row r="147">
@@ -3545,11 +3545,11 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>04/06/2026 08:17 BRT</t>
+          <t>03/06/2026 20:19 BRT</t>
         